<commit_message>
ran more tests on different hyperparameters and model sizes
</commit_message>
<xml_diff>
--- a/Code/Boiling-91_Temperature_10Hz.xlsx
+++ b/Code/Boiling-91_Temperature_10Hz.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ytrivedi/Desktop/School Stuff/Oklahoma State/Spring 2026/Deep Learning/Final-Project-Yash-Trivedi/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA6B7FD-E891-7440-A220-CB9929F8C7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71204AE-2791-0E40-B6AA-8C1540C32522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17320" xr2:uid="{130CFDE4-EB42-3F45-93C7-0A9FCD22FCB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Boiling-91_Temperature_10Hz" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'Boiling-91_Temperature_10Hz'!$J$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Boiling-91_Temperature_10Hz'!$J$2:$J$1200</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Boiling-91_Temperature_10Hz'!$J$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Boiling-91_Temperature_10Hz'!$J$2:$J$1200</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -11928,6 +11934,3848 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Boiling-91_Temperature_10Hz'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CHF Proximity</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Boiling-91_Temperature_10Hz'!$J$2:$J$1200</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1199"/>
+                <c:pt idx="0">
+                  <c:v>-4.5489186832778569E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-4.5489186832778569E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-4.5489186832778569E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-4.5201939308199171E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.4916594085106322E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.4916594085106322E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-4.49171303247572E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-4.5078002219736367E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-4.5078002219736367E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-4.5078002219736367E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4.5239585378793558E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-4.5397979396551373E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-4.5397979396551373E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-4.5397185695887438E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-4.5159075496383004E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-4.5159075496383004E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-4.5159075496383004E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.5201366270276745E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-4.5242822357843437E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-4.5242822357843437E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-4.5243980192216385E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-4.5417076430937238E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-4.5417076430937238E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-4.5417076430937238E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-4.5503403120469209E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-4.5587472903085048E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.5587472903085048E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-4.5586908409129996E-2</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-4.5502516562779961E-2</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-4.5502516562779961E-2</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-4.5502516562779961E-2</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>-4.5500322751301905E-2</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>-4.549820063300878E-2</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>-4.549820063300878E-2</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>-4.5494572322946306E-2</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>-4.5132950753342935E-2</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>-4.5132950753342935E-2</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>-4.5132950753342935E-2</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>-4.5088453267427775E-2</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>-4.5045409947717809E-2</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>-4.5045409947717809E-2</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>-4.5046461616960715E-2</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>-4.5150927428378271E-2</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>-4.5150927428378271E-2</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>-4.5150927428378271E-2</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>-4.5313685678928663E-2</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>-4.5469045827179519E-2</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>-4.5469045827179519E-2</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>-4.546968492440108E-2</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>-4.5517297667394825E-2</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>-4.5517297667394825E-2</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>-4.5517297667394825E-2</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>-4.5432124301877604E-2</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>-4.5350822452974324E-2</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>-4.5350822452974324E-2</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>-4.5352586232230006E-2</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>-4.5483546841956705E-2</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>-4.5483546841956705E-2</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>-4.5483546841956705E-2</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>-4.5459466602463319E-2</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>-4.5436784570423543E-2</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>-4.5436784570423543E-2</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>-4.544290763373679E-2</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>-4.5897545084731727E-2</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>-4.5897545084731727E-2</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>-4.5897545084731727E-2</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>-4.5720906399004162E-2</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>-4.5554524153091101E-2</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>-4.5554524153091101E-2</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>-4.5556919424535984E-2</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>-4.5698719494061305E-2</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>-4.5698719494061305E-2</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>-4.5698719494061305E-2</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>-4.5632836496016405E-2</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>-4.5571176767075769E-2</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>-4.5571176767075769E-2</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>-4.5572604709226874E-2</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>-4.5657138884524995E-2</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>-4.5657138884524995E-2</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>-4.5657138884524995E-2</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>-4.5611247632325679E-2</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>-4.5568592301755369E-2</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>-4.5568592301755369E-2</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>-4.5572927960913508E-2</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>-4.5786820479361966E-2</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>-4.5786820479361966E-2</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>-4.5786820479361966E-2</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>-4.5755752681863646E-2</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>-4.5727059493090166E-2</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>-4.5727059493090166E-2</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>-4.5729475743780848E-2</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>-4.5848274736015875E-2</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>-4.5848274736015875E-2</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>-4.5848274736015875E-2</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>-4.5800017439505611E-2</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>-4.5755755970094049E-2</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>-4.5755755970094049E-2</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>-4.5753564869956943E-2</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>-4.5661225649883584E-2</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>-4.5661225649883584E-2</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>-4.5661225649883584E-2</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>-4.5615451940671861E-2</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>-4.5573468411202085E-2</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>-4.5573468411202085E-2</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>-4.5570879504711143E-2</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>-4.5462145432088118E-2</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>-4.5462145432088118E-2</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>-4.5462145432088118E-2</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>-4.5471274279790724E-2</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>-4.5479536464735654E-2</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>-4.5479536464735654E-2</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>-4.5485280971111083E-2</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>-4.572655023883989E-2</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>-4.572655023883989E-2</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>-4.572655023883989E-2</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>-4.5800463163865421E-2</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>-4.5867359039045701E-2</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>-4.5867359039045701E-2</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>-4.5866228528447434E-2</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>-4.5824823577789962E-2</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>-4.5824823577789962E-2</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>-4.5824823577789962E-2</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>-4.5905975982766772E-2</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>-4.5978962107997172E-2</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>-4.5978962107997172E-2</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>-4.597857737571652E-2</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>-4.5964486555932611E-2</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>-4.5964486555932611E-2</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>-4.5964486555932611E-2</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>-4.5982489920290581E-2</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>-4.5998568396633494E-2</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>-4.5998568396633494E-2</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>-4.5994433539740184E-2</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>-4.5860280404966598E-2</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>-4.5860280404966598E-2</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>-4.5860280404966598E-2</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>-4.5594294549258507E-2</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>-4.5358232102316001E-2</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>-4.5358232102316001E-2</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>-4.5340747466707881E-2</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>-4.4773468178061743E-2</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>-4.4773468178061743E-2</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>-4.4773468178061743E-2</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>-4.4592532342370123E-2</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>-4.4433082637166416E-2</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>-4.4433082637166416E-2</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>-4.4405542437114726E-2</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>-4.3601368595589045E-2</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>-4.3601368595589045E-2</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>-4.3601368595589045E-2</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>-4.3042576257428342E-2</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>-4.2550140509423254E-2</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>-4.2550140509423254E-2</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>-4.2492934422963841E-2</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>-4.0828237306979064E-2</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>-4.0828237306979064E-2</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>-4.0828237306979064E-2</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>-3.9814932970323798E-2</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>-3.8933798764535628E-2</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>-3.8933798764535628E-2</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>-3.8860354911739878E-2</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>-3.6723138795373381E-2</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>-3.6723138795373381E-2</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>-3.6723138795373381E-2</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>-3.5159500859032057E-2</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>-3.3799815696995764E-2</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>-3.3799815696995764E-2</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>-3.3693662113788429E-2</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>-3.08950676473977E-2</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>-3.08950676473977E-2</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>-3.08950676473977E-2</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>-2.9117100500730339E-2</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>-2.7591560788464493E-2</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>-2.7591560788464493E-2</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>-2.7445426474625594E-2</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>-2.3592794564319855E-2</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>-2.3592794564319855E-2</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>-2.3592794564319855E-2</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>-2.1553248802801545E-2</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>-1.9803268180264056E-2</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>-1.9803268180264056E-2</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>-1.963609692863948E-2</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>-1.5610055952001493E-2</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>-1.5610055952001493E-2</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>-1.5610055952001493E-2</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>-1.3086173254244505E-2</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>-1.0933905186830607E-2</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>-1.0933905186830607E-2</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>-1.075784956338109E-2</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>-6.5178432986403127E-3</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>-6.5178432986403127E-3</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>-6.5178432986403127E-3</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>-3.783459702464219E-3</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>-1.4684600934301421E-3</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>-1.4684600934301421E-3</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>-1.2418604167333395E-3</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>3.7956247037030299E-3</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>3.7956247037030299E-3</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>3.7956247037030299E-3</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>6.8019229995423787E-3</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>9.3471325997011474E-3</c:v>
+                </c:pt>
+                <c:pt idx="201">
+                  <c:v>9.3471325997011474E-3</c:v>
+                </c:pt>
+                <c:pt idx="202">
+                  <c:v>9.5815243972398774E-3</c:v>
+                </c:pt>
+                <c:pt idx="203">
+                  <c:v>1.4774204219640447E-2</c:v>
+                </c:pt>
+                <c:pt idx="204">
+                  <c:v>1.4774204219640447E-2</c:v>
+                </c:pt>
+                <c:pt idx="205">
+                  <c:v>1.4774204219640447E-2</c:v>
+                </c:pt>
+                <c:pt idx="206">
+                  <c:v>1.7990891096113095E-2</c:v>
+                </c:pt>
+                <c:pt idx="207">
+                  <c:v>2.0678001474634628E-2</c:v>
+                </c:pt>
+                <c:pt idx="208">
+                  <c:v>2.0678001474634628E-2</c:v>
+                </c:pt>
+                <c:pt idx="209">
+                  <c:v>2.0929427043089081E-2</c:v>
+                </c:pt>
+                <c:pt idx="210">
+                  <c:v>2.6101610165671817E-2</c:v>
+                </c:pt>
+                <c:pt idx="211">
+                  <c:v>2.6101610165671817E-2</c:v>
+                </c:pt>
+                <c:pt idx="212">
+                  <c:v>2.6101610165671817E-2</c:v>
+                </c:pt>
+                <c:pt idx="213">
+                  <c:v>2.9549385792921424E-2</c:v>
+                </c:pt>
+                <c:pt idx="214">
+                  <c:v>3.2429539823021943E-2</c:v>
+                </c:pt>
+                <c:pt idx="215">
+                  <c:v>3.2429539823021943E-2</c:v>
+                </c:pt>
+                <c:pt idx="216">
+                  <c:v>3.270469818463026E-2</c:v>
+                </c:pt>
+                <c:pt idx="217">
+                  <c:v>3.8345444597816643E-2</c:v>
+                </c:pt>
+                <c:pt idx="218">
+                  <c:v>3.8345444597816643E-2</c:v>
+                </c:pt>
+                <c:pt idx="219">
+                  <c:v>3.8345444597816643E-2</c:v>
+                </c:pt>
+                <c:pt idx="220">
+                  <c:v>4.1761705465680657E-2</c:v>
+                </c:pt>
+                <c:pt idx="221">
+                  <c:v>4.457753260526167E-2</c:v>
+                </c:pt>
+                <c:pt idx="222">
+                  <c:v>4.457753260526167E-2</c:v>
+                </c:pt>
+                <c:pt idx="223">
+                  <c:v>4.486528968016805E-2</c:v>
+                </c:pt>
+                <c:pt idx="224">
+                  <c:v>5.0764309715786819E-2</c:v>
+                </c:pt>
+                <c:pt idx="225">
+                  <c:v>5.0764309715786819E-2</c:v>
+                </c:pt>
+                <c:pt idx="226">
+                  <c:v>5.0764309715786819E-2</c:v>
+                </c:pt>
+                <c:pt idx="227">
+                  <c:v>5.4181184734129924E-2</c:v>
+                </c:pt>
+                <c:pt idx="228">
+                  <c:v>5.6997518082582549E-2</c:v>
+                </c:pt>
+                <c:pt idx="229">
+                  <c:v>5.6997518082582549E-2</c:v>
+                </c:pt>
+                <c:pt idx="230">
+                  <c:v>5.7324664239572817E-2</c:v>
+                </c:pt>
+                <c:pt idx="231">
+                  <c:v>6.3562250966318457E-2</c:v>
+                </c:pt>
+                <c:pt idx="232">
+                  <c:v>6.3562250966318457E-2</c:v>
+                </c:pt>
+                <c:pt idx="233">
+                  <c:v>6.3562250966318457E-2</c:v>
+                </c:pt>
+                <c:pt idx="234">
+                  <c:v>6.7179602788340592E-2</c:v>
+                </c:pt>
+                <c:pt idx="235">
+                  <c:v>7.0143216329282346E-2</c:v>
+                </c:pt>
+                <c:pt idx="236">
+                  <c:v>7.0143216329282346E-2</c:v>
+                </c:pt>
+                <c:pt idx="237">
+                  <c:v>7.0484145977037616E-2</c:v>
+                </c:pt>
+                <c:pt idx="238">
+                  <c:v>7.6984537927708083E-2</c:v>
+                </c:pt>
+                <c:pt idx="239">
+                  <c:v>7.6984537927708083E-2</c:v>
+                </c:pt>
+                <c:pt idx="240">
+                  <c:v>7.6984537927708083E-2</c:v>
+                </c:pt>
+                <c:pt idx="241">
+                  <c:v>8.0317841235906032E-2</c:v>
+                </c:pt>
+                <c:pt idx="242">
+                  <c:v>8.3028660191370243E-2</c:v>
+                </c:pt>
+                <c:pt idx="243">
+                  <c:v>8.3028660191370243E-2</c:v>
+                </c:pt>
+                <c:pt idx="244">
+                  <c:v>8.3359562811055929E-2</c:v>
+                </c:pt>
+                <c:pt idx="245">
+                  <c:v>8.9274447138148097E-2</c:v>
+                </c:pt>
+                <c:pt idx="246">
+                  <c:v>8.9274447138148097E-2</c:v>
+                </c:pt>
+                <c:pt idx="247">
+                  <c:v>8.9274447138148097E-2</c:v>
+                </c:pt>
+                <c:pt idx="248">
+                  <c:v>9.2626413965460036E-2</c:v>
+                </c:pt>
+                <c:pt idx="249">
+                  <c:v>9.5336087748020243E-2</c:v>
+                </c:pt>
+                <c:pt idx="250">
+                  <c:v>9.5336087748020243E-2</c:v>
+                </c:pt>
+                <c:pt idx="251">
+                  <c:v>9.566148395683273E-2</c:v>
+                </c:pt>
+                <c:pt idx="252">
+                  <c:v>0.10145760392637057</c:v>
+                </c:pt>
+                <c:pt idx="253">
+                  <c:v>0.10145760392637057</c:v>
+                </c:pt>
+                <c:pt idx="254">
+                  <c:v>0.10145760392637057</c:v>
+                </c:pt>
+                <c:pt idx="255">
+                  <c:v>0.10453028084902063</c:v>
+                </c:pt>
+                <c:pt idx="256">
+                  <c:v>0.10699578209236729</c:v>
+                </c:pt>
+                <c:pt idx="257">
+                  <c:v>0.10699578209236729</c:v>
+                </c:pt>
+                <c:pt idx="258">
+                  <c:v>0.10732919148237471</c:v>
+                </c:pt>
+                <c:pt idx="259">
+                  <c:v>0.11291870184445997</c:v>
+                </c:pt>
+                <c:pt idx="260">
+                  <c:v>0.11291870184445997</c:v>
+                </c:pt>
+                <c:pt idx="261">
+                  <c:v>0.11291870184445997</c:v>
+                </c:pt>
+                <c:pt idx="262">
+                  <c:v>0.11586371875092601</c:v>
+                </c:pt>
+                <c:pt idx="263">
+                  <c:v>0.11822678620881839</c:v>
+                </c:pt>
+                <c:pt idx="264">
+                  <c:v>0.11822678620881839</c:v>
+                </c:pt>
+                <c:pt idx="265">
+                  <c:v>0.11854174376291546</c:v>
+                </c:pt>
+                <c:pt idx="266">
+                  <c:v>0.1238033876079998</c:v>
+                </c:pt>
+                <c:pt idx="267">
+                  <c:v>0.1238033876079998</c:v>
+                </c:pt>
+                <c:pt idx="268">
+                  <c:v>0.1238033876079998</c:v>
+                </c:pt>
+                <c:pt idx="269">
+                  <c:v>0.12652271292820738</c:v>
+                </c:pt>
+                <c:pt idx="270">
+                  <c:v>0.12867551214002659</c:v>
+                </c:pt>
+                <c:pt idx="271">
+                  <c:v>0.12867551214002659</c:v>
+                </c:pt>
+                <c:pt idx="272">
+                  <c:v>0.128956607627951</c:v>
+                </c:pt>
+                <c:pt idx="273">
+                  <c:v>0.13365255577898266</c:v>
+                </c:pt>
+                <c:pt idx="274">
+                  <c:v>0.13365255577898266</c:v>
+                </c:pt>
+                <c:pt idx="275">
+                  <c:v>0.13365255577898266</c:v>
+                </c:pt>
+                <c:pt idx="276">
+                  <c:v>0.1365976631161577</c:v>
+                </c:pt>
+                <c:pt idx="277">
+                  <c:v>0.13892920642475456</c:v>
+                </c:pt>
+                <c:pt idx="278">
+                  <c:v>0.13892920642475456</c:v>
+                </c:pt>
+                <c:pt idx="279">
+                  <c:v>0.13922065407027989</c:v>
+                </c:pt>
+                <c:pt idx="280">
+                  <c:v>0.14380285871954501</c:v>
+                </c:pt>
+                <c:pt idx="281">
+                  <c:v>0.14380285871954501</c:v>
+                </c:pt>
+                <c:pt idx="282">
+                  <c:v>0.14380285871954501</c:v>
+                </c:pt>
+                <c:pt idx="283">
+                  <c:v>0.14598412434788471</c:v>
+                </c:pt>
+                <c:pt idx="284">
+                  <c:v>0.14770074167670691</c:v>
+                </c:pt>
+                <c:pt idx="285">
+                  <c:v>0.14770074167670691</c:v>
+                </c:pt>
+                <c:pt idx="286">
+                  <c:v>0.1478795645302271</c:v>
+                </c:pt>
+                <c:pt idx="287">
+                  <c:v>0.15069105717171033</c:v>
+                </c:pt>
+                <c:pt idx="288">
+                  <c:v>0.15069105717171033</c:v>
+                </c:pt>
+                <c:pt idx="289">
+                  <c:v>0.15069105717171033</c:v>
+                </c:pt>
+                <c:pt idx="290">
+                  <c:v>0.15222194502642755</c:v>
+                </c:pt>
+                <c:pt idx="291">
+                  <c:v>0.15341766808455615</c:v>
+                </c:pt>
+                <c:pt idx="292">
+                  <c:v>0.15341766808455615</c:v>
+                </c:pt>
+                <c:pt idx="293">
+                  <c:v>0.15359871380749268</c:v>
+                </c:pt>
+                <c:pt idx="294">
+                  <c:v>0.15628581348491458</c:v>
+                </c:pt>
+                <c:pt idx="295">
+                  <c:v>0.15628581348491458</c:v>
+                </c:pt>
+                <c:pt idx="296">
+                  <c:v>0.15628581348491458</c:v>
+                </c:pt>
+                <c:pt idx="297">
+                  <c:v>0.15777729524299411</c:v>
+                </c:pt>
+                <c:pt idx="298">
+                  <c:v>0.15893538696104745</c:v>
+                </c:pt>
+                <c:pt idx="299">
+                  <c:v>0.15893538696104745</c:v>
+                </c:pt>
+                <c:pt idx="300">
+                  <c:v>0.15911977502452238</c:v>
+                </c:pt>
+                <c:pt idx="301">
+                  <c:v>0.16185648207208006</c:v>
+                </c:pt>
+                <c:pt idx="302">
+                  <c:v>0.16185648207208006</c:v>
+                </c:pt>
+                <c:pt idx="303">
+                  <c:v>0.16185648207208006</c:v>
+                </c:pt>
+                <c:pt idx="304">
+                  <c:v>0.16328166139119291</c:v>
+                </c:pt>
+                <c:pt idx="305">
+                  <c:v>0.16437988780770296</c:v>
+                </c:pt>
+                <c:pt idx="306">
+                  <c:v>0.16437988780770296</c:v>
+                </c:pt>
+                <c:pt idx="307">
+                  <c:v>0.16454421673466704</c:v>
+                </c:pt>
+                <c:pt idx="308">
+                  <c:v>0.16686125460496437</c:v>
+                </c:pt>
+                <c:pt idx="309">
+                  <c:v>0.16686125460496437</c:v>
+                </c:pt>
+                <c:pt idx="310">
+                  <c:v>0.16686125460496437</c:v>
+                </c:pt>
+                <c:pt idx="311">
+                  <c:v>0.16817163092813708</c:v>
+                </c:pt>
+                <c:pt idx="312">
+                  <c:v>0.16918139150658343</c:v>
+                </c:pt>
+                <c:pt idx="313">
+                  <c:v>0.16918139150658343</c:v>
+                </c:pt>
+                <c:pt idx="314">
+                  <c:v>0.16929649227245955</c:v>
+                </c:pt>
+                <c:pt idx="315">
+                  <c:v>0.17091365803302114</c:v>
+                </c:pt>
+                <c:pt idx="316">
+                  <c:v>0.17091365803302114</c:v>
+                </c:pt>
+                <c:pt idx="317">
+                  <c:v>0.17091365803300845</c:v>
+                </c:pt>
+                <c:pt idx="318">
+                  <c:v>0.17201404349296642</c:v>
+                </c:pt>
+                <c:pt idx="319">
+                  <c:v>0.17285059384263859</c:v>
+                </c:pt>
+                <c:pt idx="320">
+                  <c:v>0.17285059384263859</c:v>
+                </c:pt>
+                <c:pt idx="321">
+                  <c:v>0.17296488420058895</c:v>
+                </c:pt>
+                <c:pt idx="322">
+                  <c:v>0.17457066372979468</c:v>
+                </c:pt>
+                <c:pt idx="323">
+                  <c:v>0.17457066372978203</c:v>
+                </c:pt>
+                <c:pt idx="324">
+                  <c:v>0.17457066372978203</c:v>
+                </c:pt>
+                <c:pt idx="325">
+                  <c:v>0.17581886518462908</c:v>
+                </c:pt>
+                <c:pt idx="326">
+                  <c:v>0.17676779026725539</c:v>
+                </c:pt>
+                <c:pt idx="327">
+                  <c:v>0.17676779026725539</c:v>
+                </c:pt>
+                <c:pt idx="328">
+                  <c:v>0.17688328380181234</c:v>
+                </c:pt>
+                <c:pt idx="329">
+                  <c:v>0.17842319759596784</c:v>
+                </c:pt>
+                <c:pt idx="330">
+                  <c:v>0.17842319759596784</c:v>
+                </c:pt>
+                <c:pt idx="331">
+                  <c:v>0.17842319759596784</c:v>
+                </c:pt>
+                <c:pt idx="332">
+                  <c:v>0.17940958345138092</c:v>
+                </c:pt>
+                <c:pt idx="333">
+                  <c:v>0.18015510764443052</c:v>
+                </c:pt>
+                <c:pt idx="334">
+                  <c:v>0.18015510764443052</c:v>
+                </c:pt>
+                <c:pt idx="335">
+                  <c:v>0.18025283916053866</c:v>
+                </c:pt>
+                <c:pt idx="336">
+                  <c:v>0.18155592604206558</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>0.18155592604205292</c:v>
+                </c:pt>
+                <c:pt idx="338">
+                  <c:v>0.18155592604205292</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>0.18245800447090083</c:v>
+                </c:pt>
+                <c:pt idx="340">
+                  <c:v>0.18313456329254654</c:v>
+                </c:pt>
+                <c:pt idx="341">
+                  <c:v>0.18313456329254654</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>0.18326914971638883</c:v>
+                </c:pt>
+                <c:pt idx="343">
+                  <c:v>0.18497595027346567</c:v>
+                </c:pt>
+                <c:pt idx="344">
+                  <c:v>0.18497595027346567</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>0.18497595027346567</c:v>
+                </c:pt>
+                <c:pt idx="346">
+                  <c:v>0.18604132310721358</c:v>
+                </c:pt>
+                <c:pt idx="347">
+                  <c:v>0.18683573406417664</c:v>
+                </c:pt>
+                <c:pt idx="348">
+                  <c:v>0.18683573406417664</c:v>
+                </c:pt>
+                <c:pt idx="349">
+                  <c:v>0.18697660157242185</c:v>
+                </c:pt>
+                <c:pt idx="350">
+                  <c:v>0.18876305769983254</c:v>
+                </c:pt>
+                <c:pt idx="351">
+                  <c:v>0.18876305769983254</c:v>
+                </c:pt>
+                <c:pt idx="352">
+                  <c:v>0.18876305769983254</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>0.18997351694329556</c:v>
+                </c:pt>
+                <c:pt idx="354">
+                  <c:v>0.19086911684597221</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>0.19086911684597221</c:v>
+                </c:pt>
+                <c:pt idx="356">
+                  <c:v>0.19100886139754283</c:v>
+                </c:pt>
+                <c:pt idx="357">
+                  <c:v>0.19270402356655644</c:v>
+                </c:pt>
+                <c:pt idx="358">
+                  <c:v>0.19270402356655644</c:v>
+                </c:pt>
+                <c:pt idx="359">
+                  <c:v>0.19270402356655644</c:v>
+                </c:pt>
+                <c:pt idx="360">
+                  <c:v>0.19375636934737442</c:v>
+                </c:pt>
+                <c:pt idx="361">
+                  <c:v>0.19453498356671359</c:v>
+                </c:pt>
+                <c:pt idx="362">
+                  <c:v>0.19453498356671359</c:v>
+                </c:pt>
+                <c:pt idx="363">
+                  <c:v>0.19468994240230483</c:v>
+                </c:pt>
+                <c:pt idx="364">
+                  <c:v>0.19656292311085827</c:v>
+                </c:pt>
+                <c:pt idx="365">
+                  <c:v>0.19656292311085827</c:v>
+                </c:pt>
+                <c:pt idx="366">
+                  <c:v>0.19656292311087095</c:v>
+                </c:pt>
+                <c:pt idx="367">
+                  <c:v>0.19755468806527501</c:v>
+                </c:pt>
+                <c:pt idx="368">
+                  <c:v>0.19827856248603679</c:v>
+                </c:pt>
+                <c:pt idx="369">
+                  <c:v>0.19827856248603679</c:v>
+                </c:pt>
+                <c:pt idx="370">
+                  <c:v>0.19841119881294086</c:v>
+                </c:pt>
+                <c:pt idx="371">
+                  <c:v>0.20001436832951414</c:v>
+                </c:pt>
+                <c:pt idx="372">
+                  <c:v>0.20001436832951414</c:v>
+                </c:pt>
+                <c:pt idx="373">
+                  <c:v>0.20001436832951414</c:v>
+                </c:pt>
+                <c:pt idx="374">
+                  <c:v>0.20111403317777524</c:v>
+                </c:pt>
+                <c:pt idx="375">
+                  <c:v>0.20191666211875556</c:v>
+                </c:pt>
+                <c:pt idx="376">
+                  <c:v>0.20191666211875556</c:v>
+                </c:pt>
+                <c:pt idx="377">
+                  <c:v>0.20208613415063828</c:v>
+                </c:pt>
+                <c:pt idx="378">
+                  <c:v>0.20404212385184389</c:v>
+                </c:pt>
+                <c:pt idx="379">
+                  <c:v>0.20404212385184389</c:v>
+                </c:pt>
+                <c:pt idx="380">
+                  <c:v>0.20404212385185658</c:v>
+                </c:pt>
+                <c:pt idx="381">
+                  <c:v>0.20492750085612618</c:v>
+                </c:pt>
+                <c:pt idx="382">
+                  <c:v>0.20556497229921791</c:v>
+                </c:pt>
+                <c:pt idx="383">
+                  <c:v>0.20556497229921791</c:v>
+                </c:pt>
+                <c:pt idx="384">
+                  <c:v>0.2056916669740636</c:v>
+                </c:pt>
+                <c:pt idx="385">
+                  <c:v>0.20715393467962354</c:v>
+                </c:pt>
+                <c:pt idx="386">
+                  <c:v>0.20715393467962354</c:v>
+                </c:pt>
+                <c:pt idx="387">
+                  <c:v>0.20715393467962354</c:v>
+                </c:pt>
+                <c:pt idx="388">
+                  <c:v>0.20813379019045003</c:v>
+                </c:pt>
+                <c:pt idx="389">
+                  <c:v>0.2088392861582532</c:v>
+                </c:pt>
+                <c:pt idx="390">
+                  <c:v>0.20883928615824054</c:v>
+                </c:pt>
+                <c:pt idx="391">
+                  <c:v>0.20897871565769577</c:v>
+                </c:pt>
+                <c:pt idx="392">
+                  <c:v>0.21051801733162895</c:v>
+                </c:pt>
+                <c:pt idx="393">
+                  <c:v>0.21051801733162895</c:v>
+                </c:pt>
+                <c:pt idx="394">
+                  <c:v>0.21051801733162895</c:v>
+                </c:pt>
+                <c:pt idx="395">
+                  <c:v>0.21146908370674242</c:v>
+                </c:pt>
+                <c:pt idx="396">
+                  <c:v>0.2121499607707466</c:v>
+                </c:pt>
+                <c:pt idx="397">
+                  <c:v>0.2121499607707466</c:v>
+                </c:pt>
+                <c:pt idx="398">
+                  <c:v>0.21231512579750059</c:v>
+                </c:pt>
+                <c:pt idx="399">
+                  <c:v>0.21413854769271265</c:v>
+                </c:pt>
+                <c:pt idx="400">
+                  <c:v>0.21413854769272533</c:v>
+                </c:pt>
+                <c:pt idx="401">
+                  <c:v>0.21413854769271265</c:v>
+                </c:pt>
+                <c:pt idx="402">
+                  <c:v>0.21513583873249303</c:v>
+                </c:pt>
+                <c:pt idx="403">
+                  <c:v>0.21584414202780419</c:v>
+                </c:pt>
+                <c:pt idx="404">
+                  <c:v>0.21584414202780419</c:v>
+                </c:pt>
+                <c:pt idx="405">
+                  <c:v>0.21599814304249473</c:v>
+                </c:pt>
+                <c:pt idx="406">
+                  <c:v>0.21763292304466814</c:v>
+                </c:pt>
+                <c:pt idx="407">
+                  <c:v>0.21763292304466814</c:v>
+                </c:pt>
+                <c:pt idx="408">
+                  <c:v>0.21763292304466814</c:v>
+                </c:pt>
+                <c:pt idx="409">
+                  <c:v>0.218437236838949</c:v>
+                </c:pt>
+                <c:pt idx="410">
+                  <c:v>0.21900848243147597</c:v>
+                </c:pt>
+                <c:pt idx="411">
+                  <c:v>0.21900848243148863</c:v>
+                </c:pt>
+                <c:pt idx="412">
+                  <c:v>0.2191631413400196</c:v>
+                </c:pt>
+                <c:pt idx="413">
+                  <c:v>0.22079895671872218</c:v>
+                </c:pt>
+                <c:pt idx="414">
+                  <c:v>0.22079895671872218</c:v>
+                </c:pt>
+                <c:pt idx="415">
+                  <c:v>0.22079895671873487</c:v>
+                </c:pt>
+                <c:pt idx="416">
+                  <c:v>0.22160436672085634</c:v>
+                </c:pt>
+                <c:pt idx="417">
+                  <c:v>0.22216860875625202</c:v>
+                </c:pt>
+                <c:pt idx="418">
+                  <c:v>0.22216860875625202</c:v>
+                </c:pt>
+                <c:pt idx="419">
+                  <c:v>0.2223228542382801</c:v>
+                </c:pt>
+                <c:pt idx="420">
+                  <c:v>0.22389387303673569</c:v>
+                </c:pt>
+                <c:pt idx="421">
+                  <c:v>0.22389387303673569</c:v>
+                </c:pt>
+                <c:pt idx="422">
+                  <c:v>0.22389387303673569</c:v>
+                </c:pt>
+                <c:pt idx="423">
+                  <c:v>0.22493216699547888</c:v>
+                </c:pt>
+                <c:pt idx="424">
+                  <c:v>0.2256595593733616</c:v>
+                </c:pt>
+                <c:pt idx="425">
+                  <c:v>0.2256595593733616</c:v>
+                </c:pt>
+                <c:pt idx="426">
+                  <c:v>0.2258053067977798</c:v>
+                </c:pt>
+                <c:pt idx="427">
+                  <c:v>0.22728437325298773</c:v>
+                </c:pt>
+                <c:pt idx="428">
+                  <c:v>0.22728437325298773</c:v>
+                </c:pt>
+                <c:pt idx="429">
+                  <c:v>0.22728437325298773</c:v>
+                </c:pt>
+                <c:pt idx="430">
+                  <c:v>0.22807625684468691</c:v>
+                </c:pt>
+                <c:pt idx="431">
+                  <c:v>0.22862345730413119</c:v>
+                </c:pt>
+                <c:pt idx="432">
+                  <c:v>0.22862345730413119</c:v>
+                </c:pt>
+                <c:pt idx="433">
+                  <c:v>0.22879033315444669</c:v>
+                </c:pt>
+                <c:pt idx="434">
+                  <c:v>0.23048381400587376</c:v>
+                </c:pt>
+                <c:pt idx="435">
+                  <c:v>0.23048381400587376</c:v>
+                </c:pt>
+                <c:pt idx="436">
+                  <c:v>0.23048381400587376</c:v>
+                </c:pt>
+                <c:pt idx="437">
+                  <c:v>0.23144145258097687</c:v>
+                </c:pt>
+                <c:pt idx="438">
+                  <c:v>0.23210319159637799</c:v>
+                </c:pt>
+                <c:pt idx="439">
+                  <c:v>0.23210319159637799</c:v>
+                </c:pt>
+                <c:pt idx="440">
+                  <c:v>0.23225328421999364</c:v>
+                </c:pt>
+                <c:pt idx="441">
+                  <c:v>0.23371668730027872</c:v>
+                </c:pt>
+                <c:pt idx="442">
+                  <c:v>0.23371668730027872</c:v>
+                </c:pt>
+                <c:pt idx="443">
+                  <c:v>0.23371668730027872</c:v>
+                </c:pt>
+                <c:pt idx="444">
+                  <c:v>0.23441074452193111</c:v>
+                </c:pt>
+                <c:pt idx="445">
+                  <c:v>0.23488766652341336</c:v>
+                </c:pt>
+                <c:pt idx="446">
+                  <c:v>0.23488766652341336</c:v>
+                </c:pt>
+                <c:pt idx="447">
+                  <c:v>0.23503674774439501</c:v>
+                </c:pt>
+                <c:pt idx="448">
+                  <c:v>0.23649028964908295</c:v>
+                </c:pt>
+                <c:pt idx="449">
+                  <c:v>0.23649028964908295</c:v>
+                </c:pt>
+                <c:pt idx="450">
+                  <c:v>0.23649028964908295</c:v>
+                </c:pt>
+                <c:pt idx="451">
+                  <c:v>0.23755095319291838</c:v>
+                </c:pt>
+                <c:pt idx="452">
+                  <c:v>0.23827386354123778</c:v>
+                </c:pt>
+                <c:pt idx="453">
+                  <c:v>0.23827386354123778</c:v>
+                </c:pt>
+                <c:pt idx="454">
+                  <c:v>0.23844208851616308</c:v>
+                </c:pt>
+                <c:pt idx="455">
+                  <c:v>0.24002572362494276</c:v>
+                </c:pt>
+                <c:pt idx="456">
+                  <c:v>0.24002572362494276</c:v>
+                </c:pt>
+                <c:pt idx="457">
+                  <c:v>0.24002572362494276</c:v>
+                </c:pt>
+                <c:pt idx="458">
+                  <c:v>0.2408195279032688</c:v>
+                </c:pt>
+                <c:pt idx="459">
+                  <c:v>0.24135755080303228</c:v>
+                </c:pt>
+                <c:pt idx="460">
+                  <c:v>0.24135755080303228</c:v>
+                </c:pt>
+                <c:pt idx="461">
+                  <c:v>0.24148441039334842</c:v>
+                </c:pt>
+                <c:pt idx="462">
+                  <c:v>0.24267426586121885</c:v>
+                </c:pt>
+                <c:pt idx="463">
+                  <c:v>0.2426742658612317</c:v>
+                </c:pt>
+                <c:pt idx="464">
+                  <c:v>0.24267426586121885</c:v>
+                </c:pt>
+                <c:pt idx="465">
+                  <c:v>0.24348917755791516</c:v>
+                </c:pt>
+                <c:pt idx="466">
+                  <c:v>0.24403697930958859</c:v>
+                </c:pt>
+                <c:pt idx="467">
+                  <c:v>0.24403697930958859</c:v>
+                </c:pt>
+                <c:pt idx="468">
+                  <c:v>0.24419072181872459</c:v>
+                </c:pt>
+                <c:pt idx="469">
+                  <c:v>0.24558465390165179</c:v>
+                </c:pt>
+                <c:pt idx="470">
+                  <c:v>0.24558465390165179</c:v>
+                </c:pt>
+                <c:pt idx="471">
+                  <c:v>0.24558465390165179</c:v>
+                </c:pt>
+                <c:pt idx="472">
+                  <c:v>0.24637921488487874</c:v>
+                </c:pt>
+                <c:pt idx="473">
+                  <c:v>0.2469133364347329</c:v>
+                </c:pt>
+                <c:pt idx="474">
+                  <c:v>0.2469133364347329</c:v>
+                </c:pt>
+                <c:pt idx="475">
+                  <c:v>0.24703612592465385</c:v>
+                </c:pt>
+                <c:pt idx="476">
+                  <c:v>0.24814532431703984</c:v>
+                </c:pt>
+                <c:pt idx="477">
+                  <c:v>0.24814532431703984</c:v>
+                </c:pt>
+                <c:pt idx="478">
+                  <c:v>0.24814532431703984</c:v>
+                </c:pt>
+                <c:pt idx="479">
+                  <c:v>0.24909511745821608</c:v>
+                </c:pt>
+                <c:pt idx="480">
+                  <c:v>0.24972481456839005</c:v>
+                </c:pt>
+                <c:pt idx="481">
+                  <c:v>0.24972481456839005</c:v>
+                </c:pt>
+                <c:pt idx="482">
+                  <c:v>0.2498770528273494</c:v>
+                </c:pt>
+                <c:pt idx="483">
+                  <c:v>0.2512522717667165</c:v>
+                </c:pt>
+                <c:pt idx="484">
+                  <c:v>0.2512522717667165</c:v>
+                </c:pt>
+                <c:pt idx="485">
+                  <c:v>0.2512522717667165</c:v>
+                </c:pt>
+                <c:pt idx="486">
+                  <c:v>0.25194707542550748</c:v>
+                </c:pt>
+                <c:pt idx="487">
+                  <c:v>0.25240771873520451</c:v>
+                </c:pt>
+                <c:pt idx="488">
+                  <c:v>0.25240771873520451</c:v>
+                </c:pt>
+                <c:pt idx="489">
+                  <c:v>0.25258512316335807</c:v>
+                </c:pt>
+                <c:pt idx="490">
+                  <c:v>0.25413025850546178</c:v>
+                </c:pt>
+                <c:pt idx="491">
+                  <c:v>0.25413025850546178</c:v>
+                </c:pt>
+                <c:pt idx="492">
+                  <c:v>0.25413025850546178</c:v>
+                </c:pt>
+                <c:pt idx="493">
+                  <c:v>0.25489630016440756</c:v>
+                </c:pt>
+                <c:pt idx="494">
+                  <c:v>0.25540138257689099</c:v>
+                </c:pt>
+                <c:pt idx="495">
+                  <c:v>0.25540138257689099</c:v>
+                </c:pt>
+                <c:pt idx="496">
+                  <c:v>0.25554983958076116</c:v>
+                </c:pt>
+                <c:pt idx="497">
+                  <c:v>0.25684285219506842</c:v>
+                </c:pt>
+                <c:pt idx="498">
+                  <c:v>0.25684285219506842</c:v>
+                </c:pt>
+                <c:pt idx="499">
+                  <c:v>0.25684285219506842</c:v>
+                </c:pt>
+                <c:pt idx="500">
+                  <c:v>0.25777211980984654</c:v>
+                </c:pt>
+                <c:pt idx="501">
+                  <c:v>0.25837971786566916</c:v>
+                </c:pt>
+                <c:pt idx="502">
+                  <c:v>0.25837971786566916</c:v>
+                </c:pt>
+                <c:pt idx="503">
+                  <c:v>0.258503069057961</c:v>
+                </c:pt>
+                <c:pt idx="504">
+                  <c:v>0.25953999001817862</c:v>
+                </c:pt>
+                <c:pt idx="505">
+                  <c:v>0.25953999001817862</c:v>
+                </c:pt>
+                <c:pt idx="506">
+                  <c:v>0.25953999001817862</c:v>
+                </c:pt>
+                <c:pt idx="507">
+                  <c:v>0.26028715061206803</c:v>
+                </c:pt>
+                <c:pt idx="508">
+                  <c:v>0.26077300914034252</c:v>
+                </c:pt>
+                <c:pt idx="509">
+                  <c:v>0.26077300914034252</c:v>
+                </c:pt>
+                <c:pt idx="510">
+                  <c:v>0.26093114798111272</c:v>
+                </c:pt>
+                <c:pt idx="511">
+                  <c:v>0.26226050261137723</c:v>
+                </c:pt>
+                <c:pt idx="512">
+                  <c:v>0.26226050261137723</c:v>
+                </c:pt>
+                <c:pt idx="513">
+                  <c:v>0.26226050261137723</c:v>
+                </c:pt>
+                <c:pt idx="514">
+                  <c:v>0.26288439612644843</c:v>
+                </c:pt>
+                <c:pt idx="515">
+                  <c:v>0.26328668811978495</c:v>
+                </c:pt>
+                <c:pt idx="516">
+                  <c:v>0.26328668811978495</c:v>
+                </c:pt>
+                <c:pt idx="517">
+                  <c:v>0.26343921233930312</c:v>
+                </c:pt>
+                <c:pt idx="518">
+                  <c:v>0.26468251582576713</c:v>
+                </c:pt>
+                <c:pt idx="519">
+                  <c:v>0.26468251582576713</c:v>
+                </c:pt>
+                <c:pt idx="520">
+                  <c:v>0.26468251582576713</c:v>
+                </c:pt>
+                <c:pt idx="521">
+                  <c:v>0.26558568031119778</c:v>
+                </c:pt>
+                <c:pt idx="522">
+                  <c:v>0.26616804866793825</c:v>
+                </c:pt>
+                <c:pt idx="523">
+                  <c:v>0.26616804866793825</c:v>
+                </c:pt>
+                <c:pt idx="524">
+                  <c:v>0.26631119178980101</c:v>
+                </c:pt>
+                <c:pt idx="525">
+                  <c:v>0.26747368744619371</c:v>
+                </c:pt>
+                <c:pt idx="526">
+                  <c:v>0.26747368744619371</c:v>
+                </c:pt>
+                <c:pt idx="527">
+                  <c:v>0.26747368744619371</c:v>
+                </c:pt>
+                <c:pt idx="528">
+                  <c:v>0.26816393607103645</c:v>
+                </c:pt>
+                <c:pt idx="529">
+                  <c:v>0.26860284416401059</c:v>
+                </c:pt>
+                <c:pt idx="530">
+                  <c:v>0.26860284416401059</c:v>
+                </c:pt>
+                <c:pt idx="531">
+                  <c:v>0.26871143155110538</c:v>
+                </c:pt>
+                <c:pt idx="532">
+                  <c:v>0.26959329275540383</c:v>
+                </c:pt>
+                <c:pt idx="533">
+                  <c:v>0.26959329275540383</c:v>
+                </c:pt>
+                <c:pt idx="534">
+                  <c:v>0.26959329275540383</c:v>
+                </c:pt>
+                <c:pt idx="535">
+                  <c:v>0.27027040431245897</c:v>
+                </c:pt>
+                <c:pt idx="536">
+                  <c:v>0.27070095894385837</c:v>
+                </c:pt>
+                <c:pt idx="537">
+                  <c:v>0.27070095894385837</c:v>
+                </c:pt>
+                <c:pt idx="538">
+                  <c:v>0.27083545662888719</c:v>
+                </c:pt>
+                <c:pt idx="539">
+                  <c:v>0.27189165903782286</c:v>
+                </c:pt>
+                <c:pt idx="540">
+                  <c:v>0.27189165903782286</c:v>
+                </c:pt>
+                <c:pt idx="541">
+                  <c:v>0.27189165903781004</c:v>
+                </c:pt>
+                <c:pt idx="542">
+                  <c:v>0.27258156658074478</c:v>
+                </c:pt>
+                <c:pt idx="543">
+                  <c:v>0.27301415725630412</c:v>
+                </c:pt>
+                <c:pt idx="544">
+                  <c:v>0.27301415725630412</c:v>
+                </c:pt>
+                <c:pt idx="545">
+                  <c:v>0.27317049238958635</c:v>
+                </c:pt>
+                <c:pt idx="546">
+                  <c:v>0.2743981829950487</c:v>
+                </c:pt>
+                <c:pt idx="547">
+                  <c:v>0.2743981829950487</c:v>
+                </c:pt>
+                <c:pt idx="548">
+                  <c:v>0.2743981829950487</c:v>
+                </c:pt>
+                <c:pt idx="549">
+                  <c:v>0.27496827536356561</c:v>
+                </c:pt>
+                <c:pt idx="550">
+                  <c:v>0.27532573868653099</c:v>
+                </c:pt>
+                <c:pt idx="551">
+                  <c:v>0.27532573868653099</c:v>
+                </c:pt>
+                <c:pt idx="552">
+                  <c:v>0.2754825860348295</c:v>
+                </c:pt>
+                <c:pt idx="553">
+                  <c:v>0.27667462588197977</c:v>
+                </c:pt>
+                <c:pt idx="554">
+                  <c:v>0.27667462588197977</c:v>
+                </c:pt>
+                <c:pt idx="555">
+                  <c:v>0.27667462588197977</c:v>
+                </c:pt>
+                <c:pt idx="556">
+                  <c:v>0.27724875608847649</c:v>
+                </c:pt>
+                <c:pt idx="557">
+                  <c:v>0.27760681578715246</c:v>
+                </c:pt>
+                <c:pt idx="558">
+                  <c:v>0.27760681578715246</c:v>
+                </c:pt>
+                <c:pt idx="559">
+                  <c:v>0.27774518194341385</c:v>
+                </c:pt>
+                <c:pt idx="560">
+                  <c:v>0.27879676473109771</c:v>
+                </c:pt>
+                <c:pt idx="561">
+                  <c:v>0.27879676473109771</c:v>
+                </c:pt>
+                <c:pt idx="562">
+                  <c:v>0.27879676473109771</c:v>
+                </c:pt>
+                <c:pt idx="563">
+                  <c:v>0.2794919277440428</c:v>
+                </c:pt>
+                <c:pt idx="564">
+                  <c:v>0.27992173283270577</c:v>
+                </c:pt>
+                <c:pt idx="565">
+                  <c:v>0.27992173283270577</c:v>
+                </c:pt>
+                <c:pt idx="566">
+                  <c:v>0.28010582773829334</c:v>
+                </c:pt>
+                <c:pt idx="567">
+                  <c:v>0.2814660845407857</c:v>
+                </c:pt>
+                <c:pt idx="568">
+                  <c:v>0.2814660845407857</c:v>
+                </c:pt>
+                <c:pt idx="569">
+                  <c:v>0.2814660845407857</c:v>
+                </c:pt>
+                <c:pt idx="570">
+                  <c:v>0.28205022538991864</c:v>
+                </c:pt>
+                <c:pt idx="571">
+                  <c:v>0.28241138774289076</c:v>
+                </c:pt>
+                <c:pt idx="572">
+                  <c:v>0.28241138774289076</c:v>
+                </c:pt>
+                <c:pt idx="573">
+                  <c:v>0.28254578010872977</c:v>
+                </c:pt>
+                <c:pt idx="574">
+                  <c:v>0.28353505724616046</c:v>
+                </c:pt>
+                <c:pt idx="575">
+                  <c:v>0.28353505724616046</c:v>
+                </c:pt>
+                <c:pt idx="576">
+                  <c:v>0.28353505724616046</c:v>
+                </c:pt>
+                <c:pt idx="577">
+                  <c:v>0.28428246674211327</c:v>
+                </c:pt>
+                <c:pt idx="578">
+                  <c:v>0.28473810675568184</c:v>
+                </c:pt>
+                <c:pt idx="579">
+                  <c:v>0.28473810675568184</c:v>
+                </c:pt>
+                <c:pt idx="580">
+                  <c:v>0.28487267575323849</c:v>
+                </c:pt>
+                <c:pt idx="581">
+                  <c:v>0.28586325309629029</c:v>
+                </c:pt>
+                <c:pt idx="582">
+                  <c:v>0.28586325309629029</c:v>
+                </c:pt>
+                <c:pt idx="583">
+                  <c:v>0.28586325309629029</c:v>
+                </c:pt>
+                <c:pt idx="584">
+                  <c:v>0.28647255457372733</c:v>
+                </c:pt>
+                <c:pt idx="585">
+                  <c:v>0.28684400039421554</c:v>
+                </c:pt>
+                <c:pt idx="586">
+                  <c:v>0.28684400039421554</c:v>
+                </c:pt>
+                <c:pt idx="587">
+                  <c:v>0.28696487662777098</c:v>
+                </c:pt>
+                <c:pt idx="588">
+                  <c:v>0.28782734488881728</c:v>
+                </c:pt>
+                <c:pt idx="589">
+                  <c:v>0.28782734488881728</c:v>
+                </c:pt>
+                <c:pt idx="590">
+                  <c:v>0.28782734488881728</c:v>
+                </c:pt>
+                <c:pt idx="591">
+                  <c:v>0.28844935141386413</c:v>
+                </c:pt>
+                <c:pt idx="592">
+                  <c:v>0.28882321703797637</c:v>
+                </c:pt>
+                <c:pt idx="593">
+                  <c:v>0.28882321703797637</c:v>
+                </c:pt>
+                <c:pt idx="594">
+                  <c:v>0.28900693676870076</c:v>
+                </c:pt>
+                <c:pt idx="595">
+                  <c:v>0.29031780187443373</c:v>
+                </c:pt>
+                <c:pt idx="596">
+                  <c:v>0.29031780187444639</c:v>
+                </c:pt>
+                <c:pt idx="597">
+                  <c:v>0.29031780187444639</c:v>
+                </c:pt>
+                <c:pt idx="598">
+                  <c:v>0.29094385587106131</c:v>
+                </c:pt>
+                <c:pt idx="599">
+                  <c:v>0.29132015428392777</c:v>
+                </c:pt>
+                <c:pt idx="600">
+                  <c:v>0.29132015428392777</c:v>
+                </c:pt>
+                <c:pt idx="601">
+                  <c:v>0.29146200324863297</c:v>
+                </c:pt>
+                <c:pt idx="602">
+                  <c:v>0.29244374739907275</c:v>
+                </c:pt>
+                <c:pt idx="603">
+                  <c:v>0.29244374739907275</c:v>
+                </c:pt>
+                <c:pt idx="604">
+                  <c:v>0.29244374739907275</c:v>
+                </c:pt>
+                <c:pt idx="605">
+                  <c:v>0.29304433989816436</c:v>
+                </c:pt>
+                <c:pt idx="606">
+                  <c:v>0.29340342430239219</c:v>
+                </c:pt>
+                <c:pt idx="607">
+                  <c:v>0.29340342430239219</c:v>
+                </c:pt>
+                <c:pt idx="608">
+                  <c:v>0.29353813533280521</c:v>
+                </c:pt>
+                <c:pt idx="609">
+                  <c:v>0.29447047746438565</c:v>
+                </c:pt>
+                <c:pt idx="610">
+                  <c:v>0.29447047746438565</c:v>
+                </c:pt>
+                <c:pt idx="611">
+                  <c:v>0.29447047746438565</c:v>
+                </c:pt>
+                <c:pt idx="612">
+                  <c:v>0.29525947188414942</c:v>
+                </c:pt>
+                <c:pt idx="613">
+                  <c:v>0.29572702413291296</c:v>
+                </c:pt>
+                <c:pt idx="614">
+                  <c:v>0.29572702413291296</c:v>
+                </c:pt>
+                <c:pt idx="615">
+                  <c:v>0.29585797958003651</c:v>
+                </c:pt>
+                <c:pt idx="616">
+                  <c:v>0.29674108939016364</c:v>
+                </c:pt>
+                <c:pt idx="617">
+                  <c:v>0.29674108939016364</c:v>
+                </c:pt>
+                <c:pt idx="618">
+                  <c:v>0.29674108939016364</c:v>
+                </c:pt>
+                <c:pt idx="619">
+                  <c:v>0.29739861271934798</c:v>
+                </c:pt>
+                <c:pt idx="620">
+                  <c:v>0.29778825617368326</c:v>
+                </c:pt>
+                <c:pt idx="621">
+                  <c:v>0.29778825617368326</c:v>
+                </c:pt>
+                <c:pt idx="622">
+                  <c:v>0.29790126214504098</c:v>
+                </c:pt>
+                <c:pt idx="623">
+                  <c:v>0.29866043046544627</c:v>
+                </c:pt>
+                <c:pt idx="624">
+                  <c:v>0.29866043046544627</c:v>
+                </c:pt>
+                <c:pt idx="625">
+                  <c:v>0.29866043046544627</c:v>
+                </c:pt>
+                <c:pt idx="626">
+                  <c:v>0.29914865006197089</c:v>
+                </c:pt>
+                <c:pt idx="627">
+                  <c:v>0.29943387308943398</c:v>
+                </c:pt>
+                <c:pt idx="628">
+                  <c:v>0.29943387308943398</c:v>
+                </c:pt>
+                <c:pt idx="629">
+                  <c:v>0.29959791535010188</c:v>
+                </c:pt>
+                <c:pt idx="630">
+                  <c:v>0.3006723921574882</c:v>
+                </c:pt>
+                <c:pt idx="631">
+                  <c:v>0.3006723921574882</c:v>
+                </c:pt>
+                <c:pt idx="632">
+                  <c:v>0.3006723921574882</c:v>
+                </c:pt>
+                <c:pt idx="633">
+                  <c:v>0.30131008887367916</c:v>
+                </c:pt>
+                <c:pt idx="634">
+                  <c:v>0.30168263800787437</c:v>
+                </c:pt>
+                <c:pt idx="635">
+                  <c:v>0.30168263800786155</c:v>
+                </c:pt>
+                <c:pt idx="636">
+                  <c:v>0.30182544744977585</c:v>
+                </c:pt>
+                <c:pt idx="637">
+                  <c:v>0.30275727905819722</c:v>
+                </c:pt>
+                <c:pt idx="638">
+                  <c:v>0.30275727905819722</c:v>
+                </c:pt>
+                <c:pt idx="639">
+                  <c:v>0.30275727905819722</c:v>
+                </c:pt>
+                <c:pt idx="640">
+                  <c:v>0.30340056987310132</c:v>
+                </c:pt>
+                <c:pt idx="641">
+                  <c:v>0.30377105149425399</c:v>
+                </c:pt>
+                <c:pt idx="642">
+                  <c:v>0.30377105149425399</c:v>
+                </c:pt>
+                <c:pt idx="643">
+                  <c:v>0.30389801822253587</c:v>
+                </c:pt>
+                <c:pt idx="644">
+                  <c:v>0.30472647612457088</c:v>
+                </c:pt>
+                <c:pt idx="645">
+                  <c:v>0.30472647612458353</c:v>
+                </c:pt>
+                <c:pt idx="646">
+                  <c:v>0.30472647612458353</c:v>
+                </c:pt>
+                <c:pt idx="647">
+                  <c:v>0.30516219279222467</c:v>
+                </c:pt>
+                <c:pt idx="648">
+                  <c:v>0.30541312909296503</c:v>
+                </c:pt>
+                <c:pt idx="649">
+                  <c:v>0.30541312909296503</c:v>
+                </c:pt>
+                <c:pt idx="650">
+                  <c:v>0.30558466292780084</c:v>
+                </c:pt>
+                <c:pt idx="651">
+                  <c:v>0.30667243846580028</c:v>
+                </c:pt>
+                <c:pt idx="652">
+                  <c:v>0.30667243846580028</c:v>
+                </c:pt>
+                <c:pt idx="653">
+                  <c:v>0.30667243846580028</c:v>
+                </c:pt>
+                <c:pt idx="654">
+                  <c:v>0.30737888405590535</c:v>
+                </c:pt>
+                <c:pt idx="655">
+                  <c:v>0.3077836185085816</c:v>
+                </c:pt>
+                <c:pt idx="656">
+                  <c:v>0.3077836185085816</c:v>
+                </c:pt>
+                <c:pt idx="657">
+                  <c:v>0.30786266551162017</c:v>
+                </c:pt>
+                <c:pt idx="658">
+                  <c:v>0.30836393918950206</c:v>
+                </c:pt>
+                <c:pt idx="659">
+                  <c:v>0.30836393918950206</c:v>
+                </c:pt>
+                <c:pt idx="660">
+                  <c:v>0.30836393918950206</c:v>
+                </c:pt>
+                <c:pt idx="661">
+                  <c:v>0.30900105584647597</c:v>
+                </c:pt>
+                <c:pt idx="662">
+                  <c:v>0.30936275228195659</c:v>
+                </c:pt>
+                <c:pt idx="663">
+                  <c:v>0.30936275228195659</c:v>
+                </c:pt>
+                <c:pt idx="664">
+                  <c:v>0.30950088277578469</c:v>
+                </c:pt>
+                <c:pt idx="665">
+                  <c:v>0.31035597630901401</c:v>
+                </c:pt>
+                <c:pt idx="666">
+                  <c:v>0.31035597630901401</c:v>
+                </c:pt>
+                <c:pt idx="667">
+                  <c:v>0.31035597630901401</c:v>
+                </c:pt>
+                <c:pt idx="668">
+                  <c:v>0.31105314837079312</c:v>
+                </c:pt>
+                <c:pt idx="669">
+                  <c:v>0.31144688803263365</c:v>
+                </c:pt>
+                <c:pt idx="670">
+                  <c:v>0.31144688803263365</c:v>
+                </c:pt>
+                <c:pt idx="671">
+                  <c:v>0.31156372280076572</c:v>
+                </c:pt>
+                <c:pt idx="672">
+                  <c:v>0.31228420387096423</c:v>
+                </c:pt>
+                <c:pt idx="673">
+                  <c:v>0.31228420387096423</c:v>
+                </c:pt>
+                <c:pt idx="674">
+                  <c:v>0.31228420387096423</c:v>
+                </c:pt>
+                <c:pt idx="675">
+                  <c:v>0.31263201737574109</c:v>
+                </c:pt>
+                <c:pt idx="676">
+                  <c:v>0.31282664876701932</c:v>
+                </c:pt>
+                <c:pt idx="677">
+                  <c:v>0.31282664876701932</c:v>
+                </c:pt>
+                <c:pt idx="678">
+                  <c:v>0.31294831643680632</c:v>
+                </c:pt>
+                <c:pt idx="679">
+                  <c:v>0.31368115193629709</c:v>
+                </c:pt>
+                <c:pt idx="680">
+                  <c:v>0.31368115193629709</c:v>
+                </c:pt>
+                <c:pt idx="681">
+                  <c:v>0.31368115193629709</c:v>
+                </c:pt>
+                <c:pt idx="682">
+                  <c:v>0.31412641885529474</c:v>
+                </c:pt>
+                <c:pt idx="683">
+                  <c:v>0.3143755837633519</c:v>
+                </c:pt>
+                <c:pt idx="684">
+                  <c:v>0.31437558376333902</c:v>
+                </c:pt>
+                <c:pt idx="685">
+                  <c:v>0.31446694579461754</c:v>
+                </c:pt>
+                <c:pt idx="686">
+                  <c:v>0.31501511798221232</c:v>
+                </c:pt>
+                <c:pt idx="687">
+                  <c:v>0.31501511798221232</c:v>
+                </c:pt>
+                <c:pt idx="688">
+                  <c:v>0.31501511798222503</c:v>
+                </c:pt>
+                <c:pt idx="689">
+                  <c:v>0.31556488442325009</c:v>
+                </c:pt>
+                <c:pt idx="690">
+                  <c:v>0.31586810612010835</c:v>
+                </c:pt>
+                <c:pt idx="691">
+                  <c:v>0.31586810612010835</c:v>
+                </c:pt>
+                <c:pt idx="692">
+                  <c:v>0.31605653383024307</c:v>
+                </c:pt>
+                <c:pt idx="693">
+                  <c:v>0.3171871000910777</c:v>
+                </c:pt>
+                <c:pt idx="694">
+                  <c:v>0.3171871000910777</c:v>
+                </c:pt>
+                <c:pt idx="695">
+                  <c:v>0.3171871000910777</c:v>
+                </c:pt>
+                <c:pt idx="696">
+                  <c:v>0.31772978510643174</c:v>
+                </c:pt>
+                <c:pt idx="697">
+                  <c:v>0.3180291010685109</c:v>
+                </c:pt>
+                <c:pt idx="698">
+                  <c:v>0.3180291010685109</c:v>
+                </c:pt>
+                <c:pt idx="699">
+                  <c:v>0.31817747982317385</c:v>
+                </c:pt>
+                <c:pt idx="700">
+                  <c:v>0.31904414664019337</c:v>
+                </c:pt>
+                <c:pt idx="701">
+                  <c:v>0.31904414664019337</c:v>
+                </c:pt>
+                <c:pt idx="702">
+                  <c:v>0.31904414664019337</c:v>
+                </c:pt>
+                <c:pt idx="703">
+                  <c:v>0.31972696426641928</c:v>
+                </c:pt>
+                <c:pt idx="704">
+                  <c:v>0.32010163855363771</c:v>
+                </c:pt>
+                <c:pt idx="705">
+                  <c:v>0.32010163855363771</c:v>
+                </c:pt>
+                <c:pt idx="706">
+                  <c:v>0.3201727739281503</c:v>
+                </c:pt>
+                <c:pt idx="707">
+                  <c:v>0.32058826918384786</c:v>
+                </c:pt>
+                <c:pt idx="708">
+                  <c:v>0.32058826918386074</c:v>
+                </c:pt>
+                <c:pt idx="709">
+                  <c:v>0.32058826918386074</c:v>
+                </c:pt>
+                <c:pt idx="710">
+                  <c:v>0.32089974244913733</c:v>
+                </c:pt>
+                <c:pt idx="711">
+                  <c:v>0.32106905612156156</c:v>
+                </c:pt>
+                <c:pt idx="712">
+                  <c:v>0.32106905612156156</c:v>
+                </c:pt>
+                <c:pt idx="713">
+                  <c:v>0.32126144764006065</c:v>
+                </c:pt>
+                <c:pt idx="714">
+                  <c:v>0.32235594161205</c:v>
+                </c:pt>
+                <c:pt idx="715">
+                  <c:v>0.32235594161205</c:v>
+                </c:pt>
+                <c:pt idx="716">
+                  <c:v>0.32235594161205</c:v>
+                </c:pt>
+                <c:pt idx="717">
+                  <c:v>0.32293852223516684</c:v>
+                </c:pt>
+                <c:pt idx="718">
+                  <c:v>0.32325359134768394</c:v>
+                </c:pt>
+                <c:pt idx="719">
+                  <c:v>0.32325359134768394</c:v>
+                </c:pt>
+                <c:pt idx="720">
+                  <c:v>0.32342115735593574</c:v>
+                </c:pt>
+                <c:pt idx="721">
+                  <c:v>0.32437442175850834</c:v>
+                </c:pt>
+                <c:pt idx="722">
+                  <c:v>0.32437442175850834</c:v>
+                </c:pt>
+                <c:pt idx="723">
+                  <c:v>0.32437442175850834</c:v>
+                </c:pt>
+                <c:pt idx="724">
+                  <c:v>0.32481500366529681</c:v>
+                </c:pt>
+                <c:pt idx="725">
+                  <c:v>0.32505102968680288</c:v>
+                </c:pt>
+                <c:pt idx="726">
+                  <c:v>0.32505102968680288</c:v>
+                </c:pt>
+                <c:pt idx="727">
+                  <c:v>0.32516555961866639</c:v>
+                </c:pt>
+                <c:pt idx="728">
+                  <c:v>0.32580294358735939</c:v>
+                </c:pt>
+                <c:pt idx="729">
+                  <c:v>0.32580294358735939</c:v>
+                </c:pt>
+                <c:pt idx="730">
+                  <c:v>0.32580294358735939</c:v>
+                </c:pt>
+                <c:pt idx="731">
+                  <c:v>0.32619979476579336</c:v>
+                </c:pt>
+                <c:pt idx="732">
+                  <c:v>0.32641239361139646</c:v>
+                </c:pt>
+                <c:pt idx="733">
+                  <c:v>0.32641239361139646</c:v>
+                </c:pt>
+                <c:pt idx="734">
+                  <c:v>0.3265249536892047</c:v>
+                </c:pt>
+                <c:pt idx="735">
+                  <c:v>0.32714892803359424</c:v>
+                </c:pt>
+                <c:pt idx="736">
+                  <c:v>0.32714892803359424</c:v>
+                </c:pt>
+                <c:pt idx="737">
+                  <c:v>0.32714892803358142</c:v>
+                </c:pt>
+                <c:pt idx="738">
+                  <c:v>0.32787007104970545</c:v>
+                </c:pt>
+                <c:pt idx="739">
+                  <c:v>0.32825077599223901</c:v>
+                </c:pt>
+                <c:pt idx="740">
+                  <c:v>0.32825077599223901</c:v>
+                </c:pt>
+                <c:pt idx="741">
+                  <c:v>0.32833761060940636</c:v>
+                </c:pt>
+                <c:pt idx="742">
+                  <c:v>0.32881897642198993</c:v>
+                </c:pt>
+                <c:pt idx="743">
+                  <c:v>0.32881897642200258</c:v>
+                </c:pt>
+                <c:pt idx="744">
+                  <c:v>0.32881897642200258</c:v>
+                </c:pt>
+                <c:pt idx="745">
+                  <c:v>0.32940999106149899</c:v>
+                </c:pt>
+                <c:pt idx="746">
+                  <c:v>0.3297219987899771</c:v>
+                </c:pt>
+                <c:pt idx="747">
+                  <c:v>0.3297219987899771</c:v>
+                </c:pt>
+                <c:pt idx="748">
+                  <c:v>0.32986735589891947</c:v>
+                </c:pt>
+                <c:pt idx="749">
+                  <c:v>0.3306529028281549</c:v>
+                </c:pt>
+                <c:pt idx="750">
+                  <c:v>0.3306529028281549</c:v>
+                </c:pt>
+                <c:pt idx="751">
+                  <c:v>0.3306529028281549</c:v>
+                </c:pt>
+                <c:pt idx="752">
+                  <c:v>0.33082862244530131</c:v>
+                </c:pt>
+                <c:pt idx="753">
+                  <c:v>0.33092003214513294</c:v>
+                </c:pt>
+                <c:pt idx="754">
+                  <c:v>0.33092003214513294</c:v>
+                </c:pt>
+                <c:pt idx="755">
+                  <c:v>0.33107431118552644</c:v>
+                </c:pt>
+                <c:pt idx="756">
+                  <c:v>0.33190807451019366</c:v>
+                </c:pt>
+                <c:pt idx="757">
+                  <c:v>0.33190807451020649</c:v>
+                </c:pt>
+                <c:pt idx="758">
+                  <c:v>0.33190807451020649</c:v>
+                </c:pt>
+                <c:pt idx="759">
+                  <c:v>0.33230159700999323</c:v>
+                </c:pt>
+                <c:pt idx="760">
+                  <c:v>0.33250630820938099</c:v>
+                </c:pt>
+                <c:pt idx="761">
+                  <c:v>0.33250630820936833</c:v>
+                </c:pt>
+                <c:pt idx="762">
+                  <c:v>0.33261670505633451</c:v>
+                </c:pt>
+                <c:pt idx="763">
+                  <c:v>0.33319858843721545</c:v>
+                </c:pt>
+                <c:pt idx="764">
+                  <c:v>0.33319858843721545</c:v>
+                </c:pt>
+                <c:pt idx="765">
+                  <c:v>0.33319858843721545</c:v>
+                </c:pt>
+                <c:pt idx="766">
+                  <c:v>0.33382513620899212</c:v>
+                </c:pt>
+                <c:pt idx="767">
+                  <c:v>0.33414942977929241</c:v>
+                </c:pt>
+                <c:pt idx="768">
+                  <c:v>0.33414942977929241</c:v>
+                </c:pt>
+                <c:pt idx="769">
+                  <c:v>0.33426738524516186</c:v>
+                </c:pt>
+                <c:pt idx="770">
+                  <c:v>0.33488910884649842</c:v>
+                </c:pt>
+                <c:pt idx="771">
+                  <c:v>0.33488910884649842</c:v>
+                </c:pt>
+                <c:pt idx="772">
+                  <c:v>0.33488910884649842</c:v>
+                </c:pt>
+                <c:pt idx="773">
+                  <c:v>0.33540354370135911</c:v>
+                </c:pt>
+                <c:pt idx="774">
+                  <c:v>0.33566722387823233</c:v>
+                </c:pt>
+                <c:pt idx="775">
+                  <c:v>0.33566722387823233</c:v>
+                </c:pt>
+                <c:pt idx="776">
+                  <c:v>0.33577703355437338</c:v>
+                </c:pt>
+                <c:pt idx="777">
+                  <c:v>0.33634401004551456</c:v>
+                </c:pt>
+                <c:pt idx="778">
+                  <c:v>0.33634401004551456</c:v>
+                </c:pt>
+                <c:pt idx="779">
+                  <c:v>0.33634401004551456</c:v>
+                </c:pt>
+                <c:pt idx="780">
+                  <c:v>0.33666332024306217</c:v>
+                </c:pt>
+                <c:pt idx="781">
+                  <c:v>0.33682698677647888</c:v>
+                </c:pt>
+                <c:pt idx="782">
+                  <c:v>0.33682698677649159</c:v>
+                </c:pt>
+                <c:pt idx="783">
+                  <c:v>0.33695480692860397</c:v>
+                </c:pt>
+                <c:pt idx="784">
+                  <c:v>0.33761216771094854</c:v>
+                </c:pt>
+                <c:pt idx="785">
+                  <c:v>0.33761216771094854</c:v>
+                </c:pt>
+                <c:pt idx="786">
+                  <c:v>0.33761216771093572</c:v>
+                </c:pt>
+                <c:pt idx="787">
+                  <c:v>0.33793239727315127</c:v>
+                </c:pt>
+                <c:pt idx="788">
+                  <c:v>0.33809411320205612</c:v>
+                </c:pt>
+                <c:pt idx="789">
+                  <c:v>0.33809411320205612</c:v>
+                </c:pt>
+                <c:pt idx="790">
+                  <c:v>0.33824978564991187</c:v>
+                </c:pt>
+                <c:pt idx="791">
+                  <c:v>0.3390343747870958</c:v>
+                </c:pt>
+                <c:pt idx="792">
+                  <c:v>0.3390343747870958</c:v>
+                </c:pt>
+                <c:pt idx="793">
+                  <c:v>0.3390343747870958</c:v>
+                </c:pt>
+                <c:pt idx="794">
+                  <c:v>0.33992199141035762</c:v>
+                </c:pt>
+                <c:pt idx="795">
+                  <c:v>0.34037023780510617</c:v>
+                </c:pt>
+                <c:pt idx="796">
+                  <c:v>0.34037023780509351</c:v>
+                </c:pt>
+                <c:pt idx="797">
+                  <c:v>0.34051331752397435</c:v>
+                </c:pt>
+                <c:pt idx="798">
+                  <c:v>0.34123157771269425</c:v>
+                </c:pt>
+                <c:pt idx="799">
+                  <c:v>0.34123157771269425</c:v>
+                </c:pt>
+                <c:pt idx="800">
+                  <c:v>0.34123157771269425</c:v>
+                </c:pt>
+                <c:pt idx="801">
+                  <c:v>0.34166321598975213</c:v>
+                </c:pt>
+                <c:pt idx="802">
+                  <c:v>0.34187796140123383</c:v>
+                </c:pt>
+                <c:pt idx="803">
+                  <c:v>0.34187796140123383</c:v>
+                </c:pt>
+                <c:pt idx="804">
+                  <c:v>0.34196918516405056</c:v>
+                </c:pt>
+                <c:pt idx="805">
+                  <c:v>0.34242712845339285</c:v>
+                </c:pt>
+                <c:pt idx="806">
+                  <c:v>0.34242712845337997</c:v>
+                </c:pt>
+                <c:pt idx="807">
+                  <c:v>0.34242712845337997</c:v>
+                </c:pt>
+                <c:pt idx="808">
+                  <c:v>0.3428452150687965</c:v>
+                </c:pt>
+                <c:pt idx="809">
+                  <c:v>0.3430532183600582</c:v>
+                </c:pt>
+                <c:pt idx="810">
+                  <c:v>0.3430532183600582</c:v>
+                </c:pt>
+                <c:pt idx="811">
+                  <c:v>0.34316982472512542</c:v>
+                </c:pt>
+                <c:pt idx="812">
+                  <c:v>0.34374142455390311</c:v>
+                </c:pt>
+                <c:pt idx="813">
+                  <c:v>0.34374142455390311</c:v>
+                </c:pt>
+                <c:pt idx="814">
+                  <c:v>0.34374142455390311</c:v>
+                </c:pt>
+                <c:pt idx="815">
+                  <c:v>0.34414407974844047</c:v>
+                </c:pt>
+                <c:pt idx="816">
+                  <c:v>0.34434341400316099</c:v>
+                </c:pt>
+                <c:pt idx="817">
+                  <c:v>0.34434341400316099</c:v>
+                </c:pt>
+                <c:pt idx="818">
+                  <c:v>0.34448811280371733</c:v>
+                </c:pt>
+                <c:pt idx="819">
+                  <c:v>0.34519742064955738</c:v>
+                </c:pt>
+                <c:pt idx="820">
+                  <c:v>0.34519742064955738</c:v>
+                </c:pt>
+                <c:pt idx="821">
+                  <c:v>0.34519742064955738</c:v>
+                </c:pt>
+                <c:pt idx="822">
+                  <c:v>0.34560070441976054</c:v>
+                </c:pt>
+                <c:pt idx="823">
+                  <c:v>0.34579835339625847</c:v>
+                </c:pt>
+                <c:pt idx="824">
+                  <c:v>0.34579835339625847</c:v>
+                </c:pt>
+                <c:pt idx="825">
+                  <c:v>0.34583399562906875</c:v>
+                </c:pt>
+                <c:pt idx="826">
+                  <c:v>0.34600535251764608</c:v>
+                </c:pt>
+                <c:pt idx="827">
+                  <c:v>0.34600535251764608</c:v>
+                </c:pt>
+                <c:pt idx="828">
+                  <c:v>0.34600535251764608</c:v>
+                </c:pt>
+                <c:pt idx="829">
+                  <c:v>0.34648515605324298</c:v>
+                </c:pt>
+                <c:pt idx="830">
+                  <c:v>0.34672030729098757</c:v>
+                </c:pt>
+                <c:pt idx="831">
+                  <c:v>0.34672030729098757</c:v>
+                </c:pt>
+                <c:pt idx="832">
+                  <c:v>0.34684973535840852</c:v>
+                </c:pt>
+                <c:pt idx="833">
+                  <c:v>0.34746949668129234</c:v>
+                </c:pt>
+                <c:pt idx="834">
+                  <c:v>0.347469496681305</c:v>
+                </c:pt>
+                <c:pt idx="835">
+                  <c:v>0.34746949668129234</c:v>
+                </c:pt>
+                <c:pt idx="836">
+                  <c:v>0.34768014348428777</c:v>
+                </c:pt>
+                <c:pt idx="837">
+                  <c:v>0.34778183504436555</c:v>
+                </c:pt>
+                <c:pt idx="838">
+                  <c:v>0.34778183504436555</c:v>
+                </c:pt>
+                <c:pt idx="839">
+                  <c:v>0.34789321097242615</c:v>
+                </c:pt>
+                <c:pt idx="840">
+                  <c:v>0.3484164676910797</c:v>
+                </c:pt>
+                <c:pt idx="841">
+                  <c:v>0.3484164676910797</c:v>
+                </c:pt>
+                <c:pt idx="842">
+                  <c:v>0.3484164676910797</c:v>
+                </c:pt>
+                <c:pt idx="843">
+                  <c:v>0.3491011191718178</c:v>
+                </c:pt>
+                <c:pt idx="844">
+                  <c:v>0.34943164057632464</c:v>
+                </c:pt>
+                <c:pt idx="845">
+                  <c:v>0.34943164057632464</c:v>
+                </c:pt>
+                <c:pt idx="846">
+                  <c:v>0.34959783599697536</c:v>
+                </c:pt>
+                <c:pt idx="847">
+                  <c:v>0.35037550513517263</c:v>
+                </c:pt>
+                <c:pt idx="848">
+                  <c:v>0.35037550513517263</c:v>
+                </c:pt>
+                <c:pt idx="849">
+                  <c:v>0.35037550513517263</c:v>
+                </c:pt>
+                <c:pt idx="850">
+                  <c:v>0.35062215253383072</c:v>
+                </c:pt>
+                <c:pt idx="851">
+                  <c:v>0.35073943095377497</c:v>
+                </c:pt>
+                <c:pt idx="852">
+                  <c:v>0.35073943095377497</c:v>
+                </c:pt>
+                <c:pt idx="853">
+                  <c:v>0.35080148438781444</c:v>
+                </c:pt>
+                <c:pt idx="854">
+                  <c:v>0.3510918476263461</c:v>
+                </c:pt>
+                <c:pt idx="855">
+                  <c:v>0.3510918476263461</c:v>
+                </c:pt>
+                <c:pt idx="856">
+                  <c:v>0.3510918476263461</c:v>
+                </c:pt>
+                <c:pt idx="857">
+                  <c:v>0.35140612568131291</c:v>
+                </c:pt>
+                <c:pt idx="858">
+                  <c:v>0.35155556181530595</c:v>
+                </c:pt>
+                <c:pt idx="859">
+                  <c:v>0.35155556181529329</c:v>
+                </c:pt>
+                <c:pt idx="860">
+                  <c:v>0.35170004959678991</c:v>
+                </c:pt>
+                <c:pt idx="861">
+                  <c:v>0.35236094741214313</c:v>
+                </c:pt>
+                <c:pt idx="862">
+                  <c:v>0.35236094741214313</c:v>
+                </c:pt>
+                <c:pt idx="863">
+                  <c:v>0.35236094741214313</c:v>
+                </c:pt>
+                <c:pt idx="864">
+                  <c:v>0.35267654993474934</c:v>
+                </c:pt>
+                <c:pt idx="865">
+                  <c:v>0.35282588381130364</c:v>
+                </c:pt>
+                <c:pt idx="866">
+                  <c:v>0.35282588381130364</c:v>
+                </c:pt>
+                <c:pt idx="867">
+                  <c:v>0.35296278175880147</c:v>
+                </c:pt>
+                <c:pt idx="868">
+                  <c:v>0.35358896311129784</c:v>
+                </c:pt>
+                <c:pt idx="869">
+                  <c:v>0.35358896311129784</c:v>
+                </c:pt>
+                <c:pt idx="870">
+                  <c:v>0.35358896311129784</c:v>
+                </c:pt>
+                <c:pt idx="871">
+                  <c:v>0.35384387764362868</c:v>
+                </c:pt>
+                <c:pt idx="872">
+                  <c:v>0.35396325225390635</c:v>
+                </c:pt>
+                <c:pt idx="873">
+                  <c:v>0.35396325225390635</c:v>
+                </c:pt>
+                <c:pt idx="874">
+                  <c:v>0.3541324832782361</c:v>
+                </c:pt>
+                <c:pt idx="875">
+                  <c:v>0.35488940749620046</c:v>
+                </c:pt>
+                <c:pt idx="876">
+                  <c:v>0.35488940749620046</c:v>
+                </c:pt>
+                <c:pt idx="877">
+                  <c:v>0.35488940749620046</c:v>
+                </c:pt>
+                <c:pt idx="878">
+                  <c:v>0.3554069398260889</c:v>
+                </c:pt>
+                <c:pt idx="879">
+                  <c:v>0.35564811994098555</c:v>
+                </c:pt>
+                <c:pt idx="880">
+                  <c:v>0.35564811994098555</c:v>
+                </c:pt>
+                <c:pt idx="881">
+                  <c:v>0.35577935738370342</c:v>
+                </c:pt>
+                <c:pt idx="882">
+                  <c:v>0.3563663466728979</c:v>
+                </c:pt>
+                <c:pt idx="883">
+                  <c:v>0.3563663466728979</c:v>
+                </c:pt>
+                <c:pt idx="884">
+                  <c:v>0.3563663466728979</c:v>
+                </c:pt>
+                <c:pt idx="885">
+                  <c:v>0.35686603734830374</c:v>
+                </c:pt>
+                <c:pt idx="886">
+                  <c:v>0.35709647722289817</c:v>
+                </c:pt>
+                <c:pt idx="887">
+                  <c:v>0.35709647722289817</c:v>
+                </c:pt>
+                <c:pt idx="888">
+                  <c:v>0.35727981785886409</c:v>
+                </c:pt>
+                <c:pt idx="889">
+                  <c:v>0.35808520708119668</c:v>
+                </c:pt>
+                <c:pt idx="890">
+                  <c:v>0.35808520708119668</c:v>
+                </c:pt>
+                <c:pt idx="891">
+                  <c:v>0.35808520708119668</c:v>
+                </c:pt>
+                <c:pt idx="892">
+                  <c:v>0.35820688627842495</c:v>
+                </c:pt>
+                <c:pt idx="893">
+                  <c:v>0.35826300047133008</c:v>
+                </c:pt>
+                <c:pt idx="894">
+                  <c:v>0.35826300047133008</c:v>
+                </c:pt>
+                <c:pt idx="895">
+                  <c:v>0.35840479106635692</c:v>
+                </c:pt>
+                <c:pt idx="896">
+                  <c:v>0.35902512491960487</c:v>
+                </c:pt>
+                <c:pt idx="897">
+                  <c:v>0.35902512491960487</c:v>
+                </c:pt>
+                <c:pt idx="898">
+                  <c:v>0.35902512491960487</c:v>
+                </c:pt>
+                <c:pt idx="899">
+                  <c:v>0.35942150169641096</c:v>
+                </c:pt>
+                <c:pt idx="900">
+                  <c:v>0.35960149888007292</c:v>
+                </c:pt>
+                <c:pt idx="901">
+                  <c:v>0.35960149888007292</c:v>
+                </c:pt>
+                <c:pt idx="902">
+                  <c:v>0.35966411820386462</c:v>
+                </c:pt>
+                <c:pt idx="903">
+                  <c:v>0.35993807774545999</c:v>
+                </c:pt>
+                <c:pt idx="904">
+                  <c:v>0.35993807774545999</c:v>
+                </c:pt>
+                <c:pt idx="905">
+                  <c:v>0.35993807774545999</c:v>
+                </c:pt>
+                <c:pt idx="906">
+                  <c:v>0.36049403137183911</c:v>
+                </c:pt>
+                <c:pt idx="907">
+                  <c:v>0.36074649340508635</c:v>
+                </c:pt>
+                <c:pt idx="908">
+                  <c:v>0.36074649340508635</c:v>
+                </c:pt>
+                <c:pt idx="909">
+                  <c:v>0.36084063023756197</c:v>
+                </c:pt>
+                <c:pt idx="910">
+                  <c:v>0.36124360194150912</c:v>
+                </c:pt>
+                <c:pt idx="911">
+                  <c:v>0.36124360194150912</c:v>
+                </c:pt>
+                <c:pt idx="912">
+                  <c:v>0.36124360194149646</c:v>
+                </c:pt>
+                <c:pt idx="913">
+                  <c:v>0.36158110994210357</c:v>
+                </c:pt>
+                <c:pt idx="914">
+                  <c:v>0.36173201496160817</c:v>
+                </c:pt>
+                <c:pt idx="915">
+                  <c:v>0.36173201496160817</c:v>
+                </c:pt>
+                <c:pt idx="916">
+                  <c:v>0.36176505904873374</c:v>
+                </c:pt>
+                <c:pt idx="917">
+                  <c:v>0.36190651093047083</c:v>
+                </c:pt>
+                <c:pt idx="918">
+                  <c:v>0.36190651093047083</c:v>
+                </c:pt>
+                <c:pt idx="919">
+                  <c:v>0.36190651093047083</c:v>
+                </c:pt>
+                <c:pt idx="920">
+                  <c:v>0.36252632986168504</c:v>
+                </c:pt>
+                <c:pt idx="921">
+                  <c:v>0.36280346044151057</c:v>
+                </c:pt>
+                <c:pt idx="922">
+                  <c:v>0.36280346044151057</c:v>
+                </c:pt>
+                <c:pt idx="923">
+                  <c:v>0.36289314028417408</c:v>
+                </c:pt>
+                <c:pt idx="924">
+                  <c:v>0.36326886790085267</c:v>
+                </c:pt>
+                <c:pt idx="925">
+                  <c:v>0.36326886790085267</c:v>
+                </c:pt>
+                <c:pt idx="926">
+                  <c:v>0.36326886790085267</c:v>
+                </c:pt>
+                <c:pt idx="927">
+                  <c:v>0.36379702969067468</c:v>
+                </c:pt>
+                <c:pt idx="928">
+                  <c:v>0.36403204905169684</c:v>
+                </c:pt>
+                <c:pt idx="929">
+                  <c:v>0.36403204905169684</c:v>
+                </c:pt>
+                <c:pt idx="930">
+                  <c:v>0.36414169563687243</c:v>
+                </c:pt>
+                <c:pt idx="931">
+                  <c:v>0.36460107701961703</c:v>
+                </c:pt>
+                <c:pt idx="932">
+                  <c:v>0.36460107701961703</c:v>
+                </c:pt>
+                <c:pt idx="933">
+                  <c:v>0.36460107701961703</c:v>
+                </c:pt>
+                <c:pt idx="934">
+                  <c:v>0.36506590425056784</c:v>
+                </c:pt>
+                <c:pt idx="935">
+                  <c:v>0.36527051719433867</c:v>
+                </c:pt>
+                <c:pt idx="936">
+                  <c:v>0.36527051719433867</c:v>
+                </c:pt>
+                <c:pt idx="937">
+                  <c:v>0.36525296963346005</c:v>
+                </c:pt>
+                <c:pt idx="938">
+                  <c:v>0.36518069747594345</c:v>
+                </c:pt>
+                <c:pt idx="939">
+                  <c:v>0.36518069747594345</c:v>
+                </c:pt>
+                <c:pt idx="940">
+                  <c:v>0.36518069747594345</c:v>
+                </c:pt>
+                <c:pt idx="941">
+                  <c:v>0.36523672567930782</c:v>
+                </c:pt>
+                <c:pt idx="942">
+                  <c:v>0.36526138881190229</c:v>
+                </c:pt>
+                <c:pt idx="943">
+                  <c:v>0.36526138881190229</c:v>
+                </c:pt>
+                <c:pt idx="944">
+                  <c:v>0.36534037934862584</c:v>
+                </c:pt>
+                <c:pt idx="945">
+                  <c:v>0.36566437443151467</c:v>
+                </c:pt>
+                <c:pt idx="946">
+                  <c:v>0.36566437443151467</c:v>
+                </c:pt>
+                <c:pt idx="947">
+                  <c:v>0.36566437443151467</c:v>
+                </c:pt>
+                <c:pt idx="948">
+                  <c:v>0.36616992178458585</c:v>
+                </c:pt>
+                <c:pt idx="949">
+                  <c:v>0.36638899230425548</c:v>
+                </c:pt>
+                <c:pt idx="950">
+                  <c:v>0.36638899230425548</c:v>
+                </c:pt>
+                <c:pt idx="951">
+                  <c:v>0.36646874147754505</c:v>
+                </c:pt>
+                <c:pt idx="952">
+                  <c:v>0.36679584825617029</c:v>
+                </c:pt>
+                <c:pt idx="953">
+                  <c:v>0.36679584825617029</c:v>
+                </c:pt>
+                <c:pt idx="954">
+                  <c:v>0.36679584825617029</c:v>
+                </c:pt>
+                <c:pt idx="955">
+                  <c:v>0.36690361770648622</c:v>
+                </c:pt>
+                <c:pt idx="956">
+                  <c:v>0.36695031780164022</c:v>
+                </c:pt>
+                <c:pt idx="957">
+                  <c:v>0.36695031780164022</c:v>
+                </c:pt>
+                <c:pt idx="958">
+                  <c:v>0.3670111516901774</c:v>
+                </c:pt>
+                <c:pt idx="959">
+                  <c:v>0.3672555011424713</c:v>
+                </c:pt>
+                <c:pt idx="960">
+                  <c:v>0.3672555011424713</c:v>
+                </c:pt>
+                <c:pt idx="961">
+                  <c:v>0.36725550114248395</c:v>
+                </c:pt>
+                <c:pt idx="962">
+                  <c:v>0.36820037938798417</c:v>
+                </c:pt>
+                <c:pt idx="963">
+                  <c:v>0.36860340802351377</c:v>
+                </c:pt>
+                <c:pt idx="964">
+                  <c:v>0.36860340802351377</c:v>
+                </c:pt>
+                <c:pt idx="965">
+                  <c:v>0.36870624777425987</c:v>
+                </c:pt>
+                <c:pt idx="966">
+                  <c:v>0.36911932077312848</c:v>
+                </c:pt>
+                <c:pt idx="967">
+                  <c:v>0.36911932077312848</c:v>
+                </c:pt>
+                <c:pt idx="968">
+                  <c:v>0.36911932077312848</c:v>
+                </c:pt>
+                <c:pt idx="969">
+                  <c:v>0.36983876265164323</c:v>
+                </c:pt>
+                <c:pt idx="970">
+                  <c:v>0.37014563359509867</c:v>
+                </c:pt>
+                <c:pt idx="971">
+                  <c:v>0.37014563359509867</c:v>
+                </c:pt>
+                <c:pt idx="972">
+                  <c:v>0.37039785986560264</c:v>
+                </c:pt>
+                <c:pt idx="973">
+                  <c:v>0.37139022552010031</c:v>
+                </c:pt>
+                <c:pt idx="974">
+                  <c:v>0.37139022552010031</c:v>
+                </c:pt>
+                <c:pt idx="975">
+                  <c:v>0.37139022552010031</c:v>
+                </c:pt>
+                <c:pt idx="976">
+                  <c:v>0.37184108264118876</c:v>
+                </c:pt>
+                <c:pt idx="977">
+                  <c:v>0.37203248424921287</c:v>
+                </c:pt>
+                <c:pt idx="978">
+                  <c:v>0.37203248424921287</c:v>
+                </c:pt>
+                <c:pt idx="979">
+                  <c:v>0.3721493193134251</c:v>
+                </c:pt>
+                <c:pt idx="980">
+                  <c:v>0.37260899825461224</c:v>
+                </c:pt>
+                <c:pt idx="981">
+                  <c:v>0.37260899825461224</c:v>
+                </c:pt>
+                <c:pt idx="982">
+                  <c:v>0.37260899825461224</c:v>
+                </c:pt>
+                <c:pt idx="983">
+                  <c:v>0.37289924898346238</c:v>
+                </c:pt>
+                <c:pt idx="984">
+                  <c:v>0.37302109952530521</c:v>
+                </c:pt>
+                <c:pt idx="985">
+                  <c:v>0.37302109952530521</c:v>
+                </c:pt>
+                <c:pt idx="986">
+                  <c:v>0.37305345217801039</c:v>
+                </c:pt>
+                <c:pt idx="987">
+                  <c:v>0.37317868825305794</c:v>
+                </c:pt>
+                <c:pt idx="988">
+                  <c:v>0.37317868825305794</c:v>
+                </c:pt>
+                <c:pt idx="989">
+                  <c:v>0.37317868825305794</c:v>
+                </c:pt>
+                <c:pt idx="990">
+                  <c:v>0.37434908851668458</c:v>
+                </c:pt>
+                <c:pt idx="991">
+                  <c:v>0.37484043579718662</c:v>
+                </c:pt>
+                <c:pt idx="992">
+                  <c:v>0.37484043579718662</c:v>
+                </c:pt>
+                <c:pt idx="993">
+                  <c:v>0.37523644264560702</c:v>
+                </c:pt>
+                <c:pt idx="994">
+                  <c:v>0.37676298517424595</c:v>
+                </c:pt>
+                <c:pt idx="995">
+                  <c:v>0.37676298517424595</c:v>
+                </c:pt>
+                <c:pt idx="996">
+                  <c:v>0.37676298517424595</c:v>
+                </c:pt>
+                <c:pt idx="997">
+                  <c:v>0.37857789499463801</c:v>
+                </c:pt>
+                <c:pt idx="998">
+                  <c:v>0.37932771689228051</c:v>
+                </c:pt>
+                <c:pt idx="999">
+                  <c:v>0.37932771689228051</c:v>
+                </c:pt>
+                <c:pt idx="1000">
+                  <c:v>0.37965882532150758</c:v>
+                </c:pt>
+                <c:pt idx="1001">
+                  <c:v>0.38091493507687857</c:v>
+                </c:pt>
+                <c:pt idx="1002">
+                  <c:v>0.38091493507687857</c:v>
+                </c:pt>
+                <c:pt idx="1003">
+                  <c:v>0.38091493507687857</c:v>
+                </c:pt>
+                <c:pt idx="1004">
+                  <c:v>0.38237873710118875</c:v>
+                </c:pt>
+                <c:pt idx="1005">
+                  <c:v>0.38298350037885337</c:v>
+                </c:pt>
+                <c:pt idx="1006">
+                  <c:v>0.38298350037885337</c:v>
+                </c:pt>
+                <c:pt idx="1007">
+                  <c:v>0.38383960799508732</c:v>
+                </c:pt>
+                <c:pt idx="1008">
+                  <c:v>0.38707379232313155</c:v>
+                </c:pt>
+                <c:pt idx="1009">
+                  <c:v>0.38707379232313155</c:v>
+                </c:pt>
+                <c:pt idx="1010">
+                  <c:v>0.38707379232313155</c:v>
+                </c:pt>
+                <c:pt idx="1011">
+                  <c:v>0.39219717499274492</c:v>
+                </c:pt>
+                <c:pt idx="1012">
+                  <c:v>0.39428004551731677</c:v>
+                </c:pt>
+                <c:pt idx="1013">
+                  <c:v>0.39428004551731677</c:v>
+                </c:pt>
+                <c:pt idx="1014">
+                  <c:v>0.39617235733110434</c:v>
+                </c:pt>
+                <c:pt idx="1015">
+                  <c:v>0.40332109084987983</c:v>
+                </c:pt>
+                <c:pt idx="1016">
+                  <c:v>0.40332109084987983</c:v>
+                </c:pt>
+                <c:pt idx="1017">
+                  <c:v>0.40332109084987983</c:v>
+                </c:pt>
+                <c:pt idx="1018">
+                  <c:v>0.41104128478695595</c:v>
+                </c:pt>
+                <c:pt idx="1019">
+                  <c:v>0.41417986830343634</c:v>
+                </c:pt>
+                <c:pt idx="1020">
+                  <c:v>0.41417986830343634</c:v>
+                </c:pt>
+                <c:pt idx="1021">
+                  <c:v>0.41802884779487653</c:v>
+                </c:pt>
+                <c:pt idx="1022">
+                  <c:v>0.43228209997416134</c:v>
+                </c:pt>
+                <c:pt idx="1023">
+                  <c:v>0.43228209997416134</c:v>
+                </c:pt>
+                <c:pt idx="1024">
+                  <c:v>0.43228209997416134</c:v>
+                </c:pt>
+                <c:pt idx="1025">
+                  <c:v>0.45032018672990626</c:v>
+                </c:pt>
+                <c:pt idx="1026">
+                  <c:v>0.4576193195101449</c:v>
+                </c:pt>
+                <c:pt idx="1027">
+                  <c:v>0.4576193195101449</c:v>
+                </c:pt>
+                <c:pt idx="1028">
+                  <c:v>0.46403832417223095</c:v>
+                </c:pt>
+                <c:pt idx="1029">
+                  <c:v>0.48780870081155636</c:v>
+                </c:pt>
+                <c:pt idx="1030">
+                  <c:v>0.48780870081155636</c:v>
+                </c:pt>
+                <c:pt idx="1031">
+                  <c:v>0.48780870081155636</c:v>
+                </c:pt>
+                <c:pt idx="1032">
+                  <c:v>0.5121062214138401</c:v>
+                </c:pt>
+                <c:pt idx="1033">
+                  <c:v>0.52182522965476374</c:v>
+                </c:pt>
+                <c:pt idx="1034">
+                  <c:v>0.52182522965476374</c:v>
+                </c:pt>
+                <c:pt idx="1035">
+                  <c:v>0.52934987792288546</c:v>
+                </c:pt>
+                <c:pt idx="1036">
+                  <c:v>0.55678590314665721</c:v>
+                </c:pt>
+                <c:pt idx="1037">
+                  <c:v>0.55678590314665721</c:v>
+                </c:pt>
+                <c:pt idx="1038">
+                  <c:v>0.55678590314665721</c:v>
+                </c:pt>
+                <c:pt idx="1039">
+                  <c:v>0.58180787060957195</c:v>
+                </c:pt>
+                <c:pt idx="1040">
+                  <c:v>0.59177032061797019</c:v>
+                </c:pt>
+                <c:pt idx="1041">
+                  <c:v>0.59177032061797019</c:v>
+                </c:pt>
+                <c:pt idx="1042">
+                  <c:v>0.59915847955724033</c:v>
+                </c:pt>
+                <c:pt idx="1043">
+                  <c:v>0.62598317970602158</c:v>
+                </c:pt>
+                <c:pt idx="1044">
+                  <c:v>0.62598317970602158</c:v>
+                </c:pt>
+                <c:pt idx="1045">
+                  <c:v>0.62598317970602158</c:v>
+                </c:pt>
+                <c:pt idx="1046">
+                  <c:v>0.64926821479665886</c:v>
+                </c:pt>
+                <c:pt idx="1047">
+                  <c:v>0.65843130730917909</c:v>
+                </c:pt>
+                <c:pt idx="1048">
+                  <c:v>0.65843130730917909</c:v>
+                </c:pt>
+                <c:pt idx="1049">
+                  <c:v>0.6650818735634676</c:v>
+                </c:pt>
+                <c:pt idx="1050">
+                  <c:v>0.68886268623032965</c:v>
+                </c:pt>
+                <c:pt idx="1051">
+                  <c:v>0.68886268623032965</c:v>
+                </c:pt>
+                <c:pt idx="1052">
+                  <c:v>0.68886268623032965</c:v>
+                </c:pt>
+                <c:pt idx="1053">
+                  <c:v>0.70942267171227902</c:v>
+                </c:pt>
+                <c:pt idx="1054">
+                  <c:v>0.71751340673990804</c:v>
+                </c:pt>
+                <c:pt idx="1055">
+                  <c:v>0.71751340673990804</c:v>
+                </c:pt>
+                <c:pt idx="1056">
+                  <c:v>0.72340536539855926</c:v>
+                </c:pt>
+                <c:pt idx="1057">
+                  <c:v>0.74438430910742748</c:v>
+                </c:pt>
+                <c:pt idx="1058">
+                  <c:v>0.74438430910742748</c:v>
+                </c:pt>
+                <c:pt idx="1059">
+                  <c:v>0.74438430910742748</c:v>
+                </c:pt>
+                <c:pt idx="1060">
+                  <c:v>0.76223335229626377</c:v>
+                </c:pt>
+                <c:pt idx="1061">
+                  <c:v>0.76914265933710391</c:v>
+                </c:pt>
+                <c:pt idx="1062">
+                  <c:v>0.76914265933710391</c:v>
+                </c:pt>
+                <c:pt idx="1063">
+                  <c:v>0.77421860742652004</c:v>
+                </c:pt>
+                <c:pt idx="1064">
+                  <c:v>0.79229205895705046</c:v>
+                </c:pt>
+                <c:pt idx="1065">
+                  <c:v>0.79229205895705046</c:v>
+                </c:pt>
+                <c:pt idx="1066">
+                  <c:v>0.79229205895705046</c:v>
+                </c:pt>
+                <c:pt idx="1067">
+                  <c:v>0.80771897227674039</c:v>
+                </c:pt>
+                <c:pt idx="1068">
+                  <c:v>0.81369068065856109</c:v>
+                </c:pt>
+                <c:pt idx="1069">
+                  <c:v>0.81369068065856109</c:v>
+                </c:pt>
+                <c:pt idx="1070">
+                  <c:v>0.81807103282661309</c:v>
+                </c:pt>
+                <c:pt idx="1071">
+                  <c:v>0.83336957621954744</c:v>
+                </c:pt>
+                <c:pt idx="1072">
+                  <c:v>0.83336957621954744</c:v>
+                </c:pt>
+                <c:pt idx="1073">
+                  <c:v>0.83336957621954744</c:v>
+                </c:pt>
+                <c:pt idx="1074">
+                  <c:v>0.84645401843090273</c:v>
+                </c:pt>
+                <c:pt idx="1075">
+                  <c:v>0.85149573010867996</c:v>
+                </c:pt>
+                <c:pt idx="1076">
+                  <c:v>0.85149573010867996</c:v>
+                </c:pt>
+                <c:pt idx="1077">
+                  <c:v>0.85515945669264881</c:v>
+                </c:pt>
+                <c:pt idx="1078">
+                  <c:v>0.86795515849338778</c:v>
+                </c:pt>
+                <c:pt idx="1079">
+                  <c:v>0.86795515849338778</c:v>
+                </c:pt>
+                <c:pt idx="1080">
+                  <c:v>0.86795515849338778</c:v>
+                </c:pt>
+                <c:pt idx="1081">
+                  <c:v>0.87876246523073309</c:v>
+                </c:pt>
+                <c:pt idx="1082">
+                  <c:v>0.88287717375917563</c:v>
+                </c:pt>
+                <c:pt idx="1083">
+                  <c:v>0.88287717375917563</c:v>
+                </c:pt>
+                <c:pt idx="1084">
+                  <c:v>0.88593368883836465</c:v>
+                </c:pt>
+                <c:pt idx="1085">
+                  <c:v>0.89640674785974561</c:v>
+                </c:pt>
+                <c:pt idx="1086">
+                  <c:v>0.89640674785974561</c:v>
+                </c:pt>
+                <c:pt idx="1087">
+                  <c:v>0.89640674785974561</c:v>
+                </c:pt>
+                <c:pt idx="1088">
+                  <c:v>0.90531308578918634</c:v>
+                </c:pt>
+                <c:pt idx="1089">
+                  <c:v>0.90868854719624992</c:v>
+                </c:pt>
+                <c:pt idx="1090">
+                  <c:v>0.90868854719624992</c:v>
+                </c:pt>
+                <c:pt idx="1091">
+                  <c:v>0.91115758386530954</c:v>
+                </c:pt>
+                <c:pt idx="1092">
+                  <c:v>0.91961766539312773</c:v>
+                </c:pt>
+                <c:pt idx="1093">
+                  <c:v>0.91961766539312773</c:v>
+                </c:pt>
+                <c:pt idx="1094">
+                  <c:v>0.91961766539312773</c:v>
+                </c:pt>
+                <c:pt idx="1095">
+                  <c:v>0.9268794788181679</c:v>
+                </c:pt>
+                <c:pt idx="1096">
+                  <c:v>0.92959851398189242</c:v>
+                </c:pt>
+                <c:pt idx="1097">
+                  <c:v>0.92959851398189242</c:v>
+                </c:pt>
+                <c:pt idx="1098">
+                  <c:v>0.93165626838102356</c:v>
+                </c:pt>
+                <c:pt idx="1099">
+                  <c:v>0.93860491729407969</c:v>
+                </c:pt>
+                <c:pt idx="1100">
+                  <c:v>0.93860491729407969</c:v>
+                </c:pt>
+                <c:pt idx="1101">
+                  <c:v>0.93860491729407969</c:v>
+                </c:pt>
+                <c:pt idx="1102">
+                  <c:v>0.94451407140467936</c:v>
+                </c:pt>
+                <c:pt idx="1103">
+                  <c:v>0.94672663139130253</c:v>
+                </c:pt>
+                <c:pt idx="1104">
+                  <c:v>0.94672663139130253</c:v>
+                </c:pt>
+                <c:pt idx="1105">
+                  <c:v>0.94830376245043169</c:v>
+                </c:pt>
+                <c:pt idx="1106">
+                  <c:v>0.95360657992461328</c:v>
+                </c:pt>
+                <c:pt idx="1107">
+                  <c:v>0.95360657992461328</c:v>
+                </c:pt>
+                <c:pt idx="1108">
+                  <c:v>0.95360657992461328</c:v>
+                </c:pt>
+                <c:pt idx="1109">
+                  <c:v>0.95846918144446558</c:v>
+                </c:pt>
+                <c:pt idx="1110">
+                  <c:v>0.96025950291314344</c:v>
+                </c:pt>
+                <c:pt idx="1111">
+                  <c:v>0.96025950291314344</c:v>
+                </c:pt>
+                <c:pt idx="1112">
+                  <c:v>0.96154361529429211</c:v>
+                </c:pt>
+                <c:pt idx="1113">
+                  <c:v>0.96586121054686402</c:v>
+                </c:pt>
+                <c:pt idx="1114">
+                  <c:v>0.96586121054686402</c:v>
+                </c:pt>
+                <c:pt idx="1115">
+                  <c:v>0.96586121054686402</c:v>
+                </c:pt>
+                <c:pt idx="1116">
+                  <c:v>0.96954303333680336</c:v>
+                </c:pt>
+                <c:pt idx="1117">
+                  <c:v>0.97089861354583584</c:v>
+                </c:pt>
+                <c:pt idx="1118">
+                  <c:v>0.97089861354583584</c:v>
+                </c:pt>
+                <c:pt idx="1119">
+                  <c:v>0.97198026957345651</c:v>
+                </c:pt>
+                <c:pt idx="1120">
+                  <c:v>0.97554973446460491</c:v>
+                </c:pt>
+                <c:pt idx="1121">
+                  <c:v>0.97554973446460491</c:v>
+                </c:pt>
+                <c:pt idx="1122">
+                  <c:v>0.97554973446460491</c:v>
+                </c:pt>
+                <c:pt idx="1123">
+                  <c:v>0.97833779849208946</c:v>
+                </c:pt>
+                <c:pt idx="1124">
+                  <c:v>0.97934705243869047</c:v>
+                </c:pt>
+                <c:pt idx="1125">
+                  <c:v>0.97934705243869047</c:v>
+                </c:pt>
+                <c:pt idx="1126">
+                  <c:v>0.98018901847890116</c:v>
+                </c:pt>
+                <c:pt idx="1127">
+                  <c:v>0.98296750641164909</c:v>
+                </c:pt>
+                <c:pt idx="1128">
+                  <c:v>0.98296750641164909</c:v>
+                </c:pt>
+                <c:pt idx="1129">
+                  <c:v>0.98296750641164909</c:v>
+                </c:pt>
+                <c:pt idx="1130">
+                  <c:v>0.9852219342458064</c:v>
+                </c:pt>
+                <c:pt idx="1131">
+                  <c:v>0.98603801671971725</c:v>
+                </c:pt>
+                <c:pt idx="1132">
+                  <c:v>0.98603801671971725</c:v>
+                </c:pt>
+                <c:pt idx="1133">
+                  <c:v>0.98666940172857043</c:v>
+                </c:pt>
+                <c:pt idx="1134">
+                  <c:v>0.98871473344739091</c:v>
+                </c:pt>
+                <c:pt idx="1135">
+                  <c:v>0.98871473344739091</c:v>
+                </c:pt>
+                <c:pt idx="1136">
+                  <c:v>0.98871473344739091</c:v>
+                </c:pt>
+                <c:pt idx="1137">
+                  <c:v>0.99039274028247459</c:v>
+                </c:pt>
+                <c:pt idx="1138">
+                  <c:v>0.99099742743025698</c:v>
+                </c:pt>
+                <c:pt idx="1139">
+                  <c:v>0.99099742743025698</c:v>
+                </c:pt>
+                <c:pt idx="1140">
+                  <c:v>0.99147526208909587</c:v>
+                </c:pt>
+                <c:pt idx="1141">
+                  <c:v>0.99302317718113842</c:v>
+                </c:pt>
+                <c:pt idx="1142">
+                  <c:v>0.99302317718113842</c:v>
+                </c:pt>
+                <c:pt idx="1143">
+                  <c:v>0.99302317718113842</c:v>
+                </c:pt>
+                <c:pt idx="1144">
+                  <c:v>0.99422691591807366</c:v>
+                </c:pt>
+                <c:pt idx="1145">
+                  <c:v>0.99465527339654336</c:v>
+                </c:pt>
+                <c:pt idx="1146">
+                  <c:v>0.99465527339654336</c:v>
+                </c:pt>
+                <c:pt idx="1147">
+                  <c:v>0.9949242334994205</c:v>
+                </c:pt>
+                <c:pt idx="1148">
+                  <c:v>0.9957834116058597</c:v>
+                </c:pt>
+                <c:pt idx="1149">
+                  <c:v>0.9957834116058597</c:v>
+                </c:pt>
+                <c:pt idx="1150">
+                  <c:v>0.9957834116058597</c:v>
+                </c:pt>
+                <c:pt idx="1151">
+                  <c:v>0.996862011092844</c:v>
+                </c:pt>
+                <c:pt idx="1152">
+                  <c:v>0.99724583703642389</c:v>
+                </c:pt>
+                <c:pt idx="1153">
+                  <c:v>0.99724583703642389</c:v>
+                </c:pt>
+                <c:pt idx="1154">
+                  <c:v>0.99741491926039205</c:v>
+                </c:pt>
+                <c:pt idx="1155">
+                  <c:v>0.99795269466718584</c:v>
+                </c:pt>
+                <c:pt idx="1156">
+                  <c:v>0.99795269466718584</c:v>
+                </c:pt>
+                <c:pt idx="1157">
+                  <c:v>0.99795269466718584</c:v>
+                </c:pt>
+                <c:pt idx="1158">
+                  <c:v>0.99876708031776207</c:v>
+                </c:pt>
+                <c:pt idx="1159">
+                  <c:v>0.99905193269779791</c:v>
+                </c:pt>
+                <c:pt idx="1160">
+                  <c:v>0.99905193269779791</c:v>
+                </c:pt>
+                <c:pt idx="1161">
+                  <c:v>0.99914786807755174</c:v>
+                </c:pt>
+                <c:pt idx="1162">
+                  <c:v>0.99945299588261538</c:v>
+                </c:pt>
+                <c:pt idx="1163">
+                  <c:v>0.99945299588261538</c:v>
+                </c:pt>
+                <c:pt idx="1164">
+                  <c:v>0.99945299588261538</c:v>
+                </c:pt>
+                <c:pt idx="1165">
+                  <c:v>0.9998433663777534</c:v>
+                </c:pt>
+                <c:pt idx="1166">
+                  <c:v>0.99997990852403673</c:v>
+                </c:pt>
+                <c:pt idx="1167">
+                  <c:v>0.99997990852403673</c:v>
+                </c:pt>
+                <c:pt idx="1168">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1169">
+                  <c:v>1.0000627514592029</c:v>
+                </c:pt>
+                <c:pt idx="1170">
+                  <c:v>1.0000627514592029</c:v>
+                </c:pt>
+                <c:pt idx="1171">
+                  <c:v>1.0000627514592029</c:v>
+                </c:pt>
+                <c:pt idx="1172">
+                  <c:v>1.0002397256013549</c:v>
+                </c:pt>
+                <c:pt idx="1173">
+                  <c:v>1.0003005604627331</c:v>
+                </c:pt>
+                <c:pt idx="1174">
+                  <c:v>1.0003005604627331</c:v>
+                </c:pt>
+                <c:pt idx="1175">
+                  <c:v>1.0002716598610553</c:v>
+                </c:pt>
+                <c:pt idx="1176">
+                  <c:v>1.0001813949681648</c:v>
+                </c:pt>
+                <c:pt idx="1177">
+                  <c:v>1.0001813949681648</c:v>
+                </c:pt>
+                <c:pt idx="1178">
+                  <c:v>1.0001813949681648</c:v>
+                </c:pt>
+                <c:pt idx="1179">
+                  <c:v>1.0000320484612266</c:v>
+                </c:pt>
+                <c:pt idx="1180">
+                  <c:v>0.99998071059948068</c:v>
+                </c:pt>
+                <c:pt idx="1181">
+                  <c:v>0.99998071059948068</c:v>
+                </c:pt>
+                <c:pt idx="1182">
+                  <c:v>0.99991814566945358</c:v>
+                </c:pt>
+                <c:pt idx="1183">
+                  <c:v>0.99972622351925367</c:v>
+                </c:pt>
+                <c:pt idx="1184">
+                  <c:v>0.99972622351925367</c:v>
+                </c:pt>
+                <c:pt idx="1185">
+                  <c:v>0.99972622351925367</c:v>
+                </c:pt>
+                <c:pt idx="1186">
+                  <c:v>0.99951444562848624</c:v>
+                </c:pt>
+                <c:pt idx="1187">
+                  <c:v>0.99944197052809658</c:v>
+                </c:pt>
+                <c:pt idx="1188">
+                  <c:v>0.99944197052809658</c:v>
+                </c:pt>
+                <c:pt idx="1189">
+                  <c:v>0.99926456394278018</c:v>
+                </c:pt>
+                <c:pt idx="1190">
+                  <c:v>0.9987203572554324</c:v>
+                </c:pt>
+                <c:pt idx="1191">
+                  <c:v>0.9987203572554324</c:v>
+                </c:pt>
+                <c:pt idx="1192">
+                  <c:v>0.9987203572554324</c:v>
+                </c:pt>
+                <c:pt idx="1193">
+                  <c:v>0.99852224614339558</c:v>
+                </c:pt>
+                <c:pt idx="1194">
+                  <c:v>0.99845532861222419</c:v>
+                </c:pt>
+                <c:pt idx="1195">
+                  <c:v>0.99845532861222419</c:v>
+                </c:pt>
+                <c:pt idx="1196">
+                  <c:v>0.99828325295006481</c:v>
+                </c:pt>
+                <c:pt idx="1197">
+                  <c:v>0.99776243727927638</c:v>
+                </c:pt>
+                <c:pt idx="1198">
+                  <c:v>0.99776243727927638</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F2BF-DA42-ADBE-98237B3B3D2B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1416058208"/>
+        <c:axId val="1416059920"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1416058208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1200"/>
+          <c:min val="200"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1416059920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1416059920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1.01"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1416058208"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -11969,6 +15817,46 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -13040,6 +16928,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -13109,6 +17513,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>730250</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5FAAC39-A01A-A76E-E06E-91497FF6B43F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>

<commit_message>
inclusion of translation and scaling augmentation with ResNet 18 framework
</commit_message>
<xml_diff>
--- a/Code/Boiling-91_Temperature_10Hz.xlsx
+++ b/Code/Boiling-91_Temperature_10Hz.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ytrivedi/Desktop/School Stuff/Oklahoma State/Spring 2026/Deep Learning/Final-Project-Yash-Trivedi/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71204AE-2791-0E40-B6AA-8C1540C32522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC8F22F-9BF5-2D4B-92F4-09A136FC125C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17320" xr2:uid="{130CFDE4-EB42-3F45-93C7-0A9FCD22FCB8}"/>
+    <workbookView xWindow="-20" yWindow="760" windowWidth="30240" windowHeight="17320" xr2:uid="{130CFDE4-EB42-3F45-93C7-0A9FCD22FCB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Boiling-91_Temperature_10Hz" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Boiling-91_Temperature_10Hz'!$J$1</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Boiling-91_Temperature_10Hz'!$J$2:$J$1200</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Boiling-91_Temperature_10Hz'!$J$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Boiling-91_Temperature_10Hz'!$J$2:$J$1200</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'Boiling-91_Temperature_10Hz'!$D$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Boiling-91_Temperature_10Hz'!$D$2:$D$1200</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Boiling-91_Temperature_10Hz'!$D$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Boiling-91_Temperature_10Hz'!$D$2:$D$1200</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -11788,7 +11788,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -11948,7 +11948,37 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -15776,6 +15806,3861 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Boiling-91_Temperature_10Hz'!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Temperature_1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>'Boiling-91_Temperature_10Hz'!$D$2:$D$1200</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1199"/>
+                <c:pt idx="0">
+                  <c:v>95.269064999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>95.269064999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>95.269064999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>95.268955637873702</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>95.268846999999994</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>95.268846999999994</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>95.268950956810599</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>95.300138000000004</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>95.300138000000004</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>95.300138000000004</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>95.284537548172693</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>95.269244999999998</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>95.269244999999998</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>95.269267767441804</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>95.276098000000005</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>95.276098000000005</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>95.276098000000005</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>95.275265282391999</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>95.274449000000004</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>95.274449000000004</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>95.274461797342198</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>95.276375000000002</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>95.276375000000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>95.276375000000002</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>95.275838486754907</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>95.275316000000004</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>95.275316000000004</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>95.275207428571406</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>95.258976000000004</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>95.258976000000004</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>95.258976000000004</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>95.2639538372093</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>95.268769000000006</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>95.268769000000006</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>95.268711135761507</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>95.262944000000005</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>95.262944000000005</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>95.262944000000005</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>95.273124853820505</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>95.282972999999998</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>95.282972999999998</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>95.282841219269102</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>95.269750999999999</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>95.269750999999999</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>95.269750999999999</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>95.265373511627899</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>95.261195000000001</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>95.261195000000001</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>95.2613516357615</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>95.273021</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>95.273021</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>95.273021</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>95.267517930232501</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>95.262264999999999</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>95.262264999999999</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>95.2623230332226</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>95.266632000000001</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>95.266632000000001</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>95.266632000000001</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>95.256671833886998</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>95.247290000000007</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>95.247290000000007</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>95.247579023255796</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>95.269039000000006</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>95.269039000000006</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>95.269039000000006</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>95.272335196013302</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>95.275440000000003</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>95.275440000000003</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>95.275463438538196</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>95.276850999999994</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>95.276850999999994</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>95.276850999999994</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>95.261434377483397</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>95.247005999999999</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>95.247005999999999</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>95.247146398671006</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>95.255458000000004</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>95.255458000000004</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>95.255458000000004</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>95.254803940199295</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>95.254195999999993</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>95.254195999999993</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>95.2543289536423</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>95.260887999999994</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>95.260887999999994</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>95.260887999999994</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>95.253072831125806</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>95.245855000000006</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>95.245855000000006</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>95.246058401993295</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>95.256058999999993</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>95.256058999999993</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>95.256058999999993</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>95.2617798504983</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>95.267026999999999</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>95.267026999999999</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>95.266932407284699</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>95.262945999999999</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>95.262945999999999</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>95.262945999999999</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>95.262469262458396</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>95.262032000000005</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>95.262032000000005</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>95.262063372092996</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>95.263380999999995</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>95.263380999999995</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>95.263380999999995</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>95.261370043189302</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>95.259550000000004</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>95.259550000000004</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>95.259500069767398</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>95.257402999999996</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>95.257402999999996</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>95.257402999999996</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>95.251595843853806</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>95.246340000000004</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>95.246340000000004</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>95.246319561461803</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>95.245570999999998</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>95.245570999999998</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>95.245570999999998</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>95.248499864238397</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>95.251133999999993</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>95.251133999999993</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>95.250465136212597</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>95.225967999999995</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>95.225967999999995</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>95.225967999999995</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>95.242138986710899</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>95.256580999999997</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>95.256580999999997</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>95.256721501661104</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>95.261279999999999</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>95.261279999999999</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>95.261279999999999</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>95.2749928476821</c:v>
+                </c:pt>
+                <c:pt idx="137">
+                  <c:v>95.287163000000007</c:v>
+                </c:pt>
+                <c:pt idx="138">
+                  <c:v>95.287163000000007</c:v>
+                </c:pt>
+                <c:pt idx="139">
+                  <c:v>95.288905352159404</c:v>
+                </c:pt>
+                <c:pt idx="140">
+                  <c:v>95.345434999999995</c:v>
+                </c:pt>
+                <c:pt idx="141">
+                  <c:v>95.345434999999995</c:v>
+                </c:pt>
+                <c:pt idx="142">
+                  <c:v>95.345434999999995</c:v>
+                </c:pt>
+                <c:pt idx="143">
+                  <c:v>95.374939850498293</c:v>
+                </c:pt>
+                <c:pt idx="144">
+                  <c:v>95.400941000000003</c:v>
+                </c:pt>
+                <c:pt idx="145">
+                  <c:v>95.400941000000003</c:v>
+                </c:pt>
+                <c:pt idx="146">
+                  <c:v>95.404451364238398</c:v>
+                </c:pt>
+                <c:pt idx="147">
+                  <c:v>95.506953999999993</c:v>
+                </c:pt>
+                <c:pt idx="148">
+                  <c:v>95.506953999999993</c:v>
+                </c:pt>
+                <c:pt idx="149">
+                  <c:v>95.506953999999993</c:v>
+                </c:pt>
+                <c:pt idx="150">
+                  <c:v>95.570720112956806</c:v>
+                </c:pt>
+                <c:pt idx="151">
+                  <c:v>95.626913999999999</c:v>
+                </c:pt>
+                <c:pt idx="152">
+                  <c:v>95.626913999999999</c:v>
+                </c:pt>
+                <c:pt idx="153">
+                  <c:v>95.631871574750804</c:v>
+                </c:pt>
+                <c:pt idx="154">
+                  <c:v>95.776137000000006</c:v>
+                </c:pt>
+                <c:pt idx="155">
+                  <c:v>95.776137000000006</c:v>
+                </c:pt>
+                <c:pt idx="156">
+                  <c:v>95.776137000000006</c:v>
+                </c:pt>
+                <c:pt idx="157">
+                  <c:v>95.866931906976703</c:v>
+                </c:pt>
+                <c:pt idx="158">
+                  <c:v>95.945884000000007</c:v>
+                </c:pt>
+                <c:pt idx="159">
+                  <c:v>95.945884000000007</c:v>
+                </c:pt>
+                <c:pt idx="160">
+                  <c:v>95.952402803986701</c:v>
+                </c:pt>
+                <c:pt idx="161">
+                  <c:v>96.142099999999999</c:v>
+                </c:pt>
+                <c:pt idx="162">
+                  <c:v>96.142099999999999</c:v>
+                </c:pt>
+                <c:pt idx="163">
+                  <c:v>96.142099999999999</c:v>
+                </c:pt>
+                <c:pt idx="164">
+                  <c:v>96.274133372093004</c:v>
+                </c:pt>
+                <c:pt idx="165">
+                  <c:v>96.388945000000007</c:v>
+                </c:pt>
+                <c:pt idx="166">
+                  <c:v>96.388945000000007</c:v>
+                </c:pt>
+                <c:pt idx="167">
+                  <c:v>96.398346674418605</c:v>
+                </c:pt>
+                <c:pt idx="168">
+                  <c:v>96.646208999999999</c:v>
+                </c:pt>
+                <c:pt idx="169">
+                  <c:v>96.646208999999999</c:v>
+                </c:pt>
+                <c:pt idx="170">
+                  <c:v>96.646208999999999</c:v>
+                </c:pt>
+                <c:pt idx="171">
+                  <c:v>96.792247963455097</c:v>
+                </c:pt>
+                <c:pt idx="172">
+                  <c:v>96.917552999999998</c:v>
+                </c:pt>
+                <c:pt idx="173">
+                  <c:v>96.917552999999998</c:v>
+                </c:pt>
+                <c:pt idx="174">
+                  <c:v>96.929703870431894</c:v>
+                </c:pt>
+                <c:pt idx="175">
+                  <c:v>97.250045</c:v>
+                </c:pt>
+                <c:pt idx="176">
+                  <c:v>97.250045</c:v>
+                </c:pt>
+                <c:pt idx="177">
+                  <c:v>97.250045</c:v>
+                </c:pt>
+                <c:pt idx="178">
+                  <c:v>97.410222634551403</c:v>
+                </c:pt>
+                <c:pt idx="179">
+                  <c:v>97.547658999999996</c:v>
+                </c:pt>
+                <c:pt idx="180">
+                  <c:v>97.547658999999996</c:v>
+                </c:pt>
+                <c:pt idx="181">
+                  <c:v>97.561701671096301</c:v>
+                </c:pt>
+                <c:pt idx="182">
+                  <c:v>97.899895999999998</c:v>
+                </c:pt>
+                <c:pt idx="183">
+                  <c:v>97.899895999999998</c:v>
+                </c:pt>
+                <c:pt idx="184">
+                  <c:v>97.899895999999998</c:v>
+                </c:pt>
+                <c:pt idx="185">
+                  <c:v>98.096780029801295</c:v>
+                </c:pt>
+                <c:pt idx="186">
+                  <c:v>98.264674999999997</c:v>
+                </c:pt>
+                <c:pt idx="187">
+                  <c:v>98.264674999999997</c:v>
+                </c:pt>
+                <c:pt idx="188">
+                  <c:v>98.279919106312207</c:v>
+                </c:pt>
+                <c:pt idx="189">
+                  <c:v>98.647047999999998</c:v>
+                </c:pt>
+                <c:pt idx="190">
+                  <c:v>98.647047999999998</c:v>
+                </c:pt>
+                <c:pt idx="191">
+                  <c:v>98.647047999999998</c:v>
+                </c:pt>
+                <c:pt idx="192">
+                  <c:v>98.859121830564703</c:v>
+                </c:pt>
+                <c:pt idx="193">
+                  <c:v>99.038668999999999</c:v>
+                </c:pt>
+                <c:pt idx="194">
+                  <c:v>99.038668999999999</c:v>
+                </c:pt>
+                <c:pt idx="195">
+                  <c:v>99.056938304635693</c:v>
+                </c:pt>
+                <c:pt idx="196">
+                  <c:v>99.463078999999993</c:v>
+                </c:pt>
+                <c:pt idx="197">
+                  <c:v>99.463078999999993</c:v>
+                </c:pt>
+                <c:pt idx="198">
+                  <c:v>99.463078999999993</c:v>
+                </c:pt>
+                <c:pt idx="199">
+                  <c:v>99.690984408637803</c:v>
+                </c:pt>
+                <c:pt idx="200">
+                  <c:v>99.883934999999994</c:v>
+                </c:pt>
+                <c:pt idx="201">
+                  <c:v>99.883934999999994</c:v>
+                </c:pt>
+                <c:pt idx="202">
+                  <c:v>99.902394697674396</c:v>
+                </c:pt>
+                <c:pt idx="203">
+                  <c:v>100.311348</c:v>
+                </c:pt>
+                <c:pt idx="204">
+                  <c:v>100.311348</c:v>
+                </c:pt>
+                <c:pt idx="205">
+                  <c:v>100.311348</c:v>
+                </c:pt>
+                <c:pt idx="206">
+                  <c:v>100.567950790697</c:v>
+                </c:pt>
+                <c:pt idx="207">
+                  <c:v>100.782308</c:v>
+                </c:pt>
+                <c:pt idx="208">
+                  <c:v>100.782308</c:v>
+                </c:pt>
+                <c:pt idx="209">
+                  <c:v>100.802618476821</c:v>
+                </c:pt>
+                <c:pt idx="210">
+                  <c:v>101.220434</c:v>
+                </c:pt>
+                <c:pt idx="211">
+                  <c:v>101.220434</c:v>
+                </c:pt>
+                <c:pt idx="212">
+                  <c:v>101.220434</c:v>
+                </c:pt>
+                <c:pt idx="213">
+                  <c:v>101.482092458471</c:v>
+                </c:pt>
+                <c:pt idx="214">
+                  <c:v>101.70067299999999</c:v>
+                </c:pt>
+                <c:pt idx="215">
+                  <c:v>101.70067299999999</c:v>
+                </c:pt>
+                <c:pt idx="216">
+                  <c:v>101.722394674418</c:v>
+                </c:pt>
+                <c:pt idx="217">
+                  <c:v>102.167689</c:v>
+                </c:pt>
+                <c:pt idx="218">
+                  <c:v>102.167689</c:v>
+                </c:pt>
+                <c:pt idx="219">
+                  <c:v>102.167689</c:v>
+                </c:pt>
+                <c:pt idx="220">
+                  <c:v>102.44643265448499</c:v>
+                </c:pt>
+                <c:pt idx="221">
+                  <c:v>102.676185</c:v>
+                </c:pt>
+                <c:pt idx="222">
+                  <c:v>102.676185</c:v>
+                </c:pt>
+                <c:pt idx="223">
+                  <c:v>102.698460906976</c:v>
+                </c:pt>
+                <c:pt idx="224">
+                  <c:v>103.155117</c:v>
+                </c:pt>
+                <c:pt idx="225">
+                  <c:v>103.155117</c:v>
+                </c:pt>
+                <c:pt idx="226">
+                  <c:v>103.155117</c:v>
+                </c:pt>
+                <c:pt idx="227">
+                  <c:v>103.423438245847</c:v>
+                </c:pt>
+                <c:pt idx="228">
+                  <c:v>103.6446</c:v>
+                </c:pt>
+                <c:pt idx="229">
+                  <c:v>103.6446</c:v>
+                </c:pt>
+                <c:pt idx="230">
+                  <c:v>103.670936561461</c:v>
+                </c:pt>
+                <c:pt idx="231">
+                  <c:v>104.173087</c:v>
+                </c:pt>
+                <c:pt idx="232">
+                  <c:v>104.173087</c:v>
+                </c:pt>
+                <c:pt idx="233">
+                  <c:v>104.173087</c:v>
+                </c:pt>
+                <c:pt idx="234">
+                  <c:v>104.453362609271</c:v>
+                </c:pt>
+                <c:pt idx="235">
+                  <c:v>104.682986</c:v>
+                </c:pt>
+                <c:pt idx="236">
+                  <c:v>104.682986</c:v>
+                </c:pt>
+                <c:pt idx="237">
+                  <c:v>104.708165518272</c:v>
+                </c:pt>
+                <c:pt idx="238">
+                  <c:v>105.188255</c:v>
+                </c:pt>
+                <c:pt idx="239">
+                  <c:v>105.188255</c:v>
+                </c:pt>
+                <c:pt idx="240">
+                  <c:v>105.188255</c:v>
+                </c:pt>
+                <c:pt idx="241">
+                  <c:v>105.46897864784</c:v>
+                </c:pt>
+                <c:pt idx="242">
+                  <c:v>105.697278</c:v>
+                </c:pt>
+                <c:pt idx="243">
+                  <c:v>105.697278</c:v>
+                </c:pt>
+                <c:pt idx="244">
+                  <c:v>105.723969337748</c:v>
+                </c:pt>
+                <c:pt idx="245">
+                  <c:v>106.201077</c:v>
+                </c:pt>
+                <c:pt idx="246">
+                  <c:v>106.201077</c:v>
+                </c:pt>
+                <c:pt idx="247">
+                  <c:v>106.201077</c:v>
+                </c:pt>
+                <c:pt idx="248">
+                  <c:v>106.48572407615799</c:v>
+                </c:pt>
+                <c:pt idx="249">
+                  <c:v>106.715828</c:v>
+                </c:pt>
+                <c:pt idx="250">
+                  <c:v>106.715828</c:v>
+                </c:pt>
+                <c:pt idx="251">
+                  <c:v>106.742021913621</c:v>
+                </c:pt>
+                <c:pt idx="252">
+                  <c:v>107.208601</c:v>
+                </c:pt>
+                <c:pt idx="253">
+                  <c:v>107.208601</c:v>
+                </c:pt>
+                <c:pt idx="254">
+                  <c:v>107.208601</c:v>
+                </c:pt>
+                <c:pt idx="255">
+                  <c:v>107.473798109634</c:v>
+                </c:pt>
+                <c:pt idx="256">
+                  <c:v>107.68659100000001</c:v>
+                </c:pt>
+                <c:pt idx="257">
+                  <c:v>107.68659100000001</c:v>
+                </c:pt>
+                <c:pt idx="258">
+                  <c:v>107.713811715231</c:v>
+                </c:pt>
+                <c:pt idx="259">
+                  <c:v>108.170159</c:v>
+                </c:pt>
+                <c:pt idx="260">
+                  <c:v>108.170159</c:v>
+                </c:pt>
+                <c:pt idx="261">
+                  <c:v>108.170159</c:v>
+                </c:pt>
+                <c:pt idx="262">
+                  <c:v>108.433539637873</c:v>
+                </c:pt>
+                <c:pt idx="263">
+                  <c:v>108.644875</c:v>
+                </c:pt>
+                <c:pt idx="264">
+                  <c:v>108.644875</c:v>
+                </c:pt>
+                <c:pt idx="265">
+                  <c:v>108.669669245847</c:v>
+                </c:pt>
+                <c:pt idx="266">
+                  <c:v>109.083878999999</c:v>
+                </c:pt>
+                <c:pt idx="267">
+                  <c:v>109.083878999999</c:v>
+                </c:pt>
+                <c:pt idx="268">
+                  <c:v>109.083879</c:v>
+                </c:pt>
+                <c:pt idx="269">
+                  <c:v>109.340215744186</c:v>
+                </c:pt>
+                <c:pt idx="270">
+                  <c:v>109.543148999999</c:v>
+                </c:pt>
+                <c:pt idx="271">
+                  <c:v>109.543148999999</c:v>
+                </c:pt>
+                <c:pt idx="272">
+                  <c:v>109.568458554817</c:v>
+                </c:pt>
+                <c:pt idx="273">
+                  <c:v>109.991277</c:v>
+                </c:pt>
+                <c:pt idx="274">
+                  <c:v>109.991277</c:v>
+                </c:pt>
+                <c:pt idx="275">
+                  <c:v>109.991277</c:v>
+                </c:pt>
+                <c:pt idx="276">
+                  <c:v>110.24574174418601</c:v>
+                </c:pt>
+                <c:pt idx="277">
+                  <c:v>110.447193</c:v>
+                </c:pt>
+                <c:pt idx="278">
+                  <c:v>110.447193</c:v>
+                </c:pt>
+                <c:pt idx="279">
+                  <c:v>110.47321011627901</c:v>
+                </c:pt>
+                <c:pt idx="280">
+                  <c:v>110.882257</c:v>
+                </c:pt>
+                <c:pt idx="281">
+                  <c:v>110.882257</c:v>
+                </c:pt>
+                <c:pt idx="282">
+                  <c:v>110.882257</c:v>
+                </c:pt>
+                <c:pt idx="283">
+                  <c:v>111.105046006622</c:v>
+                </c:pt>
+                <c:pt idx="284">
+                  <c:v>111.28037699999901</c:v>
+                </c:pt>
+                <c:pt idx="285">
+                  <c:v>111.28037699999901</c:v>
+                </c:pt>
+                <c:pt idx="286">
+                  <c:v>111.302125604651</c:v>
+                </c:pt>
+                <c:pt idx="287">
+                  <c:v>111.64406200000001</c:v>
+                </c:pt>
+                <c:pt idx="288">
+                  <c:v>111.644061999999</c:v>
+                </c:pt>
+                <c:pt idx="289">
+                  <c:v>111.64406200000001</c:v>
+                </c:pt>
+                <c:pt idx="290">
+                  <c:v>111.841075013289</c:v>
+                </c:pt>
+                <c:pt idx="291">
+                  <c:v>111.994955</c:v>
+                </c:pt>
+                <c:pt idx="292">
+                  <c:v>111.994955</c:v>
+                </c:pt>
+                <c:pt idx="293">
+                  <c:v>112.01650920598</c:v>
+                </c:pt>
+                <c:pt idx="294">
+                  <c:v>112.336418999999</c:v>
+                </c:pt>
+                <c:pt idx="295">
+                  <c:v>112.336418999999</c:v>
+                </c:pt>
+                <c:pt idx="296">
+                  <c:v>112.336418999999</c:v>
+                </c:pt>
+                <c:pt idx="297">
+                  <c:v>112.518255390728</c:v>
+                </c:pt>
+                <c:pt idx="298">
+                  <c:v>112.65944599999899</c:v>
+                </c:pt>
+                <c:pt idx="299">
+                  <c:v>112.65944599999899</c:v>
+                </c:pt>
+                <c:pt idx="300">
+                  <c:v>112.679988093023</c:v>
+                </c:pt>
+                <c:pt idx="301">
+                  <c:v>112.984876</c:v>
+                </c:pt>
+                <c:pt idx="302">
+                  <c:v>112.984876</c:v>
+                </c:pt>
+                <c:pt idx="303">
+                  <c:v>112.984876</c:v>
+                </c:pt>
+                <c:pt idx="304">
+                  <c:v>113.152827528239</c:v>
+                </c:pt>
+                <c:pt idx="305">
+                  <c:v>113.28224899999999</c:v>
+                </c:pt>
+                <c:pt idx="306">
+                  <c:v>113.28224899999999</c:v>
+                </c:pt>
+                <c:pt idx="307">
+                  <c:v>113.302063569536</c:v>
+                </c:pt>
+                <c:pt idx="308">
+                  <c:v>113.58144900000001</c:v>
+                </c:pt>
+                <c:pt idx="309">
+                  <c:v>113.58144900000001</c:v>
+                </c:pt>
+                <c:pt idx="310">
+                  <c:v>113.58144900000001</c:v>
+                </c:pt>
+                <c:pt idx="311">
+                  <c:v>113.75994504651101</c:v>
+                </c:pt>
+                <c:pt idx="312">
+                  <c:v>113.897492</c:v>
+                </c:pt>
+                <c:pt idx="313">
+                  <c:v>113.897492</c:v>
+                </c:pt>
+                <c:pt idx="314">
+                  <c:v>113.915371667774</c:v>
+                </c:pt>
+                <c:pt idx="315">
+                  <c:v>114.16658099999999</c:v>
+                </c:pt>
+                <c:pt idx="316">
+                  <c:v>114.16658099999999</c:v>
+                </c:pt>
+                <c:pt idx="317">
+                  <c:v>114.16658099999999</c:v>
+                </c:pt>
+                <c:pt idx="318">
+                  <c:v>114.315139664451</c:v>
+                </c:pt>
+                <c:pt idx="319">
+                  <c:v>114.428079</c:v>
+                </c:pt>
+                <c:pt idx="320">
+                  <c:v>114.428079</c:v>
+                </c:pt>
+                <c:pt idx="321">
+                  <c:v>114.44569946511599</c:v>
+                </c:pt>
+                <c:pt idx="322">
+                  <c:v>114.693266999999</c:v>
+                </c:pt>
+                <c:pt idx="323">
+                  <c:v>114.69326700000001</c:v>
+                </c:pt>
+                <c:pt idx="324">
+                  <c:v>114.69326700000001</c:v>
+                </c:pt>
+                <c:pt idx="325">
+                  <c:v>114.842449445182</c:v>
+                </c:pt>
+                <c:pt idx="326">
+                  <c:v>114.95586299999999</c:v>
+                </c:pt>
+                <c:pt idx="327">
+                  <c:v>114.95586299999999</c:v>
+                </c:pt>
+                <c:pt idx="328">
+                  <c:v>114.974112488372</c:v>
+                </c:pt>
+                <c:pt idx="329">
+                  <c:v>115.217438999999</c:v>
+                </c:pt>
+                <c:pt idx="330">
+                  <c:v>115.217438999999</c:v>
+                </c:pt>
+                <c:pt idx="331">
+                  <c:v>115.217438999999</c:v>
+                </c:pt>
+                <c:pt idx="332">
+                  <c:v>115.361841543046</c:v>
+                </c:pt>
+                <c:pt idx="333">
+                  <c:v>115.470983</c:v>
+                </c:pt>
+                <c:pt idx="334">
+                  <c:v>115.470983</c:v>
+                </c:pt>
+                <c:pt idx="335">
+                  <c:v>115.48783211627899</c:v>
+                </c:pt>
+                <c:pt idx="336">
+                  <c:v>115.712487</c:v>
+                </c:pt>
+                <c:pt idx="337">
+                  <c:v>115.712487</c:v>
+                </c:pt>
+                <c:pt idx="338">
+                  <c:v>115.712487</c:v>
+                </c:pt>
+                <c:pt idx="339">
+                  <c:v>115.859539</c:v>
+                </c:pt>
+                <c:pt idx="340">
+                  <c:v>115.96982800000001</c:v>
+                </c:pt>
+                <c:pt idx="341">
+                  <c:v>115.96982800000001</c:v>
+                </c:pt>
+                <c:pt idx="342">
+                  <c:v>115.98649786046499</c:v>
+                </c:pt>
+                <c:pt idx="343">
+                  <c:v>116.197902</c:v>
+                </c:pt>
+                <c:pt idx="344">
+                  <c:v>116.197902</c:v>
+                </c:pt>
+                <c:pt idx="345">
+                  <c:v>116.197902</c:v>
+                </c:pt>
+                <c:pt idx="346">
+                  <c:v>116.359664447019</c:v>
+                </c:pt>
+                <c:pt idx="347">
+                  <c:v>116.48028499999999</c:v>
+                </c:pt>
+                <c:pt idx="348">
+                  <c:v>116.48028499999999</c:v>
+                </c:pt>
+                <c:pt idx="349">
+                  <c:v>116.497496455149</c:v>
+                </c:pt>
+                <c:pt idx="350">
+                  <c:v>116.715768999999</c:v>
+                </c:pt>
+                <c:pt idx="351">
+                  <c:v>116.71576899999999</c:v>
+                </c:pt>
+                <c:pt idx="352">
+                  <c:v>116.715768999999</c:v>
+                </c:pt>
+                <c:pt idx="353">
+                  <c:v>116.86620313289001</c:v>
+                </c:pt>
+                <c:pt idx="354">
+                  <c:v>116.977507</c:v>
+                </c:pt>
+                <c:pt idx="355">
+                  <c:v>116.977507</c:v>
+                </c:pt>
+                <c:pt idx="356">
+                  <c:v>116.996668894039</c:v>
+                </c:pt>
+                <c:pt idx="357">
+                  <c:v>117.229111</c:v>
+                </c:pt>
+                <c:pt idx="358">
+                  <c:v>117.229111</c:v>
+                </c:pt>
+                <c:pt idx="359">
+                  <c:v>117.229111</c:v>
+                </c:pt>
+                <c:pt idx="360">
+                  <c:v>117.37213774418601</c:v>
+                </c:pt>
+                <c:pt idx="361">
+                  <c:v>117.47796099999999</c:v>
+                </c:pt>
+                <c:pt idx="362">
+                  <c:v>117.477960999999</c:v>
+                </c:pt>
+                <c:pt idx="363">
+                  <c:v>117.49669155813901</c:v>
+                </c:pt>
+                <c:pt idx="364">
+                  <c:v>117.72308700000001</c:v>
+                </c:pt>
+                <c:pt idx="365">
+                  <c:v>117.72308700000001</c:v>
+                </c:pt>
+                <c:pt idx="366">
+                  <c:v>117.72308700000001</c:v>
+                </c:pt>
+                <c:pt idx="367">
+                  <c:v>117.87084305979999</c:v>
+                </c:pt>
+                <c:pt idx="368">
+                  <c:v>117.97868800000001</c:v>
+                </c:pt>
+                <c:pt idx="369">
+                  <c:v>117.97868800000001</c:v>
+                </c:pt>
+                <c:pt idx="370">
+                  <c:v>117.994816730897</c:v>
+                </c:pt>
+                <c:pt idx="371">
+                  <c:v>118.189763999999</c:v>
+                </c:pt>
+                <c:pt idx="372">
+                  <c:v>118.189764</c:v>
+                </c:pt>
+                <c:pt idx="373">
+                  <c:v>118.189764</c:v>
+                </c:pt>
+                <c:pt idx="374">
+                  <c:v>118.33533320930199</c:v>
+                </c:pt>
+                <c:pt idx="375">
+                  <c:v>118.441582</c:v>
+                </c:pt>
+                <c:pt idx="376">
+                  <c:v>118.441582</c:v>
+                </c:pt>
+                <c:pt idx="377">
+                  <c:v>118.46130689036499</c:v>
+                </c:pt>
+                <c:pt idx="378">
+                  <c:v>118.688965</c:v>
+                </c:pt>
+                <c:pt idx="379">
+                  <c:v>118.688965</c:v>
+                </c:pt>
+                <c:pt idx="380">
+                  <c:v>118.688964999999</c:v>
+                </c:pt>
+                <c:pt idx="381">
+                  <c:v>118.82245046511601</c:v>
+                </c:pt>
+                <c:pt idx="382">
+                  <c:v>118.918559999999</c:v>
+                </c:pt>
+                <c:pt idx="383">
+                  <c:v>118.918559999999</c:v>
+                </c:pt>
+                <c:pt idx="384">
+                  <c:v>118.937368744186</c:v>
+                </c:pt>
+                <c:pt idx="385">
+                  <c:v>119.154453</c:v>
+                </c:pt>
+                <c:pt idx="386">
+                  <c:v>119.154453</c:v>
+                </c:pt>
+                <c:pt idx="387">
+                  <c:v>119.154453</c:v>
+                </c:pt>
+                <c:pt idx="388">
+                  <c:v>119.28465706976699</c:v>
+                </c:pt>
+                <c:pt idx="389">
+                  <c:v>119.37840399999899</c:v>
+                </c:pt>
+                <c:pt idx="390">
+                  <c:v>119.378404</c:v>
+                </c:pt>
+                <c:pt idx="391">
+                  <c:v>119.397056408637</c:v>
+                </c:pt>
+                <c:pt idx="392">
+                  <c:v>119.602979</c:v>
+                </c:pt>
+                <c:pt idx="393">
+                  <c:v>119.602979</c:v>
+                </c:pt>
+                <c:pt idx="394">
+                  <c:v>119.602979</c:v>
+                </c:pt>
+                <c:pt idx="395">
+                  <c:v>119.742083688741</c:v>
+                </c:pt>
+                <c:pt idx="396">
+                  <c:v>119.84166999999999</c:v>
+                </c:pt>
+                <c:pt idx="397">
+                  <c:v>119.84166999999999</c:v>
+                </c:pt>
+                <c:pt idx="398">
+                  <c:v>119.860219335548</c:v>
+                </c:pt>
+                <c:pt idx="399">
+                  <c:v>120.065004</c:v>
+                </c:pt>
+                <c:pt idx="400">
+                  <c:v>120.065004</c:v>
+                </c:pt>
+                <c:pt idx="401">
+                  <c:v>120.065004</c:v>
+                </c:pt>
+                <c:pt idx="402">
+                  <c:v>120.20694536876999</c:v>
+                </c:pt>
+                <c:pt idx="403">
+                  <c:v>120.307756</c:v>
+                </c:pt>
+                <c:pt idx="404">
+                  <c:v>120.307756</c:v>
+                </c:pt>
+                <c:pt idx="405">
+                  <c:v>120.327336152317</c:v>
+                </c:pt>
+                <c:pt idx="406">
+                  <c:v>120.535186999999</c:v>
+                </c:pt>
+                <c:pt idx="407">
+                  <c:v>120.535186999999</c:v>
+                </c:pt>
+                <c:pt idx="408">
+                  <c:v>120.535186999999</c:v>
+                </c:pt>
+                <c:pt idx="409">
+                  <c:v>120.654838348837</c:v>
+                </c:pt>
+                <c:pt idx="410">
+                  <c:v>120.739818</c:v>
+                </c:pt>
+                <c:pt idx="411">
+                  <c:v>120.739818</c:v>
+                </c:pt>
+                <c:pt idx="412">
+                  <c:v>120.75970592691</c:v>
+                </c:pt>
+                <c:pt idx="413">
+                  <c:v>120.97005900000001</c:v>
+                </c:pt>
+                <c:pt idx="414">
+                  <c:v>120.97005900000001</c:v>
+                </c:pt>
+                <c:pt idx="415">
+                  <c:v>120.97005900000001</c:v>
+                </c:pt>
+                <c:pt idx="416">
+                  <c:v>121.088440245847</c:v>
+                </c:pt>
+                <c:pt idx="417">
+                  <c:v>121.17137399999901</c:v>
+                </c:pt>
+                <c:pt idx="418">
+                  <c:v>121.17137399999901</c:v>
+                </c:pt>
+                <c:pt idx="419">
+                  <c:v>121.19160147019799</c:v>
+                </c:pt>
+                <c:pt idx="420">
+                  <c:v>121.397621999999</c:v>
+                </c:pt>
+                <c:pt idx="421">
+                  <c:v>121.397621999999</c:v>
+                </c:pt>
+                <c:pt idx="422">
+                  <c:v>121.397621999999</c:v>
+                </c:pt>
+                <c:pt idx="423">
+                  <c:v>121.525524199335</c:v>
+                </c:pt>
+                <c:pt idx="424">
+                  <c:v>121.615128</c:v>
+                </c:pt>
+                <c:pt idx="425">
+                  <c:v>121.615128</c:v>
+                </c:pt>
+                <c:pt idx="426">
+                  <c:v>121.634393262458</c:v>
+                </c:pt>
+                <c:pt idx="427">
+                  <c:v>121.82989999999999</c:v>
+                </c:pt>
+                <c:pt idx="428">
+                  <c:v>121.82989999999999</c:v>
+                </c:pt>
+                <c:pt idx="429">
+                  <c:v>121.829899999999</c:v>
+                </c:pt>
+                <c:pt idx="430">
+                  <c:v>121.95560998671</c:v>
+                </c:pt>
+                <c:pt idx="431">
+                  <c:v>122.04247700000001</c:v>
+                </c:pt>
+                <c:pt idx="432">
+                  <c:v>122.04247700000001</c:v>
+                </c:pt>
+                <c:pt idx="433">
+                  <c:v>122.061824428571</c:v>
+                </c:pt>
+                <c:pt idx="434">
+                  <c:v>122.25816500000001</c:v>
+                </c:pt>
+                <c:pt idx="435">
+                  <c:v>122.25816500000001</c:v>
+                </c:pt>
+                <c:pt idx="436">
+                  <c:v>122.25816500000001</c:v>
+                </c:pt>
+                <c:pt idx="437">
+                  <c:v>122.37994834219199</c:v>
+                </c:pt>
+                <c:pt idx="438">
+                  <c:v>122.464102</c:v>
+                </c:pt>
+                <c:pt idx="439">
+                  <c:v>122.464102</c:v>
+                </c:pt>
+                <c:pt idx="440">
+                  <c:v>122.482956232558</c:v>
+                </c:pt>
+                <c:pt idx="441">
+                  <c:v>122.666785</c:v>
+                </c:pt>
+                <c:pt idx="442">
+                  <c:v>122.666785</c:v>
+                </c:pt>
+                <c:pt idx="443">
+                  <c:v>122.666785</c:v>
+                </c:pt>
+                <c:pt idx="444">
+                  <c:v>122.788183748344</c:v>
+                </c:pt>
+                <c:pt idx="445">
+                  <c:v>122.871602999999</c:v>
+                </c:pt>
+                <c:pt idx="446">
+                  <c:v>122.871602999999</c:v>
+                </c:pt>
+                <c:pt idx="447">
+                  <c:v>122.892680581395</c:v>
+                </c:pt>
+                <c:pt idx="448">
+                  <c:v>123.098187</c:v>
+                </c:pt>
+                <c:pt idx="449">
+                  <c:v>123.098187</c:v>
+                </c:pt>
+                <c:pt idx="450">
+                  <c:v>123.098187</c:v>
+                </c:pt>
+                <c:pt idx="451">
+                  <c:v>123.20028895681</c:v>
+                </c:pt>
+                <c:pt idx="452">
+                  <c:v>123.26987800000001</c:v>
+                </c:pt>
+                <c:pt idx="453">
+                  <c:v>123.26987800000001</c:v>
+                </c:pt>
+                <c:pt idx="454">
+                  <c:v>123.292631572847</c:v>
+                </c:pt>
+                <c:pt idx="455">
+                  <c:v>123.506829</c:v>
+                </c:pt>
+                <c:pt idx="456">
+                  <c:v>123.506829</c:v>
+                </c:pt>
+                <c:pt idx="457">
+                  <c:v>123.506829</c:v>
+                </c:pt>
+                <c:pt idx="458">
+                  <c:v>123.61233105298</c:v>
+                </c:pt>
+                <c:pt idx="459">
+                  <c:v>123.68383799999999</c:v>
+                </c:pt>
+                <c:pt idx="460">
+                  <c:v>123.68383799999999</c:v>
+                </c:pt>
+                <c:pt idx="461">
+                  <c:v>123.70472002325501</c:v>
+                </c:pt>
+                <c:pt idx="462">
+                  <c:v>123.90057899999999</c:v>
+                </c:pt>
+                <c:pt idx="463">
+                  <c:v>123.90057899999999</c:v>
+                </c:pt>
+                <c:pt idx="464">
+                  <c:v>123.90057899999999</c:v>
+                </c:pt>
+                <c:pt idx="465">
+                  <c:v>124.01347727242501</c:v>
+                </c:pt>
+                <c:pt idx="466">
+                  <c:v>124.08937</c:v>
+                </c:pt>
+                <c:pt idx="467">
+                  <c:v>124.08937</c:v>
+                </c:pt>
+                <c:pt idx="468">
+                  <c:v>124.10826205298</c:v>
+                </c:pt>
+                <c:pt idx="469">
+                  <c:v>124.27954999999901</c:v>
+                </c:pt>
+                <c:pt idx="470">
+                  <c:v>124.27954999999901</c:v>
+                </c:pt>
+                <c:pt idx="471">
+                  <c:v>124.27954999999901</c:v>
+                </c:pt>
+                <c:pt idx="472">
+                  <c:v>124.394587940199</c:v>
+                </c:pt>
+                <c:pt idx="473">
+                  <c:v>124.471919</c:v>
+                </c:pt>
+                <c:pt idx="474">
+                  <c:v>124.471918999999</c:v>
+                </c:pt>
+                <c:pt idx="475">
+                  <c:v>124.48888783720901</c:v>
+                </c:pt>
+                <c:pt idx="476">
+                  <c:v>124.642172999999</c:v>
+                </c:pt>
+                <c:pt idx="477">
+                  <c:v>124.642172999999</c:v>
+                </c:pt>
+                <c:pt idx="478">
+                  <c:v>124.642172999999</c:v>
+                </c:pt>
+                <c:pt idx="479">
+                  <c:v>124.764586727574</c:v>
+                </c:pt>
+                <c:pt idx="480">
+                  <c:v>124.84574499999999</c:v>
+                </c:pt>
+                <c:pt idx="481">
+                  <c:v>124.84574499999999</c:v>
+                </c:pt>
+                <c:pt idx="482">
+                  <c:v>124.864452043189</c:v>
+                </c:pt>
+                <c:pt idx="483">
+                  <c:v>125.03343899999901</c:v>
+                </c:pt>
+                <c:pt idx="484">
+                  <c:v>125.033439</c:v>
+                </c:pt>
+                <c:pt idx="485">
+                  <c:v>125.033439</c:v>
+                </c:pt>
+                <c:pt idx="486">
+                  <c:v>125.148248923588</c:v>
+                </c:pt>
+                <c:pt idx="487">
+                  <c:v>125.22436599999899</c:v>
+                </c:pt>
+                <c:pt idx="488">
+                  <c:v>125.224366</c:v>
+                </c:pt>
+                <c:pt idx="489">
+                  <c:v>125.243392996677</c:v>
+                </c:pt>
+                <c:pt idx="490">
+                  <c:v>125.40911199999999</c:v>
+                </c:pt>
+                <c:pt idx="491">
+                  <c:v>125.40911199999999</c:v>
+                </c:pt>
+                <c:pt idx="492">
+                  <c:v>125.40911199999999</c:v>
+                </c:pt>
+                <c:pt idx="493">
+                  <c:v>125.522220178807</c:v>
+                </c:pt>
+                <c:pt idx="494">
+                  <c:v>125.596797</c:v>
+                </c:pt>
+                <c:pt idx="495">
+                  <c:v>125.596797</c:v>
+                </c:pt>
+                <c:pt idx="496">
+                  <c:v>125.615102551495</c:v>
+                </c:pt>
+                <c:pt idx="497">
+                  <c:v>125.77453800000001</c:v>
+                </c:pt>
+                <c:pt idx="498">
+                  <c:v>125.774537999999</c:v>
+                </c:pt>
+                <c:pt idx="499">
+                  <c:v>125.774537999999</c:v>
+                </c:pt>
+                <c:pt idx="500">
+                  <c:v>125.892414744186</c:v>
+                </c:pt>
+                <c:pt idx="501">
+                  <c:v>125.969487999999</c:v>
+                </c:pt>
+                <c:pt idx="502">
+                  <c:v>125.969488</c:v>
+                </c:pt>
+                <c:pt idx="503">
+                  <c:v>125.988221714285</c:v>
+                </c:pt>
+                <c:pt idx="504">
+                  <c:v>126.145702</c:v>
+                </c:pt>
+                <c:pt idx="505">
+                  <c:v>126.145702</c:v>
+                </c:pt>
+                <c:pt idx="506">
+                  <c:v>126.145702</c:v>
+                </c:pt>
+                <c:pt idx="507">
+                  <c:v>126.24448018874099</c:v>
+                </c:pt>
+                <c:pt idx="508">
+                  <c:v>126.308713</c:v>
+                </c:pt>
+                <c:pt idx="509">
+                  <c:v>126.308713</c:v>
+                </c:pt>
+                <c:pt idx="510">
+                  <c:v>126.330187976744</c:v>
+                </c:pt>
+                <c:pt idx="511">
+                  <c:v>126.510712</c:v>
+                </c:pt>
+                <c:pt idx="512">
+                  <c:v>126.510712</c:v>
+                </c:pt>
+                <c:pt idx="513">
+                  <c:v>126.510712</c:v>
+                </c:pt>
+                <c:pt idx="514">
+                  <c:v>126.606680604651</c:v>
+                </c:pt>
+                <c:pt idx="515">
+                  <c:v>126.66856199999999</c:v>
+                </c:pt>
+                <c:pt idx="516">
+                  <c:v>126.66856199999999</c:v>
+                </c:pt>
+                <c:pt idx="517">
+                  <c:v>126.688691781456</c:v>
+                </c:pt>
+                <c:pt idx="518">
+                  <c:v>126.852779999999</c:v>
+                </c:pt>
+                <c:pt idx="519">
+                  <c:v>126.852779999999</c:v>
+                </c:pt>
+                <c:pt idx="520">
+                  <c:v>126.852779999999</c:v>
+                </c:pt>
+                <c:pt idx="521">
+                  <c:v>126.96447444518201</c:v>
+                </c:pt>
+                <c:pt idx="522">
+                  <c:v>127.036496</c:v>
+                </c:pt>
+                <c:pt idx="523">
+                  <c:v>127.036496</c:v>
+                </c:pt>
+                <c:pt idx="524">
+                  <c:v>127.05415626245799</c:v>
+                </c:pt>
+                <c:pt idx="525">
+                  <c:v>127.197579</c:v>
+                </c:pt>
+                <c:pt idx="526">
+                  <c:v>127.197579</c:v>
+                </c:pt>
+                <c:pt idx="527">
+                  <c:v>127.197579</c:v>
+                </c:pt>
+                <c:pt idx="528">
+                  <c:v>127.308240023255</c:v>
+                </c:pt>
+                <c:pt idx="529">
+                  <c:v>127.378605999999</c:v>
+                </c:pt>
+                <c:pt idx="530">
+                  <c:v>127.378605999999</c:v>
+                </c:pt>
+                <c:pt idx="531">
+                  <c:v>127.395420870431</c:v>
+                </c:pt>
+                <c:pt idx="532">
+                  <c:v>127.531977999999</c:v>
+                </c:pt>
+                <c:pt idx="533">
+                  <c:v>127.531978</c:v>
+                </c:pt>
+                <c:pt idx="534">
+                  <c:v>127.531978</c:v>
+                </c:pt>
+                <c:pt idx="535">
+                  <c:v>127.62338993355399</c:v>
+                </c:pt>
+                <c:pt idx="536">
+                  <c:v>127.681516</c:v>
+                </c:pt>
+                <c:pt idx="537">
+                  <c:v>127.681516</c:v>
+                </c:pt>
+                <c:pt idx="538">
+                  <c:v>127.700681607973</c:v>
+                </c:pt>
+                <c:pt idx="539">
+                  <c:v>127.85118799999999</c:v>
+                </c:pt>
+                <c:pt idx="540">
+                  <c:v>127.85118799999999</c:v>
+                </c:pt>
+                <c:pt idx="541">
+                  <c:v>127.85118799999999</c:v>
+                </c:pt>
+                <c:pt idx="542">
+                  <c:v>127.942093681063</c:v>
+                </c:pt>
+                <c:pt idx="543">
+                  <c:v>127.999093999999</c:v>
+                </c:pt>
+                <c:pt idx="544">
+                  <c:v>127.999093999999</c:v>
+                </c:pt>
+                <c:pt idx="545">
+                  <c:v>128.01915524252399</c:v>
+                </c:pt>
+                <c:pt idx="546">
+                  <c:v>128.176695</c:v>
+                </c:pt>
+                <c:pt idx="547">
+                  <c:v>128.176695</c:v>
+                </c:pt>
+                <c:pt idx="548">
+                  <c:v>128.176695</c:v>
+                </c:pt>
+                <c:pt idx="549">
+                  <c:v>128.285433820598</c:v>
+                </c:pt>
+                <c:pt idx="550">
+                  <c:v>128.35361599999999</c:v>
+                </c:pt>
+                <c:pt idx="551">
+                  <c:v>128.35361599999999</c:v>
+                </c:pt>
+                <c:pt idx="552">
+                  <c:v>128.36816751162701</c:v>
+                </c:pt>
+                <c:pt idx="553">
+                  <c:v>128.478759</c:v>
+                </c:pt>
+                <c:pt idx="554">
+                  <c:v>128.478759</c:v>
+                </c:pt>
+                <c:pt idx="555">
+                  <c:v>128.478759</c:v>
+                </c:pt>
+                <c:pt idx="556">
+                  <c:v>128.573702761589</c:v>
+                </c:pt>
+                <c:pt idx="557">
+                  <c:v>128.632915</c:v>
+                </c:pt>
+                <c:pt idx="558">
+                  <c:v>128.632915</c:v>
+                </c:pt>
+                <c:pt idx="559">
+                  <c:v>128.65348348837199</c:v>
+                </c:pt>
+                <c:pt idx="560">
+                  <c:v>128.80980400000001</c:v>
+                </c:pt>
+                <c:pt idx="561">
+                  <c:v>128.80980400000001</c:v>
+                </c:pt>
+                <c:pt idx="562">
+                  <c:v>128.80980400000001</c:v>
+                </c:pt>
+                <c:pt idx="563">
+                  <c:v>128.90534620598001</c:v>
+                </c:pt>
+                <c:pt idx="564">
+                  <c:v>128.96441799999999</c:v>
+                </c:pt>
+                <c:pt idx="565">
+                  <c:v>128.96441799999999</c:v>
+                </c:pt>
+                <c:pt idx="566">
+                  <c:v>128.982070874172</c:v>
+                </c:pt>
+                <c:pt idx="567">
+                  <c:v>129.112506</c:v>
+                </c:pt>
+                <c:pt idx="568">
+                  <c:v>129.112506</c:v>
+                </c:pt>
+                <c:pt idx="569">
+                  <c:v>129.112506</c:v>
+                </c:pt>
+                <c:pt idx="570">
+                  <c:v>129.20423118936799</c:v>
+                </c:pt>
+                <c:pt idx="571">
+                  <c:v>129.260943</c:v>
+                </c:pt>
+                <c:pt idx="572">
+                  <c:v>129.260943</c:v>
+                </c:pt>
+                <c:pt idx="573">
+                  <c:v>129.28081703322201</c:v>
+                </c:pt>
+                <c:pt idx="574">
+                  <c:v>129.42711199999999</c:v>
+                </c:pt>
+                <c:pt idx="575">
+                  <c:v>129.42711199999999</c:v>
+                </c:pt>
+                <c:pt idx="576">
+                  <c:v>129.42711199999999</c:v>
+                </c:pt>
+                <c:pt idx="577">
+                  <c:v>129.51523683720899</c:v>
+                </c:pt>
+                <c:pt idx="578">
+                  <c:v>129.56896</c:v>
+                </c:pt>
+                <c:pt idx="579">
+                  <c:v>129.56896</c:v>
+                </c:pt>
+                <c:pt idx="580">
+                  <c:v>129.58725445847099</c:v>
+                </c:pt>
+                <c:pt idx="581">
+                  <c:v>129.72192200000001</c:v>
+                </c:pt>
+                <c:pt idx="582">
+                  <c:v>129.72192200000001</c:v>
+                </c:pt>
+                <c:pt idx="583">
+                  <c:v>129.72192200000001</c:v>
+                </c:pt>
+                <c:pt idx="584">
+                  <c:v>129.83010305315599</c:v>
+                </c:pt>
+                <c:pt idx="585">
+                  <c:v>129.89605299999999</c:v>
+                </c:pt>
+                <c:pt idx="586">
+                  <c:v>129.89605299999999</c:v>
+                </c:pt>
+                <c:pt idx="587">
+                  <c:v>129.91344865448499</c:v>
+                </c:pt>
+                <c:pt idx="588">
+                  <c:v>130.03756899999999</c:v>
+                </c:pt>
+                <c:pt idx="589">
+                  <c:v>130.03756899999999</c:v>
+                </c:pt>
+                <c:pt idx="590">
+                  <c:v>130.03756899999999</c:v>
+                </c:pt>
+                <c:pt idx="591">
+                  <c:v>130.12070434883699</c:v>
+                </c:pt>
+                <c:pt idx="592">
+                  <c:v>130.17067399999999</c:v>
+                </c:pt>
+                <c:pt idx="593">
+                  <c:v>130.17067399999999</c:v>
+                </c:pt>
+                <c:pt idx="594">
+                  <c:v>130.18977780066399</c:v>
+                </c:pt>
+                <c:pt idx="595">
+                  <c:v>130.326086</c:v>
+                </c:pt>
+                <c:pt idx="596">
+                  <c:v>130.326086</c:v>
+                </c:pt>
+                <c:pt idx="597">
+                  <c:v>130.326086</c:v>
+                </c:pt>
+                <c:pt idx="598">
+                  <c:v>130.42364550830499</c:v>
+                </c:pt>
+                <c:pt idx="599">
+                  <c:v>130.48228499999999</c:v>
+                </c:pt>
+                <c:pt idx="600">
+                  <c:v>130.48228499999999</c:v>
+                </c:pt>
+                <c:pt idx="601">
+                  <c:v>130.499546089701</c:v>
+                </c:pt>
+                <c:pt idx="602">
+                  <c:v>130.619011</c:v>
+                </c:pt>
+                <c:pt idx="603">
+                  <c:v>130.619011</c:v>
+                </c:pt>
+                <c:pt idx="604">
+                  <c:v>130.619011</c:v>
+                </c:pt>
+                <c:pt idx="605">
+                  <c:v>130.70636905297999</c:v>
+                </c:pt>
+                <c:pt idx="606">
+                  <c:v>130.758599</c:v>
+                </c:pt>
+                <c:pt idx="607">
+                  <c:v>130.758599</c:v>
+                </c:pt>
+                <c:pt idx="608">
+                  <c:v>130.77584367774</c:v>
+                </c:pt>
+                <c:pt idx="609">
+                  <c:v>130.895195</c:v>
+                </c:pt>
+                <c:pt idx="610">
+                  <c:v>130.895195</c:v>
+                </c:pt>
+                <c:pt idx="611">
+                  <c:v>130.895195</c:v>
+                </c:pt>
+                <c:pt idx="612">
+                  <c:v>130.99605883720901</c:v>
+                </c:pt>
+                <c:pt idx="613">
+                  <c:v>131.05582999999999</c:v>
+                </c:pt>
+                <c:pt idx="614">
+                  <c:v>131.05582999999999</c:v>
+                </c:pt>
+                <c:pt idx="615">
+                  <c:v>131.07409181456899</c:v>
+                </c:pt>
+                <c:pt idx="616">
+                  <c:v>131.19724199999999</c:v>
+                </c:pt>
+                <c:pt idx="617">
+                  <c:v>131.19724199999999</c:v>
+                </c:pt>
+                <c:pt idx="618">
+                  <c:v>131.19724199999999</c:v>
+                </c:pt>
+                <c:pt idx="619">
+                  <c:v>131.27956437209301</c:v>
+                </c:pt>
+                <c:pt idx="620">
+                  <c:v>131.32834800000001</c:v>
+                </c:pt>
+                <c:pt idx="621">
+                  <c:v>131.32834800000001</c:v>
+                </c:pt>
+                <c:pt idx="622">
+                  <c:v>131.347359657807</c:v>
+                </c:pt>
+                <c:pt idx="623">
+                  <c:v>131.47507899999999</c:v>
+                </c:pt>
+                <c:pt idx="624">
+                  <c:v>131.47507899999999</c:v>
+                </c:pt>
+                <c:pt idx="625">
+                  <c:v>131.47507899999999</c:v>
+                </c:pt>
+                <c:pt idx="626">
+                  <c:v>131.55572295348799</c:v>
+                </c:pt>
+                <c:pt idx="627">
+                  <c:v>131.602836</c:v>
+                </c:pt>
+                <c:pt idx="628">
+                  <c:v>131.602836</c:v>
+                </c:pt>
+                <c:pt idx="629">
+                  <c:v>131.620870966887</c:v>
+                </c:pt>
+                <c:pt idx="630">
+                  <c:v>131.739</c:v>
+                </c:pt>
+                <c:pt idx="631">
+                  <c:v>131.739</c:v>
+                </c:pt>
+                <c:pt idx="632">
+                  <c:v>131.739</c:v>
+                </c:pt>
+                <c:pt idx="633">
+                  <c:v>131.827529900332</c:v>
+                </c:pt>
+                <c:pt idx="634">
+                  <c:v>131.87925000000001</c:v>
+                </c:pt>
+                <c:pt idx="635">
+                  <c:v>131.87925000000001</c:v>
+                </c:pt>
+                <c:pt idx="636">
+                  <c:v>131.89787644518199</c:v>
+                </c:pt>
+                <c:pt idx="637">
+                  <c:v>132.01941400000001</c:v>
+                </c:pt>
+                <c:pt idx="638">
+                  <c:v>132.01941400000001</c:v>
+                </c:pt>
+                <c:pt idx="639">
+                  <c:v>132.01941400000001</c:v>
+                </c:pt>
+                <c:pt idx="640">
+                  <c:v>132.10411583720901</c:v>
+                </c:pt>
+                <c:pt idx="641">
+                  <c:v>132.152897</c:v>
+                </c:pt>
+                <c:pt idx="642">
+                  <c:v>132.152897</c:v>
+                </c:pt>
+                <c:pt idx="643">
+                  <c:v>132.17266909302299</c:v>
+                </c:pt>
+                <c:pt idx="644">
+                  <c:v>132.301682</c:v>
+                </c:pt>
+                <c:pt idx="645">
+                  <c:v>132.301682</c:v>
+                </c:pt>
+                <c:pt idx="646">
+                  <c:v>132.301682</c:v>
+                </c:pt>
+                <c:pt idx="647">
+                  <c:v>132.364838910299</c:v>
+                </c:pt>
+                <c:pt idx="648">
+                  <c:v>132.40121199999999</c:v>
+                </c:pt>
+                <c:pt idx="649">
+                  <c:v>132.40121199999999</c:v>
+                </c:pt>
+                <c:pt idx="650">
+                  <c:v>132.420974</c:v>
+                </c:pt>
+                <c:pt idx="651">
+                  <c:v>132.54629399999999</c:v>
+                </c:pt>
+                <c:pt idx="652">
+                  <c:v>132.54629399999999</c:v>
+                </c:pt>
+                <c:pt idx="653">
+                  <c:v>132.54629399999999</c:v>
+                </c:pt>
+                <c:pt idx="654">
+                  <c:v>132.63047900662201</c:v>
+                </c:pt>
+                <c:pt idx="655">
+                  <c:v>132.67871</c:v>
+                </c:pt>
+                <c:pt idx="656">
+                  <c:v>132.67871</c:v>
+                </c:pt>
+                <c:pt idx="657">
+                  <c:v>132.69410584053099</c:v>
+                </c:pt>
+                <c:pt idx="658">
+                  <c:v>132.79173800000001</c:v>
+                </c:pt>
+                <c:pt idx="659">
+                  <c:v>132.79173800000001</c:v>
+                </c:pt>
+                <c:pt idx="660">
+                  <c:v>132.79173800000001</c:v>
+                </c:pt>
+                <c:pt idx="661">
+                  <c:v>132.87757348172701</c:v>
+                </c:pt>
+                <c:pt idx="662">
+                  <c:v>132.92630299999999</c:v>
+                </c:pt>
+                <c:pt idx="663">
+                  <c:v>132.92630299999999</c:v>
+                </c:pt>
+                <c:pt idx="664">
+                  <c:v>132.94473849668799</c:v>
+                </c:pt>
+                <c:pt idx="665">
+                  <c:v>133.058863</c:v>
+                </c:pt>
+                <c:pt idx="666">
+                  <c:v>133.058863</c:v>
+                </c:pt>
+                <c:pt idx="667">
+                  <c:v>133.058863</c:v>
+                </c:pt>
+                <c:pt idx="668">
+                  <c:v>133.137231864238</c:v>
+                </c:pt>
+                <c:pt idx="669">
+                  <c:v>133.18149199999999</c:v>
+                </c:pt>
+                <c:pt idx="670">
+                  <c:v>133.18149199999999</c:v>
+                </c:pt>
+                <c:pt idx="671">
+                  <c:v>133.19840753488299</c:v>
+                </c:pt>
+                <c:pt idx="672">
+                  <c:v>133.30271999999999</c:v>
+                </c:pt>
+                <c:pt idx="673">
+                  <c:v>133.30271999999999</c:v>
+                </c:pt>
+                <c:pt idx="674">
+                  <c:v>133.30271999999999</c:v>
+                </c:pt>
+                <c:pt idx="675">
+                  <c:v>133.38497134219199</c:v>
+                </c:pt>
+                <c:pt idx="676">
+                  <c:v>133.43099799999999</c:v>
+                </c:pt>
+                <c:pt idx="677">
+                  <c:v>133.43099799999999</c:v>
+                </c:pt>
+                <c:pt idx="678">
+                  <c:v>133.44700624503301</c:v>
+                </c:pt>
+                <c:pt idx="679">
+                  <c:v>133.54342800000001</c:v>
+                </c:pt>
+                <c:pt idx="680">
+                  <c:v>133.54342800000001</c:v>
+                </c:pt>
+                <c:pt idx="681">
+                  <c:v>133.54342800000001</c:v>
+                </c:pt>
+                <c:pt idx="682">
+                  <c:v>133.60880434551399</c:v>
+                </c:pt>
+                <c:pt idx="683">
+                  <c:v>133.645388</c:v>
+                </c:pt>
+                <c:pt idx="684">
+                  <c:v>133.645388</c:v>
+                </c:pt>
+                <c:pt idx="685">
+                  <c:v>133.662340142857</c:v>
+                </c:pt>
+                <c:pt idx="686">
+                  <c:v>133.76405299999999</c:v>
+                </c:pt>
+                <c:pt idx="687">
+                  <c:v>133.76405299999999</c:v>
+                </c:pt>
+                <c:pt idx="688">
+                  <c:v>133.76405299999999</c:v>
+                </c:pt>
+                <c:pt idx="689">
+                  <c:v>133.827910581395</c:v>
+                </c:pt>
+                <c:pt idx="690">
+                  <c:v>133.86313100000001</c:v>
+                </c:pt>
+                <c:pt idx="691">
+                  <c:v>133.86313100000001</c:v>
+                </c:pt>
+                <c:pt idx="692">
+                  <c:v>133.88332800000001</c:v>
+                </c:pt>
+                <c:pt idx="693">
+                  <c:v>134.00451000000001</c:v>
+                </c:pt>
+                <c:pt idx="694">
+                  <c:v>134.00451000000001</c:v>
+                </c:pt>
+                <c:pt idx="695">
+                  <c:v>134.00451000000001</c:v>
+                </c:pt>
+                <c:pt idx="696">
+                  <c:v>134.09032051827199</c:v>
+                </c:pt>
+                <c:pt idx="697">
+                  <c:v>134.13764900000001</c:v>
+                </c:pt>
+                <c:pt idx="698">
+                  <c:v>134.13764900000001</c:v>
+                </c:pt>
+                <c:pt idx="699">
+                  <c:v>134.153906196013</c:v>
+                </c:pt>
+                <c:pt idx="700">
+                  <c:v>134.248863</c:v>
+                </c:pt>
+                <c:pt idx="701">
+                  <c:v>134.248863</c:v>
+                </c:pt>
+                <c:pt idx="702">
+                  <c:v>134.248863</c:v>
+                </c:pt>
+                <c:pt idx="703">
+                  <c:v>134.328802668874</c:v>
+                </c:pt>
+                <c:pt idx="704">
+                  <c:v>134.37266700000001</c:v>
+                </c:pt>
+                <c:pt idx="705">
+                  <c:v>134.37266700000001</c:v>
+                </c:pt>
+                <c:pt idx="706">
+                  <c:v>134.389063797342</c:v>
+                </c:pt>
+                <c:pt idx="707">
+                  <c:v>134.484836</c:v>
+                </c:pt>
+                <c:pt idx="708">
+                  <c:v>134.484836</c:v>
+                </c:pt>
+                <c:pt idx="709">
+                  <c:v>134.484836</c:v>
+                </c:pt>
+                <c:pt idx="710">
+                  <c:v>134.56272910631199</c:v>
+                </c:pt>
+                <c:pt idx="711">
+                  <c:v>134.60507100000001</c:v>
+                </c:pt>
+                <c:pt idx="712">
+                  <c:v>134.60507100000001</c:v>
+                </c:pt>
+                <c:pt idx="713">
+                  <c:v>134.619504039867</c:v>
+                </c:pt>
+                <c:pt idx="714">
+                  <c:v>134.70161200000001</c:v>
+                </c:pt>
+                <c:pt idx="715">
+                  <c:v>134.70161200000001</c:v>
+                </c:pt>
+                <c:pt idx="716">
+                  <c:v>134.70161200000001</c:v>
+                </c:pt>
+                <c:pt idx="717">
+                  <c:v>134.792773417218</c:v>
+                </c:pt>
+                <c:pt idx="718">
+                  <c:v>134.84207499999999</c:v>
+                </c:pt>
+                <c:pt idx="719">
+                  <c:v>134.84207499999999</c:v>
+                </c:pt>
+                <c:pt idx="720">
+                  <c:v>134.85754079734201</c:v>
+                </c:pt>
+                <c:pt idx="721">
+                  <c:v>134.94552400000001</c:v>
+                </c:pt>
+                <c:pt idx="722">
+                  <c:v>134.94552400000001</c:v>
+                </c:pt>
+                <c:pt idx="723">
+                  <c:v>134.94552400000001</c:v>
+                </c:pt>
+                <c:pt idx="724">
+                  <c:v>135.01926297674399</c:v>
+                </c:pt>
+                <c:pt idx="725">
+                  <c:v>135.05876599999999</c:v>
+                </c:pt>
+                <c:pt idx="726">
+                  <c:v>135.05876599999999</c:v>
+                </c:pt>
+                <c:pt idx="727">
+                  <c:v>135.07188300662199</c:v>
+                </c:pt>
+                <c:pt idx="728">
+                  <c:v>135.144882</c:v>
+                </c:pt>
+                <c:pt idx="729">
+                  <c:v>135.144882</c:v>
+                </c:pt>
+                <c:pt idx="730">
+                  <c:v>135.144882</c:v>
+                </c:pt>
+                <c:pt idx="731">
+                  <c:v>135.21370730232499</c:v>
+                </c:pt>
+                <c:pt idx="732">
+                  <c:v>135.25057799999999</c:v>
+                </c:pt>
+                <c:pt idx="733">
+                  <c:v>135.25057799999999</c:v>
+                </c:pt>
+                <c:pt idx="734">
+                  <c:v>135.26775861793999</c:v>
+                </c:pt>
+                <c:pt idx="735">
+                  <c:v>135.362999</c:v>
+                </c:pt>
+                <c:pt idx="736">
+                  <c:v>135.362999</c:v>
+                </c:pt>
+                <c:pt idx="737">
+                  <c:v>135.362999</c:v>
+                </c:pt>
+                <c:pt idx="738">
+                  <c:v>135.44341099667699</c:v>
+                </c:pt>
+                <c:pt idx="739">
+                  <c:v>135.485862</c:v>
+                </c:pt>
+                <c:pt idx="740">
+                  <c:v>135.485862</c:v>
+                </c:pt>
+                <c:pt idx="741">
+                  <c:v>135.50104796013201</c:v>
+                </c:pt>
+                <c:pt idx="742">
+                  <c:v>135.58523099999999</c:v>
+                </c:pt>
+                <c:pt idx="743">
+                  <c:v>135.58523099999999</c:v>
+                </c:pt>
+                <c:pt idx="744">
+                  <c:v>135.58523099999999</c:v>
+                </c:pt>
+                <c:pt idx="745">
+                  <c:v>135.65606591694299</c:v>
+                </c:pt>
+                <c:pt idx="746">
+                  <c:v>135.69346100000001</c:v>
+                </c:pt>
+                <c:pt idx="747">
+                  <c:v>135.69346100000001</c:v>
+                </c:pt>
+                <c:pt idx="748">
+                  <c:v>135.711542727574</c:v>
+                </c:pt>
+                <c:pt idx="749">
+                  <c:v>135.80926099999999</c:v>
+                </c:pt>
+                <c:pt idx="750">
+                  <c:v>135.80926099999999</c:v>
+                </c:pt>
+                <c:pt idx="751">
+                  <c:v>135.80926099999999</c:v>
+                </c:pt>
+                <c:pt idx="752">
+                  <c:v>135.873797817275</c:v>
+                </c:pt>
+                <c:pt idx="753">
+                  <c:v>135.90736999999999</c:v>
+                </c:pt>
+                <c:pt idx="754">
+                  <c:v>135.90736999999999</c:v>
+                </c:pt>
+                <c:pt idx="755">
+                  <c:v>135.92184678072999</c:v>
+                </c:pt>
+                <c:pt idx="756">
+                  <c:v>136.00008299999999</c:v>
+                </c:pt>
+                <c:pt idx="757">
+                  <c:v>136.00008299999999</c:v>
+                </c:pt>
+                <c:pt idx="758">
+                  <c:v>136.00008299999999</c:v>
+                </c:pt>
+                <c:pt idx="759">
+                  <c:v>136.06999936544801</c:v>
+                </c:pt>
+                <c:pt idx="760">
+                  <c:v>136.10637</c:v>
+                </c:pt>
+                <c:pt idx="761">
+                  <c:v>136.10637</c:v>
+                </c:pt>
+                <c:pt idx="762">
+                  <c:v>136.120281069767</c:v>
+                </c:pt>
+                <c:pt idx="763">
+                  <c:v>136.19360399999999</c:v>
+                </c:pt>
+                <c:pt idx="764">
+                  <c:v>136.19360399999999</c:v>
+                </c:pt>
+                <c:pt idx="765">
+                  <c:v>136.19360399999999</c:v>
+                </c:pt>
+                <c:pt idx="766">
+                  <c:v>136.275736966887</c:v>
+                </c:pt>
+                <c:pt idx="767">
+                  <c:v>136.31824800000001</c:v>
+                </c:pt>
+                <c:pt idx="768">
+                  <c:v>136.31824800000001</c:v>
+                </c:pt>
+                <c:pt idx="769">
+                  <c:v>136.33551795348799</c:v>
+                </c:pt>
+                <c:pt idx="770">
+                  <c:v>136.426545</c:v>
+                </c:pt>
+                <c:pt idx="771">
+                  <c:v>136.426545</c:v>
+                </c:pt>
+                <c:pt idx="772">
+                  <c:v>136.426545</c:v>
+                </c:pt>
+                <c:pt idx="773">
+                  <c:v>136.47785063787299</c:v>
+                </c:pt>
+                <c:pt idx="774">
+                  <c:v>136.50414799999999</c:v>
+                </c:pt>
+                <c:pt idx="775">
+                  <c:v>136.50414799999999</c:v>
+                </c:pt>
+                <c:pt idx="776">
+                  <c:v>136.52337449668801</c:v>
+                </c:pt>
+                <c:pt idx="777">
+                  <c:v>136.622646</c:v>
+                </c:pt>
+                <c:pt idx="778">
+                  <c:v>136.622646</c:v>
+                </c:pt>
+                <c:pt idx="779">
+                  <c:v>136.622646</c:v>
+                </c:pt>
+                <c:pt idx="780">
+                  <c:v>136.68927992690999</c:v>
+                </c:pt>
+                <c:pt idx="781">
+                  <c:v>136.723434</c:v>
+                </c:pt>
+                <c:pt idx="782">
+                  <c:v>136.723434</c:v>
+                </c:pt>
+                <c:pt idx="783">
+                  <c:v>136.73766386046501</c:v>
+                </c:pt>
+                <c:pt idx="784">
+                  <c:v>136.810846</c:v>
+                </c:pt>
+                <c:pt idx="785">
+                  <c:v>136.810846</c:v>
+                </c:pt>
+                <c:pt idx="786">
+                  <c:v>136.810846</c:v>
+                </c:pt>
+                <c:pt idx="787">
+                  <c:v>136.87183869102901</c:v>
+                </c:pt>
+                <c:pt idx="788">
+                  <c:v>136.90263999999999</c:v>
+                </c:pt>
+                <c:pt idx="789">
+                  <c:v>136.90263999999999</c:v>
+                </c:pt>
+                <c:pt idx="790">
+                  <c:v>136.91896764900599</c:v>
+                </c:pt>
+                <c:pt idx="791">
+                  <c:v>137.001259</c:v>
+                </c:pt>
+                <c:pt idx="792">
+                  <c:v>137.001259</c:v>
+                </c:pt>
+                <c:pt idx="793">
+                  <c:v>137.001259</c:v>
+                </c:pt>
+                <c:pt idx="794">
+                  <c:v>137.06861846843799</c:v>
+                </c:pt>
+                <c:pt idx="795">
+                  <c:v>137.10263499999999</c:v>
+                </c:pt>
+                <c:pt idx="796">
+                  <c:v>137.10263499999999</c:v>
+                </c:pt>
+                <c:pt idx="797">
+                  <c:v>137.11845127906901</c:v>
+                </c:pt>
+                <c:pt idx="798">
+                  <c:v>137.19784899999999</c:v>
+                </c:pt>
+                <c:pt idx="799">
+                  <c:v>137.19784899999999</c:v>
+                </c:pt>
+                <c:pt idx="800">
+                  <c:v>137.19784899999999</c:v>
+                </c:pt>
+                <c:pt idx="801">
+                  <c:v>137.27200330897</c:v>
+                </c:pt>
+                <c:pt idx="802">
+                  <c:v>137.308896</c:v>
+                </c:pt>
+                <c:pt idx="803">
+                  <c:v>137.308896</c:v>
+                </c:pt>
+                <c:pt idx="804">
+                  <c:v>137.32423005315599</c:v>
+                </c:pt>
+                <c:pt idx="805">
+                  <c:v>137.401207</c:v>
+                </c:pt>
+                <c:pt idx="806">
+                  <c:v>137.401207</c:v>
+                </c:pt>
+                <c:pt idx="807">
+                  <c:v>137.401207</c:v>
+                </c:pt>
+                <c:pt idx="808">
+                  <c:v>137.45675445182701</c:v>
+                </c:pt>
+                <c:pt idx="809">
+                  <c:v>137.48438999999999</c:v>
+                </c:pt>
+                <c:pt idx="810">
+                  <c:v>137.48438999999999</c:v>
+                </c:pt>
+                <c:pt idx="811">
+                  <c:v>137.500867744186</c:v>
+                </c:pt>
+                <c:pt idx="812">
+                  <c:v>137.58164099999999</c:v>
+                </c:pt>
+                <c:pt idx="813">
+                  <c:v>137.58164099999999</c:v>
+                </c:pt>
+                <c:pt idx="814">
+                  <c:v>137.58164099999999</c:v>
+                </c:pt>
+                <c:pt idx="815">
+                  <c:v>137.647909039735</c:v>
+                </c:pt>
+                <c:pt idx="816">
+                  <c:v>137.68071499999999</c:v>
+                </c:pt>
+                <c:pt idx="817">
+                  <c:v>137.68071499999999</c:v>
+                </c:pt>
+                <c:pt idx="818">
+                  <c:v>137.696416730897</c:v>
+                </c:pt>
+                <c:pt idx="819">
+                  <c:v>137.77338599999999</c:v>
+                </c:pt>
+                <c:pt idx="820">
+                  <c:v>137.77338599999999</c:v>
+                </c:pt>
+                <c:pt idx="821">
+                  <c:v>137.77338599999999</c:v>
+                </c:pt>
+                <c:pt idx="822">
+                  <c:v>137.821667355481</c:v>
+                </c:pt>
+                <c:pt idx="823">
+                  <c:v>137.84532999999999</c:v>
+                </c:pt>
+                <c:pt idx="824">
+                  <c:v>137.84532999999999</c:v>
+                </c:pt>
+                <c:pt idx="825">
+                  <c:v>137.862113947019</c:v>
+                </c:pt>
+                <c:pt idx="826">
+                  <c:v>137.94280599999999</c:v>
+                </c:pt>
+                <c:pt idx="827">
+                  <c:v>137.94280599999999</c:v>
+                </c:pt>
+                <c:pt idx="828">
+                  <c:v>137.94280599999999</c:v>
+                </c:pt>
+                <c:pt idx="829">
+                  <c:v>137.99932573421901</c:v>
+                </c:pt>
+                <c:pt idx="830">
+                  <c:v>138.02702600000001</c:v>
+                </c:pt>
+                <c:pt idx="831">
+                  <c:v>138.02702600000001</c:v>
+                </c:pt>
+                <c:pt idx="832">
+                  <c:v>138.04323220597999</c:v>
+                </c:pt>
+                <c:pt idx="833">
+                  <c:v>138.120835</c:v>
+                </c:pt>
+                <c:pt idx="834">
+                  <c:v>138.120835</c:v>
+                </c:pt>
+                <c:pt idx="835">
+                  <c:v>138.120835</c:v>
+                </c:pt>
+                <c:pt idx="836">
+                  <c:v>138.178246906976</c:v>
+                </c:pt>
+                <c:pt idx="837">
+                  <c:v>138.205963</c:v>
+                </c:pt>
+                <c:pt idx="838">
+                  <c:v>138.205963</c:v>
+                </c:pt>
+                <c:pt idx="839">
+                  <c:v>138.21788957947001</c:v>
+                </c:pt>
+                <c:pt idx="840">
+                  <c:v>138.273922</c:v>
+                </c:pt>
+                <c:pt idx="841">
+                  <c:v>138.273922</c:v>
+                </c:pt>
+                <c:pt idx="842">
+                  <c:v>138.273922</c:v>
+                </c:pt>
+                <c:pt idx="843">
+                  <c:v>138.34843513953399</c:v>
+                </c:pt>
+                <c:pt idx="844">
+                  <c:v>138.38440700000001</c:v>
+                </c:pt>
+                <c:pt idx="845">
+                  <c:v>138.38440700000001</c:v>
+                </c:pt>
+                <c:pt idx="846">
+                  <c:v>138.40132702989999</c:v>
+                </c:pt>
+                <c:pt idx="847">
+                  <c:v>138.48050000000001</c:v>
+                </c:pt>
+                <c:pt idx="848">
+                  <c:v>138.48050000000001</c:v>
+                </c:pt>
+                <c:pt idx="849">
+                  <c:v>138.48050000000001</c:v>
+                </c:pt>
+                <c:pt idx="850">
+                  <c:v>138.53590599335499</c:v>
+                </c:pt>
+                <c:pt idx="851">
+                  <c:v>138.562251</c:v>
+                </c:pt>
+                <c:pt idx="852">
+                  <c:v>138.562251</c:v>
+                </c:pt>
+                <c:pt idx="853">
+                  <c:v>138.57512929568099</c:v>
+                </c:pt>
+                <c:pt idx="854">
+                  <c:v>138.63539</c:v>
+                </c:pt>
+                <c:pt idx="855">
+                  <c:v>138.63539</c:v>
+                </c:pt>
+                <c:pt idx="856">
+                  <c:v>138.63539</c:v>
+                </c:pt>
+                <c:pt idx="857">
+                  <c:v>138.67405172757401</c:v>
+                </c:pt>
+                <c:pt idx="858">
+                  <c:v>138.69243499999999</c:v>
+                </c:pt>
+                <c:pt idx="859">
+                  <c:v>138.69243499999999</c:v>
+                </c:pt>
+                <c:pt idx="860">
+                  <c:v>138.71148713289</c:v>
+                </c:pt>
+                <c:pt idx="861">
+                  <c:v>138.798633</c:v>
+                </c:pt>
+                <c:pt idx="862">
+                  <c:v>138.798633</c:v>
+                </c:pt>
+                <c:pt idx="863">
+                  <c:v>138.798633</c:v>
+                </c:pt>
+                <c:pt idx="864">
+                  <c:v>138.85050410927099</c:v>
+                </c:pt>
+                <c:pt idx="865">
+                  <c:v>138.87504799999999</c:v>
+                </c:pt>
+                <c:pt idx="866">
+                  <c:v>138.87504799999999</c:v>
+                </c:pt>
+                <c:pt idx="867">
+                  <c:v>138.889567900332</c:v>
+                </c:pt>
+                <c:pt idx="868">
+                  <c:v>138.955983</c:v>
+                </c:pt>
+                <c:pt idx="869">
+                  <c:v>138.955983</c:v>
+                </c:pt>
+                <c:pt idx="870">
+                  <c:v>138.955983</c:v>
+                </c:pt>
+                <c:pt idx="871">
+                  <c:v>139.006662950166</c:v>
+                </c:pt>
+                <c:pt idx="872">
+                  <c:v>139.030396</c:v>
+                </c:pt>
+                <c:pt idx="873">
+                  <c:v>139.030396</c:v>
+                </c:pt>
+                <c:pt idx="874">
+                  <c:v>139.046991747508</c:v>
+                </c:pt>
+                <c:pt idx="875">
+                  <c:v>139.12121999999999</c:v>
+                </c:pt>
+                <c:pt idx="876">
+                  <c:v>139.12121999999999</c:v>
+                </c:pt>
+                <c:pt idx="877">
+                  <c:v>139.12121999999999</c:v>
+                </c:pt>
+                <c:pt idx="878">
+                  <c:v>139.193015092715</c:v>
+                </c:pt>
+                <c:pt idx="879">
+                  <c:v>139.226473</c:v>
+                </c:pt>
+                <c:pt idx="880">
+                  <c:v>139.226473</c:v>
+                </c:pt>
+                <c:pt idx="881">
+                  <c:v>139.24027288372</c:v>
+                </c:pt>
+                <c:pt idx="882">
+                  <c:v>139.301996</c:v>
+                </c:pt>
+                <c:pt idx="883">
+                  <c:v>139.301996</c:v>
+                </c:pt>
+                <c:pt idx="884">
+                  <c:v>139.301996</c:v>
+                </c:pt>
+                <c:pt idx="885">
+                  <c:v>139.363013063122</c:v>
+                </c:pt>
+                <c:pt idx="886">
+                  <c:v>139.39115200000001</c:v>
+                </c:pt>
+                <c:pt idx="887">
+                  <c:v>139.39115200000001</c:v>
+                </c:pt>
+                <c:pt idx="888">
+                  <c:v>139.40738588079401</c:v>
+                </c:pt>
+                <c:pt idx="889">
+                  <c:v>139.47869900000001</c:v>
+                </c:pt>
+                <c:pt idx="890">
+                  <c:v>139.47869900000001</c:v>
+                </c:pt>
+                <c:pt idx="891">
+                  <c:v>139.47869900000001</c:v>
+                </c:pt>
+                <c:pt idx="892">
+                  <c:v>139.531343292358</c:v>
+                </c:pt>
+                <c:pt idx="893">
+                  <c:v>139.555621</c:v>
+                </c:pt>
+                <c:pt idx="894">
+                  <c:v>139.555621</c:v>
+                </c:pt>
+                <c:pt idx="895">
+                  <c:v>139.571159604651</c:v>
+                </c:pt>
+                <c:pt idx="896">
+                  <c:v>139.639141</c:v>
+                </c:pt>
+                <c:pt idx="897">
+                  <c:v>139.639141</c:v>
+                </c:pt>
+                <c:pt idx="898">
+                  <c:v>139.639141</c:v>
+                </c:pt>
+                <c:pt idx="899">
+                  <c:v>139.67876121262401</c:v>
+                </c:pt>
+                <c:pt idx="900">
+                  <c:v>139.696753</c:v>
+                </c:pt>
+                <c:pt idx="901">
+                  <c:v>139.696753</c:v>
+                </c:pt>
+                <c:pt idx="902">
+                  <c:v>139.711765465116</c:v>
+                </c:pt>
+                <c:pt idx="903">
+                  <c:v>139.777445</c:v>
+                </c:pt>
+                <c:pt idx="904">
+                  <c:v>139.777445</c:v>
+                </c:pt>
+                <c:pt idx="905">
+                  <c:v>139.777445</c:v>
+                </c:pt>
+                <c:pt idx="906">
+                  <c:v>139.82964957474999</c:v>
+                </c:pt>
+                <c:pt idx="907">
+                  <c:v>139.85335599999999</c:v>
+                </c:pt>
+                <c:pt idx="908">
+                  <c:v>139.85335599999999</c:v>
+                </c:pt>
+                <c:pt idx="909">
+                  <c:v>139.86821046511599</c:v>
+                </c:pt>
+                <c:pt idx="910">
+                  <c:v>139.93179799999999</c:v>
+                </c:pt>
+                <c:pt idx="911">
+                  <c:v>139.93179799999999</c:v>
+                </c:pt>
+                <c:pt idx="912">
+                  <c:v>139.93179799999999</c:v>
+                </c:pt>
+                <c:pt idx="913">
+                  <c:v>139.980212936877</c:v>
+                </c:pt>
+                <c:pt idx="914">
+                  <c:v>140.00185999999999</c:v>
+                </c:pt>
+                <c:pt idx="915">
+                  <c:v>140.00185999999999</c:v>
+                </c:pt>
+                <c:pt idx="916">
+                  <c:v>140.01199482724201</c:v>
+                </c:pt>
+                <c:pt idx="917">
+                  <c:v>140.05537899999999</c:v>
+                </c:pt>
+                <c:pt idx="918">
+                  <c:v>140.05537899999999</c:v>
+                </c:pt>
+                <c:pt idx="919">
+                  <c:v>140.05537899999999</c:v>
+                </c:pt>
+                <c:pt idx="920">
+                  <c:v>140.104568581395</c:v>
+                </c:pt>
+                <c:pt idx="921">
+                  <c:v>140.12656200000001</c:v>
+                </c:pt>
+                <c:pt idx="922">
+                  <c:v>140.12656200000001</c:v>
+                </c:pt>
+                <c:pt idx="923">
+                  <c:v>140.14572627906901</c:v>
+                </c:pt>
+                <c:pt idx="924">
+                  <c:v>140.22601800000001</c:v>
+                </c:pt>
+                <c:pt idx="925">
+                  <c:v>140.22601800000001</c:v>
+                </c:pt>
+                <c:pt idx="926">
+                  <c:v>140.22601800000001</c:v>
+                </c:pt>
+                <c:pt idx="927">
+                  <c:v>140.27026025496599</c:v>
+                </c:pt>
+                <c:pt idx="928">
+                  <c:v>140.28994700000001</c:v>
+                </c:pt>
+                <c:pt idx="929">
+                  <c:v>140.28994700000001</c:v>
+                </c:pt>
+                <c:pt idx="930">
+                  <c:v>140.30493913289001</c:v>
+                </c:pt>
+                <c:pt idx="931">
+                  <c:v>140.367751</c:v>
+                </c:pt>
+                <c:pt idx="932">
+                  <c:v>140.367751</c:v>
+                </c:pt>
+                <c:pt idx="933">
+                  <c:v>140.367751</c:v>
+                </c:pt>
+                <c:pt idx="934">
+                  <c:v>140.42394630896999</c:v>
+                </c:pt>
+                <c:pt idx="935">
+                  <c:v>140.44868299999999</c:v>
+                </c:pt>
+                <c:pt idx="936">
+                  <c:v>140.44868299999999</c:v>
+                </c:pt>
+                <c:pt idx="937">
+                  <c:v>140.45905645033099</c:v>
+                </c:pt>
+                <c:pt idx="938">
+                  <c:v>140.50178099999999</c:v>
+                </c:pt>
+                <c:pt idx="939">
+                  <c:v>140.50178099999999</c:v>
+                </c:pt>
+                <c:pt idx="940">
+                  <c:v>140.50178099999999</c:v>
+                </c:pt>
+                <c:pt idx="941">
+                  <c:v>140.54217493687699</c:v>
+                </c:pt>
+                <c:pt idx="942">
+                  <c:v>140.559956</c:v>
+                </c:pt>
+                <c:pt idx="943">
+                  <c:v>140.559956</c:v>
+                </c:pt>
+                <c:pt idx="944">
+                  <c:v>140.572162335548</c:v>
+                </c:pt>
+                <c:pt idx="945">
+                  <c:v>140.622229</c:v>
+                </c:pt>
+                <c:pt idx="946">
+                  <c:v>140.622229</c:v>
+                </c:pt>
+                <c:pt idx="947">
+                  <c:v>140.622229</c:v>
+                </c:pt>
+                <c:pt idx="948">
+                  <c:v>140.665546906976</c:v>
+                </c:pt>
+                <c:pt idx="949">
+                  <c:v>140.68431799999999</c:v>
+                </c:pt>
+                <c:pt idx="950">
+                  <c:v>140.68431799999999</c:v>
+                </c:pt>
+                <c:pt idx="951">
+                  <c:v>140.698843564784</c:v>
+                </c:pt>
+                <c:pt idx="952">
+                  <c:v>140.75842299999999</c:v>
+                </c:pt>
+                <c:pt idx="953">
+                  <c:v>140.75842299999999</c:v>
+                </c:pt>
+                <c:pt idx="954">
+                  <c:v>140.75842299999999</c:v>
+                </c:pt>
+                <c:pt idx="955">
+                  <c:v>140.79089416279001</c:v>
+                </c:pt>
+                <c:pt idx="956">
+                  <c:v>140.80496500000001</c:v>
+                </c:pt>
+                <c:pt idx="957">
+                  <c:v>140.80496500000001</c:v>
+                </c:pt>
+                <c:pt idx="958">
+                  <c:v>140.817710714285</c:v>
+                </c:pt>
+                <c:pt idx="959">
+                  <c:v>140.86890600000001</c:v>
+                </c:pt>
+                <c:pt idx="960">
+                  <c:v>140.86890600000001</c:v>
+                </c:pt>
+                <c:pt idx="961">
+                  <c:v>140.86890600000001</c:v>
+                </c:pt>
+                <c:pt idx="962">
+                  <c:v>140.92700250166101</c:v>
+                </c:pt>
+                <c:pt idx="963">
+                  <c:v>140.95178300000001</c:v>
+                </c:pt>
+                <c:pt idx="964">
+                  <c:v>140.95178300000001</c:v>
+                </c:pt>
+                <c:pt idx="965">
+                  <c:v>140.969838415282</c:v>
+                </c:pt>
+                <c:pt idx="966">
+                  <c:v>141.042361</c:v>
+                </c:pt>
+                <c:pt idx="967">
+                  <c:v>141.042361</c:v>
+                </c:pt>
+                <c:pt idx="968">
+                  <c:v>141.042361</c:v>
+                </c:pt>
+                <c:pt idx="969">
+                  <c:v>141.09707659468401</c:v>
+                </c:pt>
+                <c:pt idx="970">
+                  <c:v>141.12041500000001</c:v>
+                </c:pt>
+                <c:pt idx="971">
+                  <c:v>141.12041500000001</c:v>
+                </c:pt>
+                <c:pt idx="972">
+                  <c:v>141.137699481727</c:v>
+                </c:pt>
+                <c:pt idx="973">
+                  <c:v>141.205704</c:v>
+                </c:pt>
+                <c:pt idx="974">
+                  <c:v>141.205704</c:v>
+                </c:pt>
+                <c:pt idx="975">
+                  <c:v>141.205704</c:v>
+                </c:pt>
+                <c:pt idx="976">
+                  <c:v>141.254263231788</c:v>
+                </c:pt>
+                <c:pt idx="977">
+                  <c:v>141.274878</c:v>
+                </c:pt>
+                <c:pt idx="978">
+                  <c:v>141.274878</c:v>
+                </c:pt>
+                <c:pt idx="979">
+                  <c:v>141.29160699667699</c:v>
+                </c:pt>
+                <c:pt idx="980">
+                  <c:v>141.357426</c:v>
+                </c:pt>
+                <c:pt idx="981">
+                  <c:v>141.357426</c:v>
+                </c:pt>
+                <c:pt idx="982">
+                  <c:v>141.357426</c:v>
+                </c:pt>
+                <c:pt idx="983">
+                  <c:v>141.40716641195999</c:v>
+                </c:pt>
+                <c:pt idx="984">
+                  <c:v>141.42804799999999</c:v>
+                </c:pt>
+                <c:pt idx="985">
+                  <c:v>141.42804799999999</c:v>
+                </c:pt>
+                <c:pt idx="986">
+                  <c:v>141.44206390066199</c:v>
+                </c:pt>
+                <c:pt idx="987">
+                  <c:v>141.496319</c:v>
+                </c:pt>
+                <c:pt idx="988">
+                  <c:v>141.496319</c:v>
+                </c:pt>
+                <c:pt idx="989">
+                  <c:v>141.496319</c:v>
+                </c:pt>
+                <c:pt idx="990">
+                  <c:v>141.55469717940099</c:v>
+                </c:pt>
+                <c:pt idx="991">
+                  <c:v>141.579205</c:v>
+                </c:pt>
+                <c:pt idx="992">
+                  <c:v>141.579205</c:v>
+                </c:pt>
+                <c:pt idx="993">
+                  <c:v>141.60414630232501</c:v>
+                </c:pt>
+                <c:pt idx="994">
+                  <c:v>141.70029099999999</c:v>
+                </c:pt>
+                <c:pt idx="995">
+                  <c:v>141.70029099999999</c:v>
+                </c:pt>
+                <c:pt idx="996">
+                  <c:v>141.70029099999999</c:v>
+                </c:pt>
+                <c:pt idx="997">
+                  <c:v>141.80257345847099</c:v>
+                </c:pt>
+                <c:pt idx="998">
+                  <c:v>141.844831</c:v>
+                </c:pt>
+                <c:pt idx="999">
+                  <c:v>141.844831</c:v>
+                </c:pt>
+                <c:pt idx="1000">
+                  <c:v>141.871988589403</c:v>
+                </c:pt>
+                <c:pt idx="1001">
+                  <c:v>141.97501500000001</c:v>
+                </c:pt>
+                <c:pt idx="1002">
+                  <c:v>141.97501500000001</c:v>
+                </c:pt>
+                <c:pt idx="1003">
+                  <c:v>141.97501500000001</c:v>
+                </c:pt>
+                <c:pt idx="1004">
+                  <c:v>142.04668914617901</c:v>
+                </c:pt>
+                <c:pt idx="1005">
+                  <c:v>142.076301</c:v>
+                </c:pt>
+                <c:pt idx="1006">
+                  <c:v>142.076301</c:v>
+                </c:pt>
+                <c:pt idx="1007">
+                  <c:v>142.121814418604</c:v>
+                </c:pt>
+                <c:pt idx="1008">
+                  <c:v>142.29375400000001</c:v>
+                </c:pt>
+                <c:pt idx="1009">
+                  <c:v>142.29375400000001</c:v>
+                </c:pt>
+                <c:pt idx="1010">
+                  <c:v>142.29375400000001</c:v>
+                </c:pt>
+                <c:pt idx="1011">
+                  <c:v>142.51852580730801</c:v>
+                </c:pt>
+                <c:pt idx="1012">
+                  <c:v>142.609905</c:v>
+                </c:pt>
+                <c:pt idx="1013">
+                  <c:v>142.609905</c:v>
+                </c:pt>
+                <c:pt idx="1014">
+                  <c:v>142.69545334883699</c:v>
+                </c:pt>
+                <c:pt idx="1015">
+                  <c:v>143.01863599999999</c:v>
+                </c:pt>
+                <c:pt idx="1016">
+                  <c:v>143.01863599999999</c:v>
+                </c:pt>
+                <c:pt idx="1017">
+                  <c:v>143.01863599999999</c:v>
+                </c:pt>
+                <c:pt idx="1018">
+                  <c:v>143.37947768106301</c:v>
+                </c:pt>
+                <c:pt idx="1019">
+                  <c:v>143.52617499999999</c:v>
+                </c:pt>
+                <c:pt idx="1020">
+                  <c:v>143.52617499999999</c:v>
+                </c:pt>
+                <c:pt idx="1021">
+                  <c:v>143.70638092690999</c:v>
+                </c:pt>
+                <c:pt idx="1022">
+                  <c:v>144.373706</c:v>
+                </c:pt>
+                <c:pt idx="1023">
+                  <c:v>144.373706</c:v>
+                </c:pt>
+                <c:pt idx="1024">
+                  <c:v>144.373706</c:v>
+                </c:pt>
+                <c:pt idx="1025">
+                  <c:v>145.225614311258</c:v>
+                </c:pt>
+                <c:pt idx="1026">
+                  <c:v>145.57033999999999</c:v>
+                </c:pt>
+                <c:pt idx="1027">
+                  <c:v>145.57033999999999</c:v>
+                </c:pt>
+                <c:pt idx="1028">
+                  <c:v>145.88019121594601</c:v>
+                </c:pt>
+                <c:pt idx="1029">
+                  <c:v>147.02760900000001</c:v>
+                </c:pt>
+                <c:pt idx="1030">
+                  <c:v>147.02760900000001</c:v>
+                </c:pt>
+                <c:pt idx="1031">
+                  <c:v>147.02760900000001</c:v>
+                </c:pt>
+                <c:pt idx="1032">
+                  <c:v>148.21915328571399</c:v>
+                </c:pt>
+                <c:pt idx="1033">
+                  <c:v>148.69577100000001</c:v>
+                </c:pt>
+                <c:pt idx="1034">
+                  <c:v>148.69577100000001</c:v>
+                </c:pt>
+                <c:pt idx="1035">
+                  <c:v>149.083631165562</c:v>
+                </c:pt>
+                <c:pt idx="1036">
+                  <c:v>150.497829</c:v>
+                </c:pt>
+                <c:pt idx="1037">
+                  <c:v>150.497829</c:v>
+                </c:pt>
+                <c:pt idx="1038">
+                  <c:v>150.497829</c:v>
+                </c:pt>
+                <c:pt idx="1039">
+                  <c:v>151.79829848344301</c:v>
+                </c:pt>
+                <c:pt idx="1040">
+                  <c:v>152.316078</c:v>
+                </c:pt>
+                <c:pt idx="1041">
+                  <c:v>152.316078</c:v>
+                </c:pt>
+                <c:pt idx="1042">
+                  <c:v>152.70516756810599</c:v>
+                </c:pt>
+                <c:pt idx="1043">
+                  <c:v>154.117862</c:v>
+                </c:pt>
+                <c:pt idx="1044">
+                  <c:v>154.117862</c:v>
+                </c:pt>
+                <c:pt idx="1045">
+                  <c:v>154.117862</c:v>
+                </c:pt>
+                <c:pt idx="1046">
+                  <c:v>155.40067021262399</c:v>
+                </c:pt>
+                <c:pt idx="1047">
+                  <c:v>155.90547900000001</c:v>
+                </c:pt>
+                <c:pt idx="1048">
+                  <c:v>155.90547900000001</c:v>
+                </c:pt>
+                <c:pt idx="1049">
+                  <c:v>156.28575832450301</c:v>
+                </c:pt>
+                <c:pt idx="1050">
+                  <c:v>157.645545</c:v>
+                </c:pt>
+                <c:pt idx="1051">
+                  <c:v>157.645545</c:v>
+                </c:pt>
+                <c:pt idx="1052">
+                  <c:v>157.645545</c:v>
+                </c:pt>
+                <c:pt idx="1053">
+                  <c:v>158.81671637541501</c:v>
+                </c:pt>
+                <c:pt idx="1054">
+                  <c:v>159.27759399999999</c:v>
+                </c:pt>
+                <c:pt idx="1055">
+                  <c:v>159.27759399999999</c:v>
+                </c:pt>
+                <c:pt idx="1056">
+                  <c:v>159.62802702990001</c:v>
+                </c:pt>
+                <c:pt idx="1057">
+                  <c:v>160.87578099999999</c:v>
+                </c:pt>
+                <c:pt idx="1058">
+                  <c:v>160.87578099999999</c:v>
+                </c:pt>
+                <c:pt idx="1059">
+                  <c:v>160.87578099999999</c:v>
+                </c:pt>
+                <c:pt idx="1060">
+                  <c:v>161.92825911627901</c:v>
+                </c:pt>
+                <c:pt idx="1061">
+                  <c:v>162.33566999999999</c:v>
+                </c:pt>
+                <c:pt idx="1062">
+                  <c:v>162.33566999999999</c:v>
+                </c:pt>
+                <c:pt idx="1063">
+                  <c:v>162.638672053156</c:v>
+                </c:pt>
+                <c:pt idx="1064">
+                  <c:v>163.71754300000001</c:v>
+                </c:pt>
+                <c:pt idx="1065">
+                  <c:v>163.71754300000001</c:v>
+                </c:pt>
+                <c:pt idx="1066">
+                  <c:v>163.71754300000001</c:v>
+                </c:pt>
+                <c:pt idx="1067">
+                  <c:v>164.66210506976699</c:v>
+                </c:pt>
+                <c:pt idx="1068">
+                  <c:v>165.02774199999999</c:v>
+                </c:pt>
+                <c:pt idx="1069">
+                  <c:v>165.02774199999999</c:v>
+                </c:pt>
+                <c:pt idx="1070">
+                  <c:v>165.294484358803</c:v>
+                </c:pt>
+                <c:pt idx="1071">
+                  <c:v>166.22609199999999</c:v>
+                </c:pt>
+                <c:pt idx="1072">
+                  <c:v>166.22609199999999</c:v>
+                </c:pt>
+                <c:pt idx="1073">
+                  <c:v>166.22609199999999</c:v>
+                </c:pt>
+                <c:pt idx="1074">
+                  <c:v>167.04354724503301</c:v>
+                </c:pt>
+                <c:pt idx="1075">
+                  <c:v>167.35853</c:v>
+                </c:pt>
+                <c:pt idx="1076">
+                  <c:v>167.35853</c:v>
+                </c:pt>
+                <c:pt idx="1077">
+                  <c:v>167.587737445182</c:v>
+                </c:pt>
+                <c:pt idx="1078">
+                  <c:v>168.38825299999999</c:v>
+                </c:pt>
+                <c:pt idx="1079">
+                  <c:v>168.38825299999999</c:v>
+                </c:pt>
+                <c:pt idx="1080">
+                  <c:v>168.38825299999999</c:v>
+                </c:pt>
+                <c:pt idx="1081">
+                  <c:v>169.08295671428499</c:v>
+                </c:pt>
+                <c:pt idx="1082">
+                  <c:v>169.347454</c:v>
+                </c:pt>
+                <c:pt idx="1083">
+                  <c:v>169.347454</c:v>
+                </c:pt>
+                <c:pt idx="1084">
+                  <c:v>169.547545242524</c:v>
+                </c:pt>
+                <c:pt idx="1085">
+                  <c:v>170.23315199999999</c:v>
+                </c:pt>
+                <c:pt idx="1086">
+                  <c:v>170.23315199999999</c:v>
+                </c:pt>
+                <c:pt idx="1087">
+                  <c:v>170.23315199999999</c:v>
+                </c:pt>
+                <c:pt idx="1088">
+                  <c:v>170.79637431456899</c:v>
+                </c:pt>
+                <c:pt idx="1089">
+                  <c:v>171.00983299999999</c:v>
+                </c:pt>
+                <c:pt idx="1090">
+                  <c:v>171.00983299999999</c:v>
+                </c:pt>
+                <c:pt idx="1091">
+                  <c:v>171.17719952491601</c:v>
+                </c:pt>
+                <c:pt idx="1092">
+                  <c:v>171.750676</c:v>
+                </c:pt>
+                <c:pt idx="1093">
+                  <c:v>171.750676</c:v>
+                </c:pt>
+                <c:pt idx="1094">
+                  <c:v>171.750676</c:v>
+                </c:pt>
+                <c:pt idx="1095">
+                  <c:v>172.22949585382</c:v>
+                </c:pt>
+                <c:pt idx="1096">
+                  <c:v>172.40878000000001</c:v>
+                </c:pt>
+                <c:pt idx="1097">
+                  <c:v>172.40878000000001</c:v>
+                </c:pt>
+                <c:pt idx="1098">
+                  <c:v>172.548126413907</c:v>
+                </c:pt>
+                <c:pt idx="1099">
+                  <c:v>173.01867300000001</c:v>
+                </c:pt>
+                <c:pt idx="1100">
+                  <c:v>173.01867300000001</c:v>
+                </c:pt>
+                <c:pt idx="1101">
+                  <c:v>173.01867300000001</c:v>
+                </c:pt>
+                <c:pt idx="1102">
+                  <c:v>173.409288239202</c:v>
+                </c:pt>
+                <c:pt idx="1103">
+                  <c:v>173.55554599999999</c:v>
+                </c:pt>
+                <c:pt idx="1104">
+                  <c:v>173.55554599999999</c:v>
+                </c:pt>
+                <c:pt idx="1105">
+                  <c:v>173.67127344186</c:v>
+                </c:pt>
+                <c:pt idx="1106">
+                  <c:v>174.06038599999999</c:v>
+                </c:pt>
+                <c:pt idx="1107">
+                  <c:v>174.06038599999999</c:v>
+                </c:pt>
+                <c:pt idx="1108">
+                  <c:v>174.06038599999999</c:v>
+                </c:pt>
+                <c:pt idx="1109">
+                  <c:v>174.36215510298999</c:v>
+                </c:pt>
+                <c:pt idx="1110">
+                  <c:v>174.47326100000001</c:v>
+                </c:pt>
+                <c:pt idx="1111">
+                  <c:v>174.47326100000001</c:v>
+                </c:pt>
+                <c:pt idx="1112">
+                  <c:v>174.566002043189</c:v>
+                </c:pt>
+                <c:pt idx="1113">
+                  <c:v>174.877827</c:v>
+                </c:pt>
+                <c:pt idx="1114">
+                  <c:v>174.877827</c:v>
+                </c:pt>
+                <c:pt idx="1115">
+                  <c:v>174.877827</c:v>
+                </c:pt>
+                <c:pt idx="1116">
+                  <c:v>175.15759025581301</c:v>
+                </c:pt>
+                <c:pt idx="1117">
+                  <c:v>175.260594</c:v>
+                </c:pt>
+                <c:pt idx="1118">
+                  <c:v>175.260594</c:v>
+                </c:pt>
+                <c:pt idx="1119">
+                  <c:v>175.33398399999999</c:v>
+                </c:pt>
+                <c:pt idx="1120">
+                  <c:v>175.57617099999999</c:v>
+                </c:pt>
+                <c:pt idx="1121">
+                  <c:v>175.57617099999999</c:v>
+                </c:pt>
+                <c:pt idx="1122">
+                  <c:v>175.57617099999999</c:v>
+                </c:pt>
+                <c:pt idx="1123">
+                  <c:v>175.77705412624499</c:v>
+                </c:pt>
+                <c:pt idx="1124">
+                  <c:v>175.849772</c:v>
+                </c:pt>
+                <c:pt idx="1125">
+                  <c:v>175.849772</c:v>
+                </c:pt>
+                <c:pt idx="1126">
+                  <c:v>175.911971767441</c:v>
+                </c:pt>
+                <c:pt idx="1127">
+                  <c:v>176.117231</c:v>
+                </c:pt>
+                <c:pt idx="1128">
+                  <c:v>176.117231</c:v>
+                </c:pt>
+                <c:pt idx="1129">
+                  <c:v>176.117231</c:v>
+                </c:pt>
+                <c:pt idx="1130">
+                  <c:v>176.287029485049</c:v>
+                </c:pt>
+                <c:pt idx="1131">
+                  <c:v>176.34849500000001</c:v>
+                </c:pt>
+                <c:pt idx="1132">
+                  <c:v>176.34849500000001</c:v>
+                </c:pt>
+                <c:pt idx="1133">
+                  <c:v>176.40130814950101</c:v>
+                </c:pt>
+                <c:pt idx="1134">
+                  <c:v>176.57239300000001</c:v>
+                </c:pt>
+                <c:pt idx="1135">
+                  <c:v>176.57239300000001</c:v>
+                </c:pt>
+                <c:pt idx="1136">
+                  <c:v>176.57239300000001</c:v>
+                </c:pt>
+                <c:pt idx="1137">
+                  <c:v>176.69690486092699</c:v>
+                </c:pt>
+                <c:pt idx="1138">
+                  <c:v>176.74177399999999</c:v>
+                </c:pt>
+                <c:pt idx="1139">
+                  <c:v>176.74177399999999</c:v>
+                </c:pt>
+                <c:pt idx="1140">
+                  <c:v>176.77896361129501</c:v>
+                </c:pt>
+                <c:pt idx="1141">
+                  <c:v>176.89943700000001</c:v>
+                </c:pt>
+                <c:pt idx="1142">
+                  <c:v>176.89943700000001</c:v>
+                </c:pt>
+                <c:pt idx="1143">
+                  <c:v>176.89943700000001</c:v>
+                </c:pt>
+                <c:pt idx="1144">
+                  <c:v>177.00431245514901</c:v>
+                </c:pt>
+                <c:pt idx="1145">
+                  <c:v>177.04163299999999</c:v>
+                </c:pt>
+                <c:pt idx="1146">
+                  <c:v>177.04163299999999</c:v>
+                </c:pt>
+                <c:pt idx="1147">
+                  <c:v>177.06635784768201</c:v>
+                </c:pt>
+                <c:pt idx="1148">
+                  <c:v>177.14534</c:v>
+                </c:pt>
+                <c:pt idx="1149">
+                  <c:v>177.14534</c:v>
+                </c:pt>
+                <c:pt idx="1150">
+                  <c:v>177.14534</c:v>
+                </c:pt>
+                <c:pt idx="1151">
+                  <c:v>177.226270431893</c:v>
+                </c:pt>
+                <c:pt idx="1152">
+                  <c:v>177.25506999999999</c:v>
+                </c:pt>
+                <c:pt idx="1153">
+                  <c:v>177.25506999999999</c:v>
+                </c:pt>
+                <c:pt idx="1154">
+                  <c:v>177.273895727574</c:v>
+                </c:pt>
+                <c:pt idx="1155">
+                  <c:v>177.33377200000001</c:v>
+                </c:pt>
+                <c:pt idx="1156">
+                  <c:v>177.33377200000001</c:v>
+                </c:pt>
+                <c:pt idx="1157">
+                  <c:v>177.33377200000001</c:v>
+                </c:pt>
+                <c:pt idx="1158">
+                  <c:v>177.39147639867099</c:v>
+                </c:pt>
+                <c:pt idx="1159">
+                  <c:v>177.41166000000001</c:v>
+                </c:pt>
+                <c:pt idx="1160">
+                  <c:v>177.41166000000001</c:v>
+                </c:pt>
+                <c:pt idx="1161">
+                  <c:v>177.42861013953399</c:v>
+                </c:pt>
+                <c:pt idx="1162">
+                  <c:v>177.48252099999999</c:v>
+                </c:pt>
+                <c:pt idx="1163">
+                  <c:v>177.48252099999999</c:v>
+                </c:pt>
+                <c:pt idx="1164">
+                  <c:v>177.48252099999999</c:v>
+                </c:pt>
+                <c:pt idx="1165">
+                  <c:v>177.51672668106301</c:v>
+                </c:pt>
+                <c:pt idx="1166">
+                  <c:v>177.52869100000001</c:v>
+                </c:pt>
+                <c:pt idx="1167">
+                  <c:v>177.52869100000001</c:v>
+                </c:pt>
+                <c:pt idx="1168">
+                  <c:v>177.537939687707</c:v>
+                </c:pt>
+                <c:pt idx="1169">
+                  <c:v>177.56682599999999</c:v>
+                </c:pt>
+                <c:pt idx="1170">
+                  <c:v>177.56682599999999</c:v>
+                </c:pt>
+                <c:pt idx="1171">
+                  <c:v>177.56682599999999</c:v>
+                </c:pt>
+                <c:pt idx="1172">
+                  <c:v>177.56348534883699</c:v>
+                </c:pt>
+                <c:pt idx="1173">
+                  <c:v>177.56233700000001</c:v>
+                </c:pt>
+                <c:pt idx="1174">
+                  <c:v>177.56233700000001</c:v>
+                </c:pt>
+                <c:pt idx="1175">
+                  <c:v>177.576388408637</c:v>
+                </c:pt>
+                <c:pt idx="1176">
+                  <c:v>177.62027499999999</c:v>
+                </c:pt>
+                <c:pt idx="1177">
+                  <c:v>177.62027499999999</c:v>
+                </c:pt>
+                <c:pt idx="1178">
+                  <c:v>177.62027499999999</c:v>
+                </c:pt>
+                <c:pt idx="1179">
+                  <c:v>177.60881900000001</c:v>
+                </c:pt>
+                <c:pt idx="1180">
+                  <c:v>177.60488100000001</c:v>
+                </c:pt>
+                <c:pt idx="1181">
+                  <c:v>177.60488100000001</c:v>
+                </c:pt>
+                <c:pt idx="1182">
+                  <c:v>177.60484928571401</c:v>
+                </c:pt>
+                <c:pt idx="1183">
+                  <c:v>177.60475199999999</c:v>
+                </c:pt>
+                <c:pt idx="1184">
+                  <c:v>177.60475199999999</c:v>
+                </c:pt>
+                <c:pt idx="1185">
+                  <c:v>177.60475199999999</c:v>
+                </c:pt>
+                <c:pt idx="1186">
+                  <c:v>177.604830973509</c:v>
+                </c:pt>
+                <c:pt idx="1187">
+                  <c:v>177.60485800000001</c:v>
+                </c:pt>
+                <c:pt idx="1188">
+                  <c:v>177.60485800000001</c:v>
+                </c:pt>
+                <c:pt idx="1189">
+                  <c:v>177.59933332225901</c:v>
+                </c:pt>
+                <c:pt idx="1190">
+                  <c:v>177.58238600000001</c:v>
+                </c:pt>
+                <c:pt idx="1191">
+                  <c:v>177.58238600000001</c:v>
+                </c:pt>
+                <c:pt idx="1192">
+                  <c:v>177.58238600000001</c:v>
+                </c:pt>
+                <c:pt idx="1193">
+                  <c:v>177.549507594684</c:v>
+                </c:pt>
+                <c:pt idx="1194">
+                  <c:v>177.53840199999999</c:v>
+                </c:pt>
+                <c:pt idx="1195">
+                  <c:v>177.53840199999999</c:v>
+                </c:pt>
+                <c:pt idx="1196">
+                  <c:v>177.53804016225101</c:v>
+                </c:pt>
+                <c:pt idx="1197">
+                  <c:v>177.536945</c:v>
+                </c:pt>
+                <c:pt idx="1198">
+                  <c:v>177.536945</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FF27-D940-AD53-B573F44D7B39}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1381531376"/>
+        <c:axId val="1381533088"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1381531376"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1381533088"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1381533088"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="180"/>
+          <c:min val="90"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1381531376"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -15857,6 +19742,46 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -17444,6 +21369,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -17485,15 +21926,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>297018</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>198208</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>749300</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>198721</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>10717</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -17528,8 +21969,8 @@
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>71120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -17549,6 +21990,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>679194</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>55909</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>498604</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>63250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1715B88-E0E0-D319-2819-7BBC434A2954}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>